<commit_message>
chore: ISSUE-026 完了・tracker 更新
- ISSUE-026 を解決済に更新（issues.json）
- issues_export.xlsx 再生成

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -2364,17 +2364,17 @@
       <c r="O26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="40" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>ISSUE-026</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>SRS 用語統一（Keyコル / dominant peak / ピーク・サミット候補）</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>URD/SRS レビュー指摘 L-1 + L-2 + L-3。
 L-1: 'Keyコル' / 'Key Col' / 'key_col_boundary' / 'prominence boundary polygon' が FR-006 / FR-009 / FR-016 / FR-018 で混在。
@@ -2382,7 +2382,7 @@
 L-3: 'dominant peak' と 'ドミナントピーク' が GLOSSARY 見出しと本文で混在。</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>改善</t>
         </is>
@@ -2392,29 +2392,29 @@
           <t>低</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>その他</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr"/>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="G27" s="5" t="inlineStr"/>
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="I27" s="5" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>未対応</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr"/>
-      <c r="L27" s="4" t="inlineStr">
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr"/>
+      <c r="L27" s="5" t="inlineStr">
         <is>
           <t>表記ルールを SRS 冒頭または GLOSSARY に明示し、全文を統一:
 (1) 本文表記: 'Keyコル'、プロパティ名 / feature_type 値: 'key_col_boundary' に統一
@@ -2422,9 +2422,17 @@
 (3) 'dominant peak' は本文・GLOSSARY 見出しとも英語表記に統一</t>
         </is>
       </c>
-      <c r="M27" s="4" t="inlineStr"/>
-      <c r="N27" s="4" t="inlineStr"/>
-      <c r="O27" s="4" t="inlineStr"/>
+      <c r="M27" s="5" t="inlineStr"/>
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="O27" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="40" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -2963,7 +2971,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -2973,7 +2981,7 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -2984,7 +2992,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>8.8%</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3011,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9">
@@ -3033,7 +3041,7 @@
         </is>
       </c>
       <c r="B11" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -3081,7 +3089,7 @@
         </is>
       </c>
       <c r="B17" s="11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
@@ -3109,7 +3117,7 @@
         </is>
       </c>
       <c r="B21" s="11" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22">
@@ -3187,7 +3195,7 @@
         </is>
       </c>
       <c r="B30" s="11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="32">
@@ -3215,7 +3223,7 @@
         </is>
       </c>
       <c r="B34" s="11" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35">
@@ -3598,10 +3606,10 @@
         <v>34</v>
       </c>
       <c r="C22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: ISSUE-010 解決済み更新・issues_export.xlsx 再生成
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -743,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:O37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1442,22 +1442,22 @@
       <c r="O10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>ISSUE-010</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>セットアップ手順の整備（README・requirements.txt・.gitignore・CLAUDE.md）</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>.venv仮想環境の導入に伴い、新規参加者がすぐに使い始められるよう以下を整備する。① scripts/requirements.txt 新規作成、② .gitignore に .venv/ 追記、③ README.md にセットアップ手順・プロジェクト概要を記載、④ CLAUDE.md に .venv/bin/python3 使用の旨を追記</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>改善</t>
         </is>
@@ -1467,40 +1467,48 @@
           <t>中</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>設定</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr"/>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr"/>
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>OPS</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>未対応</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="L11" s="5" t="inlineStr">
         <is>
           <t>requirements.txt・.gitignore・CLAUDE.md は小規模な編集。README.md は現状に合わせて内容を整理してから更新する</t>
         </is>
       </c>
-      <c r="M11" s="4" t="inlineStr"/>
-      <c r="N11" s="4" t="inlineStr"/>
-      <c r="O11" s="4" t="inlineStr"/>
+      <c r="M11" s="5" t="inlineStr"/>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="40" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -2914,18 +2922,108 @@
       <c r="N35" s="4" t="inlineStr"/>
       <c r="O35" s="4" t="inlineStr"/>
     </row>
+    <row r="36" ht="40" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>SRS: 竹島除外方針の記述追加・ADR-009 リンク</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>URD UR-001・ADR-009 に竹島除外方針を追加済み。SRS の前提・制約・スコープ外・FR-003 関連箇所に竹島の記述を追加し、ADR-009 へのリンクを貼る。北方領土の記述（ADR-005 参照）に準じた形で記載すること。</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="40" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>ISSUE-036</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>COD: mesh_list_japan.txt からメッシュ 5531（竹島）を削除</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>ADR-009 の決定に基づく実装。params/mesh_list_japan.txt から 5531 を1行削除する。竹島（HL/GB-430）は韓国 SOTA サミットであり SOTA 日本支部の管轄外。除外根拠: docs/decisions/ADR-009-takeshima-exclusion.md</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr"/>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr"/>
+      <c r="L37" s="4" t="inlineStr"/>
+      <c r="M37" s="4" t="inlineStr"/>
+      <c r="N37" s="4" t="inlineStr"/>
+      <c r="O37" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation sqref="J2:J35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2961,7 +3059,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3">
@@ -2971,7 +3069,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
@@ -2981,7 +3079,7 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -2992,7 +3090,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>11.1%</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3109,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9">
@@ -3041,7 +3139,7 @@
         </is>
       </c>
       <c r="B11" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -3079,7 +3177,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17">
@@ -3117,7 +3215,7 @@
         </is>
       </c>
       <c r="B21" s="11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22">
@@ -3185,7 +3283,7 @@
         </is>
       </c>
       <c r="B29" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -3223,7 +3321,7 @@
         </is>
       </c>
       <c r="B34" s="11" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="35">
@@ -3243,7 +3341,7 @@
         </is>
       </c>
       <c r="B36" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="37">
@@ -3273,7 +3371,7 @@
         </is>
       </c>
       <c r="B39" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -3603,13 +3701,13 @@
         <v>46159</v>
       </c>
       <c r="B22" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: ADR-010 Phase 1〜4 を ISSUE-037〜040 として登録
- ISSUE-037 [高/改善] Phase 1: ビルド基盤 + elevation.c の C++/OpenCV 化
- ISSUE-038 [高/改善] Phase 2: 残り src/ の C++ 翻訳
- ISSUE-039 [中/改善] Phase 3: FR-015 標高地形図出力の OpenCV 化
- ISSUE-040 [高/機能追加] Phase 4: FR-016 アクティベーションゾーン計算 新規実装

issues_export.xlsx を再生成

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -743,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O37"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3064,18 +3064,314 @@
       <c r="N37" s="7" t="inlineStr"/>
       <c r="O37" s="7" t="inlineStr"/>
     </row>
+    <row r="38" ht="40" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>ISSUE-037</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>ADR-010 Phase 1: ビルド基盤 + elevation.c の C++/OpenCV 化（標高値同値性検証含む）</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>ADR-010（C++/OpenCV 全面移行）の Phase 1 として、ビルド基盤の C++ 化と elevation.c の C++ + cv::imread 化を行う。
+【作業範囲】
+- Makefile を g++ + pkg-config（opencv4）対応に変更
+- src/elevation.c を C++ に翻訳し、PNG デコードを libpng → cv::imread に置換
+- RGB→標高変換ロジックは cv::Mat ベースで再実装
+- Dockerfile / コンテナ環境に libopencv-dev インストール手順を追加
+- docs/environment.md・CLAUDE.md の依存ライブラリ記述を更新
+【検証ポイント】
+- 既知タイル（例: tiles/15/29097/12863.png）を libpng と cv::imread でデコードした結果が完全一致すること（全 256×256 ピクセルの RGB 値）
+- ランダムサンプル 100 枚で全ピクセル一致を確認
+- test_mesh_analyze 4929 の結果が現行と同一であること
+- 9 メッシュ実行でメモリ消費が ±10% 以内
+【参照】
+- ADR-010 docs/decisions/ADR-010-cpp-opencv-migration.md
+- 検討資料 docs/decisions/research/cpp-opencv-migration-research.md（§3 同値性検証手順、§6 ビルド基盤変更）</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>解析エンジン</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr"/>
+      <c r="L38" s="4" t="inlineStr"/>
+      <c r="M38" s="4" t="inlineStr"/>
+      <c r="N38" s="4" t="inlineStr"/>
+      <c r="O38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39" ht="40" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-038</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>ADR-010 Phase 2: 残り src/ の C++ 翻訳（mesh / unionfind / analyze / mesh_analyze / main / tests）</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>ADR-010 Phase 2: Phase 1 で C++ 化したビルド基盤の上に、残りの src/ を C++ に翻訳する。
+【作業範囲】
+- src/mesh.c → mesh.cpp
+- src/unionfind.c → unionfind.cpp
+- src/analyze.c → analyze.cpp
+- src/mesh_analyze.c → mesh_analyze.cpp
+- src/main.c → main.cpp
+- tests/*.c → *.cpp
+- malloc/realloc → std::vector への機械的置換主体
+- 構造体は class 化せず原則そのまま維持
+【方針】
+- 過剰な C++ 機能（テンプレートメタプログラミング・複雑な継承等）は採用しない
+- 採用するのは RAII / std::vector / std::string / 参照 / const 厳格化 / cv::Mat / auto（限定的）
+- 既存の C コード構造を保持したまま安全性を底上げする翻訳に留める
+【検証ポイント】
+- 既存テスト（test_mesh_analyze / test_analyze）が全通過
+- 既知メッシュ（4929 / 5339）の per-mesh CSV がバイト単位で現行実装と一致
+- 標高地形図 PNG が現行実装と一致（Phase 3 まで cv::imread/imwrite で再生成しない場合）
+【参照】
+- ADR-010 docs/decisions/ADR-010-cpp-opencv-migration.md
+- 検討資料 §4 C++ 利用方針と踏まない罠</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>解析エンジン</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="K39" s="7" t="inlineStr"/>
+      <c r="L39" s="7" t="inlineStr"/>
+      <c r="M39" s="7" t="inlineStr"/>
+      <c r="N39" s="7" t="inlineStr"/>
+      <c r="O39" s="7" t="inlineStr"/>
+    </row>
+    <row r="40" ht="40" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>ISSUE-039</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>ADR-010 Phase 3: FR-015 標高地形図出力の OpenCV 化</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>ADR-010 Phase 3: FR-015（標高地形図 PNG 出力）の実装を OpenCV ベースに書き直す。
+【作業範囲】
+- 標高値から RGB 色への変換を cv::applyColorMap or cv::LUT で実装
+- 長辺 6000px への縮小を cv::resize に置換
+- PNG 出力を cv::imwrite に置換
+- 配色は現行のカラーマップを LUT 形式で再現（または同等の可読性を持つ標準カラーマップを採用）
+【検証ポイント】
+- 標高地形図 PNG が新カラーマップ実装で正常に生成される
+- 視覚的な可読性が現行と同等以上であることを目視確認
+- 長辺 6000px の縮小が正しく動作
+【参照】
+- ADR-010 docs/decisions/ADR-010-cpp-opencv-migration.md
+- SRS 6.7 標高地形図（Terrain-RGB PNG）</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>解析エンジン</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr"/>
+      <c r="L40" s="4" t="inlineStr"/>
+      <c r="M40" s="4" t="inlineStr"/>
+      <c r="N40" s="4" t="inlineStr"/>
+      <c r="O40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41" ht="40" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-040</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>ADR-010 Phase 4: FR-016 アクティベーションゾーン計算（C++/OpenCV 新規実装）</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>ADR-010 Phase 4: FR-016（アクティベーションゾーン計算）を C++ + OpenCV で新規実装する。
+【作業範囲】
+- ピーク位置を起点とした cv::floodFill で標高差 25m 以内の連続領域を抽出
+  - 4 連結 + FLOODFILL_FIXED_RANGE + FLOODFILL_MASK_ONLY を使用
+- cv::findContours で外周輪郭を取得（CHAIN_APPROX_SIMPLE モードで lossless 出力）
+- 形状を変える簡略化（Douglas-Peucker / approxPolyDP / 等間隔抽出）は使用しない
+- ピクセル座標 → 緯度経度変換は既存の pixel_to_latlon() を再利用
+- 解析範囲外（メッシュ地理範囲外）に Flood Fill が到達したら area_truncated=true を付与
+- 同じ Flood Fill を col_elev 閾値で再実行してコル等高線ポリゴンを生成（is_tile_top=1 はスキップ）
+- per-mesh GeoJSON ファイル &lt;meshcode&gt;_activation.geojson を出力
+【新規モジュール】
+- src/activation.cpp / activation.h（Flood Fill 呼び出し + 輪郭抽出 + GeoJSON シリアライズ）
+- mesh_analyze.cpp の CSV 出力ループ内から呼び出し
+【検証ポイント】
+- per-mesh &lt;meshcode&gt;_activation.geojson が生成される
+- 地理院地図上に重ねて目視確認（SOTA ルール 25m 連続が反映されている）
+- area_truncated フラグが解析範囲端のケースで正しく付与される
+- コル等高線ポリゴンが feature_type="key_col_boundary" で出力される
+- is_tile_top=1 のピークではコル等高線が出力されない
+【参照】
+- ADR-010 docs/decisions/ADR-010-cpp-opencv-migration.md
+- SRS FR-016 docs/02_SRS.md
+- SRS 6.8 中間ファイル: メッシュ別アクティベーションゾーン GeoJSON</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>機能追加</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>解析エンジン</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="K41" s="7" t="inlineStr"/>
+      <c r="L41" s="7" t="inlineStr"/>
+      <c r="M41" s="7" t="inlineStr"/>
+      <c r="N41" s="7" t="inlineStr"/>
+      <c r="O41" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation sqref="J2:J37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3111,7 +3407,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -3121,7 +3417,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
@@ -3142,7 +3438,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>22.5%</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3457,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9">
@@ -3219,7 +3515,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16">
@@ -3229,7 +3525,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17">
@@ -3257,7 +3553,7 @@
         </is>
       </c>
       <c r="B20" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
@@ -3267,7 +3563,7 @@
         </is>
       </c>
       <c r="B21" s="11" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22">
@@ -3305,7 +3601,7 @@
         </is>
       </c>
       <c r="B26" s="11" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27">
@@ -3383,7 +3679,7 @@
         </is>
       </c>
       <c r="B35" s="11" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36">
@@ -3723,7 +4019,7 @@
         <v>46159</v>
       </c>
       <c r="B22" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C22" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
chore: ISSUE-019/020/029/040 に Opus 相談推奨フラグを追加
設計判断の複雑性が高く、Opus との独立検証が望ましい4件に
notes フィールドで【Opus相談推奨】を明示し、相談ポイントを列挙:

- ISSUE-019 仮サミットコード採番順序＋採番安定性ポリシー
- ISSUE-020 手動調査待ちピークの GeoJSON フィーチャ扱い（3案比較）
- ISSUE-029 UR-008/009 の要件性検討（URD/SRS構造判断）
- ISSUE-040 ADR-010 Phase 4: FR-016 OpenCV 実装の細部設計

issues_export.xlsx を再生成

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -2068,7 +2068,16 @@
 (3) NFR-003 とのトレース確認</t>
         </is>
       </c>
-      <c r="M20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>【Opus相談推奨】複数の独立した設計判断と副次的影響の整理が必要。
+相談ポイント:
+(1) 採番順序の選択肢比較（peak_lat降順→peak_lon昇順タイブレーク vs (peak_lat, peak_lon)昇順タプル vs その他）。実データでの順序安定性・可読性・申請書での扱いやすさを総合評価
+(2) 採番安定性ポリシーの設計（フル解析時のみ採番再生成 / 部分解析時は既存コード保持 / その他）。将来の部分再実行ユースケース・ビューア localStorage との整合性・ユーザー混乱の回避を考慮
+(3) (1)(2)の組み合わせがNFR-003（決定論的出力）と整合することの検証方法
+(4) 既存仮コード割当がない初回実行と、再実行の境界ケースの扱い</t>
+        </is>
+      </c>
       <c r="N20" s="4" t="inlineStr"/>
       <c r="O20" s="4" t="inlineStr"/>
     </row>
@@ -2132,7 +2141,17 @@
 併せて area_truncated=true が残るケースの FR-014 挙動も明示。</t>
         </is>
       </c>
-      <c r="M21" s="7" t="inlineStr"/>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>【Opus相談推奨】3案あり、FR-013/FR-014/FR-016/merge.py/ビューアの広範囲に影響する複合判断。
+相談ポイント:
+(1) 案A・案B・案Cそれぞれの長所短所を、影響範囲（FR-013出力構造、merge.py突合ロジック、ビューア表示）を含めて比較
+(2) 'unresolved' を第4のmatch_statusに追加した場合のADR-007との整合性
+(3) コル等高線フォールバック表現（仮Polygon/空Polygon）の point-in-polygon 突合動作への影響
+(4) 手動調査待ちピーク = 何件想定か。1〜2件なら手動対応で十分か、自動化が必要か
+(5) area_truncated=true が4×4でも解消しなかった場合の挙動（is_tile_top=1とは独立に発生しうる）</t>
+        </is>
+      </c>
       <c r="N21" s="7" t="inlineStr"/>
       <c r="O21" s="7" t="inlineStr"/>
     </row>
@@ -2669,7 +2688,17 @@
 案C: URD に残し、トレース確認のための専用節を新設</t>
         </is>
       </c>
-      <c r="M30" s="4" t="inlineStr"/>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>【Opus相談推奨】URD/SRS構造に関わる設計哲学的判断。後から変更すると影響範囲が大きい。
+相談ポイント:
+(1) 案A・案B・案Cそれぞれの長所短所。要件管理の一般的なプラクティスに照らした評価
+(2) UR-008（環境構築から成果物生成までの実行可能性）とUR-009（仕様・実装の整合性）は本質的に '品質目標' であり、ユーザー要求とは性質が異なる。これをURDに残すべきか、NFRに移すべきか
+(3) ISO/IEC 25010 等の品質特性モデルとのマッピング
+(4) 既存のNFR-003 / NFR-007との対応関係を明示するか、独立した品質目標として扱うか
+(5) ISSUE-031（UR↔FR/NFRトレース調査）・ISSUE-032（RTM作成）の進め方への影響</t>
+        </is>
+      </c>
       <c r="N30" s="4" t="inlineStr"/>
       <c r="O30" s="4" t="inlineStr"/>
     </row>
@@ -3356,7 +3385,19 @@
       </c>
       <c r="K41" s="7" t="inlineStr"/>
       <c r="L41" s="7" t="inlineStr"/>
-      <c r="M41" s="7" t="inlineStr"/>
+      <c r="M41" s="7" t="inlineStr">
+        <is>
+          <t>【Opus相談推奨】OpenCV実装の細部設計・メモリ最適化・エッジケース整理に深い設計判断が必要。
+相談ポイント:
+(1) cv::floodFill のメモリ戦略: 全画像サイズのmask（H+2 × W+2、4GB）を全ピーク間で再利用 vs ピークごとにbbox限定でmaskを確保。9メッシュ56.9GB環境での最適解
+(2) cv::Mat の参照カウント・shared_ptr 的挙動の正確な理解と、メモリリーク回避策
+(3) area_truncated 判定の正確な定義（'メッシュ地理範囲外' = フリンジ含むか含まないか、1px海面ボーダーの扱い）
+(4) ピーク座標がメッシュ境界に近い場合の Flood Fill 挙動（隣接メッシュの標高データを参照すべきか）
+(5) ピーク数百件の per-mesh GeoJSON 出力性能・ファイルサイズ実測値の事前見積
+(6) cv::findContours の RETR_EXTERNAL モードと、複数 contour が返るケース（ピークが薄い橋でつながっている場合等）の扱い
+(7) GeoJSON シリアライズ時の座標精度（小数点何桁）と、形状再現性への影響</t>
+        </is>
+      </c>
       <c r="N41" s="7" t="inlineStr"/>
       <c r="O41" s="7" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
chore: issues_export.xlsx を再生成（ISSUE-033/021 対応完了反映）
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -280,12 +280,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'収束グラフ'!$A$2:$A$22</f>
+              <f>'収束グラフ'!$A$2:$A$23</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'収束グラフ'!$B$2:$B$22</f>
+              <f>'収束グラフ'!$B$2:$B$23</f>
             </numRef>
           </yVal>
         </ser>
@@ -314,12 +314,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'収束グラフ'!$A$2:$A$22</f>
+              <f>'収束グラフ'!$A$2:$A$23</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'収束グラフ'!$C$2:$C$22</f>
+              <f>'収束グラフ'!$C$2:$C$23</f>
             </numRef>
           </yVal>
         </ser>
@@ -348,12 +348,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'収束グラフ'!$A$2:$A$22</f>
+              <f>'収束グラフ'!$A$2:$A$23</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'収束グラフ'!$D$2:$D$22</f>
+              <f>'収束グラフ'!$D$2:$D$23</f>
             </numRef>
           </yVal>
         </ser>
@@ -364,7 +364,7 @@
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="46159"/>
+          <max val="46160"/>
           <min val="46139"/>
         </scaling>
         <axPos val="l"/>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr"/>
@@ -2211,7 +2211,11 @@
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr"/>
-      <c r="N22" s="4" t="inlineStr"/>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
       <c r="O22" s="4" t="inlineStr"/>
     </row>
     <row r="23" ht="40" customHeight="1">
@@ -2934,7 +2938,7 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr"/>
@@ -2947,7 +2951,11 @@
         </is>
       </c>
       <c r="M34" s="4" t="inlineStr"/>
-      <c r="N34" s="4" t="inlineStr"/>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
       <c r="O34" s="4" t="inlineStr"/>
     </row>
     <row r="35" ht="40" customHeight="1">
@@ -3498,7 +3506,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -3518,7 +3526,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -3744,7 +3752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4069,6 +4077,20 @@
         <v>13</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="12" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B23" t="n">
+        <v>40</v>
+      </c>
+      <c r="C23" t="n">
+        <v>12</v>
+      </c>
+      <c r="D23" t="n">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
refactor: is_tile_top → key_col_unresolved リネーム + dominant peak 特定アルゴリズム改訂
- フラグ名 is_tile_top を key_col_unresolved に全置換（SRS/ADR-004/ADR-008/GLOSSARY/モックアップ）
  - 旧名称はタイル(256×256px)の最頂点と誤読されやすかったため改名
  - area_truncated と並ぶ「未解決フラグ」として命名を統一
- ADR-008 dominant peak 特定アルゴリズム全面改訂（ISSUE-014 対応中）
  - タイブレーク: Haversine 最近接 → 最小プロミネンス（地形学的により適切）
  - フォールバック廃止: 包含なし時はログ警告 + 処理中止（稀少ケースのため人手判断）
  - 実装補足追加: 処理方向・STRtree 空間インデックス・複数 delete サミットの扱い
- SRS FR-009 主ピーク特定ロジックを ADR-008 新方針に整合
- ISSUE-014 ステータス 対応完了 → 対応中（設計再変更のため）
- lessons.md にフラグ命名教訓を追記

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -1767,12 +1767,20 @@
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>対応完了</t>
+          <t>対応中</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr"/>
-      <c r="L15" s="7" t="inlineStr"/>
-      <c r="M15" s="7" t="inlineStr"/>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>ADR-008 の dominant peak 特定アルゴリズムを全面改訂。タイブレーク: Haversine 最近接 → 最小プロミネンスに変更。フォールバック廃止（包含なし時はログ警告 + 処理中止）。SRS FR-009 の主ピーク特定ロジックも同様に更新。フラグ名 is_tile_top → key_col_unresolved にリネーム（SRS 全体・ADR-004・ADR-008・GLOSSARY の全箇所を更新）。実装コード（src/*.c 等）への追従は別タスク（本 ISSUE のスコープ外）。</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>【設計変更 2026-05-19】タイブレーク「Haversine 最近接」を「最小プロミネンス」に変更。最小プロミネンスのピークが地形学的に delete 候補サミットと同一の局所的な隆起を表すため。フォールバック廃止: フェーズ3.5 広域再解析後に包含なしが残るのは陸地最高峰のみと想定され稀少なため、自動処理せず中止 + 個別対応とする。フラグ名 is_tile_top はタイル（256×256px）の最頂点と誤読されやすいため key_col_unresolved に改名。実装コード追従 ISSUE は今後起票予定。</t>
+        </is>
+      </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
           <t>2026-05-10</t>
@@ -2906,17 +2914,17 @@
       <c r="O33" s="7" t="inlineStr"/>
     </row>
     <row r="34" ht="40" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>ISSUE-033</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>SRS FR-018: FR-014 参照記述の整合性修正（フェーズ構成組み替えの取り残し）</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>ISSUE-018 確認時に Opus が独立検証で発見した残課題。2026-05-16 のフェーズ構成組み替えで FR-014 を per-mesh フェーズ2 へ移動したが、SRS FR-018 本文に旧設計の記述が残っている。
 - L291: 「（いずれも FR-014 で後処理される）」← FR-014 はフェーズ2 で完了済みのため矛盾
@@ -2924,7 +2932,7 @@
 - L304（FR-009 入力）: FR-014 完了タイミングの表現が薄く、読み手依存になっている可能性</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>設計</t>
         </is>
@@ -2934,29 +2942,29 @@
           <t>高</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>解析エンジン</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr"/>
-      <c r="H34" s="4" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="J34" s="4" t="inlineStr">
-        <is>
-          <t>対応完了</t>
-        </is>
-      </c>
-      <c r="K34" s="4" t="inlineStr"/>
-      <c r="L34" s="4" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>(1) L291 の括弧書き「（いずれも FR-014 で後処理される）」を削除またはフェーズ2 完了済み前提の表現に修正
 (2) L294 を削除または FR-009 入力として使う旨に修正
@@ -2964,13 +2972,27 @@
 (4) フェーズ2 内の FR-016 → FR-014 → FR-007 の処理順序が SRS から読み取れるかも合わせて確認</t>
         </is>
       </c>
-      <c r="M34" s="4" t="inlineStr"/>
-      <c r="N34" s="4" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>当初方針（フェーズ2 配置前提の参照記述整合化）から大幅に範囲拡大。
+FR-014 をフェーズ3.5（新設）に移し、縮小版パイプラインのループ構造
+（N=4→5→6 エスカレーション、per-mesh エンジンを広域モードで再呼び出し
+→ FR-008/FR-018 再実行で merged 再生成）として全面書き直し。
+関連 FR（FR-004/006/008/009/016/018）も整合化。ISSUE-021 同時解消。
+詳細は ADR-004（決定日 2026-05-18 追記）を参照。
+関連 commit: 8f273a8（暫定・却下）→ 282f427（確定）</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="O34" s="4" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="40" customHeight="1">
       <c r="A35" s="7" t="inlineStr">
@@ -3480,7 +3502,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4">
@@ -3490,7 +3512,7 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -3501,7 +3523,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>25.0%</t>
         </is>
       </c>
     </row>
@@ -3530,7 +3552,7 @@
         </is>
       </c>
       <c r="B9" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -3540,7 +3562,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -3550,7 +3572,7 @@
         </is>
       </c>
       <c r="B11" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -3578,7 +3600,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
@@ -3646,7 +3668,7 @@
         </is>
       </c>
       <c r="B23" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
@@ -3664,7 +3686,7 @@
         </is>
       </c>
       <c r="B26" s="11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
@@ -3722,7 +3744,7 @@
         </is>
       </c>
       <c r="B33" s="11" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="34">
@@ -4162,7 +4184,7 @@
         <v>16</v>
       </c>
       <c r="D24" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: issues_export.xlsx 更新（ISSUE-025/020 解決済反映）
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -279,12 +279,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$26</f>
+              <f>'収束グラフ'!$A$2:$A$27</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$B$2:$B$26</f>
+              <f>'収束グラフ'!$B$2:$B$27</f>
             </numRef>
           </val>
         </ser>
@@ -314,12 +314,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$26</f>
+              <f>'収束グラフ'!$A$2:$A$27</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$C$2:$C$26</f>
+              <f>'収束グラフ'!$C$2:$C$27</f>
             </numRef>
           </val>
         </ser>
@@ -349,12 +349,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$26</f>
+              <f>'収束グラフ'!$A$2:$A$27</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$D$2:$D$26</f>
+              <f>'収束グラフ'!$D$2:$D$27</f>
             </numRef>
           </val>
         </ser>
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1047,7 +1047,7 @@
       <c r="L4" s="4" t="inlineStr"/>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>着手前に plan.md の Ph.2〜Ph.5 設計と現在のアーキテクチャの整合を確認すること。ref/SOTA-Summit-list-revision-request.xlsx の列定義を事前確認。</t>
+          <t>【2026-05-22 更新】MOVED/ELEV_CHANGE シート言及は廃止。最新仕様: 変更行 = is_band_change_candidate=true の matched ピーク（FR-011）。変更前標高=sota_alt_m、変更後標高=round(peak_elev)、山岳名は変更前後同値。根拠文は自動生成（FR-011 ※5参照）。名称変更申請は廃止されたため変更シートは標高バンド遷移のみ対象。</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr"/>
@@ -2121,17 +2121,17 @@
       </c>
     </row>
     <row r="21" ht="40" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>ISSUE-020</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>FR-013 / FR-014: 手動調査待ちピークの GeoJSON フィーチャ扱い</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>URD/SRS レビュー指摘 H-5。FR-014 で 5×5 エスカレーション後も is_tile_top=1 が残るピークは '手動調査待ち' としてフラグ維持のまま処理継続するが、このピークは:
 (1) FR-016 によりコル等高線が生成されない（is_tile_top=1 はコル等高線非生成）
@@ -2139,7 +2139,7 @@
 ため矛盾する。area_truncated=true が 4×4 でも解消しなかったケースの挙動も FR-014 で未規定。</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>設計</t>
         </is>
@@ -2149,29 +2149,29 @@
           <t>高</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>GeoJSON出力</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr"/>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>対応完了</t>
-        </is>
-      </c>
-      <c r="K21" s="7" t="inlineStr"/>
-      <c r="L21" s="7" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>delete判定ゾーンポリゴン方式（max(col_elev, peak_elev - delete_zone_max_drop) 以上の Flood Fill）を採用し、コル等高線ポリゴンを廃止。実装可能な仕様レベルまで確定。
 Phase A 完了（SRS / ADR / GLOSSARY 改修）:
@@ -2191,7 +2191,7 @@
 - ISSUE-045: params/config.ini.example に delete_zone_max_drop = 250 追加</t>
         </is>
       </c>
-      <c r="M21" s="7" t="inlineStr">
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>【議論結論 2026-05-21】
 - 旧3案（A/B/C）は破棄。delete判定ゾーンポリゴン方式を採用。
@@ -2223,12 +2223,16 @@
 - HTML ビューア（merged_viewer.html）実装範囲</t>
         </is>
       </c>
-      <c r="N21" s="7" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="O21" s="7" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="40" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -2478,22 +2482,22 @@
       <c r="O25" s="7" t="inlineStr"/>
     </row>
     <row r="26" ht="40" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>ISSUE-025</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>FR-009 等: 標高バンド境界値（points 1/2/4/6/8/10）の規定</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>URD/SRS レビュー指摘 M-5。FR-009 / FR-013 / FR-012 の points / sota_points カラムで '標高バンドに基づくポイント数（1/2/4/6/8/10）' とあるが、各バンドの標高境界値（何 m 以上で何 pt）が SRS にない。sotl.as 由来のはずだが SOTA 日本支部の正式表との対応を SRS / GLOSSARY で明示すべきか HLD で十分か議論が必要。緯度依存の可能性もあり。</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>設計</t>
         </is>
@@ -2503,36 +2507,48 @@
           <t>中</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>merge.py</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr"/>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>未対応</t>
-        </is>
-      </c>
-      <c r="K26" s="4" t="inlineStr"/>
-      <c r="L26" s="4" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>FR-009 の用語定義または GLOSSARY で標高バンド境界表を提示する（SOTA 日本支部の正式表を出典として引用）。緯度区分がある場合は区分も含めて表で記述。</t>
         </is>
       </c>
-      <c r="M26" s="4" t="inlineStr"/>
-      <c r="N26" s="4" t="inlineStr"/>
-      <c r="O26" s="4" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>【2026-05-22 対応完了】GLOSSARY に SOTA 日本支部参照マニュアル（2025年7月改定版）に基づく標高バンド表を追加（全国統一・地域依存なし）。SRS FR-009 に変更申請判定（Points バンド遷移）セクションを追加し、GLOSSARY への参照リンクで出典を明示。ref/SOURCES.md にも出典エントリを追加。本 ISSUE は ISSUE-046（変更申請判定スコープ変更）に統合。</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="40" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -3746,35 +3762,7 @@
       <c r="L44" s="4" t="inlineStr"/>
       <c r="M44" s="4" t="inlineStr">
         <is>
-          <t>【作業範囲】
-1. per-mesh activation.geojson から AZ ポリゴン（feature_type='activation_zone'）と delete判定ゾーンポリゴン（feature_type='delete_zone'）を読み込む
-2. 各ポリゴンに対して shapely.strtree.STRtree で空間インデックス構築
-3. summit.match_status 判定（SRS FR-009 / ADR-011）:
-   - matched: いずれかのピークの AZ 内
-   - delete: いずれかのピークの delete判定ゾーン内かつ AZ 外
-   - unmatched: いずれにも該当しない（エラー）
-4. peak.match_status 判定（ADR-007 / ADR-008）:
-   - matched: ピークの AZ 内に既存サミット座標あり
-   - dominant: ピークの delete判定ゾーン内かつ AZ 外に既存サミット座標あり（複数ピーク該当時は最小プロミネンスを採用）
-   - new: いずれにも該当せず
-5. merged.csv に不備フラグ列追加（いずれか true なら non-zero exit）:
-   - is_unmatched_summit
-   - is_area_incomplete（FR-018 統合後も area_complete=true が見つからない）
-   - is_key_col_unresolved（FR-014 広域でも未確定）
-   - is_out_of_range_summit（解析範囲外のサミット）
-   - is_dem_invalid_summit（DEM が NODATA）
-6. 既存の peak.match_status 出力値: deleted → dominant にリネーム（ADR-007）
-7. summit.match_status 出力値: deleted → delete にリネーム（ADR-007）
-【検証ポイント】
-- 九州・四国の既存解析結果に新ロジック適用 → 削除 6 件すべて delete 判定
-- 不備フラグが立つテストケースで non-zero exit を確認
-【依存関係】
-- ISSUE-040（C++/OpenCV で FR-016 実装）完了後、per-mesh activation.geojson が出力される必要がある
-- ただし Python 側の実装はモック GeoJSON で先行可能
-【参照】
-- SRS docs/02_SRS.md FR-009 / FR-013 / 6.8 / 6.11
-- ADR docs/decisions/ADR-007 / ADR-008 / ADR-011
-【元 ISSUE】ISSUE-020 から分離（設計フェーズは完結、これは実装フェーズ）</t>
+          <t>【2026-05-22 追記】merge.py 改修スコープに以下を追加: points/sota_points/is_band_change_candidate 列の計算・追加（FR-009 変更申請判定セクション参照）。バンド定義は GLOSSARY 標高バンド（Points 算出表）に従う。peak_elev は切り捨て（floor）した整数 m でバンド判定（例: 1499.5m → 1499m → 8pt）、sota_alt_m はそのまま判定。</t>
         </is>
       </c>
       <c r="N44" s="4" t="inlineStr"/>
@@ -3835,26 +3823,7 @@
       <c r="L45" s="7" t="inlineStr"/>
       <c r="M45" s="7" t="inlineStr">
         <is>
-          <t>【作業範囲】
-1. dominant フィーチャ構成変更:
-   - 旧: コル等高線ポリゴン（feature_type='key_col_boundary'）→ 廃止
-   - 新: delete判定ゾーンポリゴン（feature_type='delete_zone'）→ dominant ピークに付与
-2. summit.match_status の出力値変更: deleted → delete
-3. peak.match_status の出力値変更: deleted → dominant
-4. merged.csv の不備フラグ列確認、いずれか true なら実行スキップ（merge.py が non-zero exit するため二重チェック）
-5. merged_viewer.html の実装（SRS FR-013 で要求済みだが未実装）:
-   - peak の matched / new / dominant をフィルタ UI で切替表示
-   - summit の matched / delete をフィルタ表示
-   - HTML データ属性 data-cat に dominant / delete を分けて格納
-【検証ポイント】
-- 地理院地図上で AZ・delete判定ゾーン両ポリゴンが目視確認できる
-- HTML ビューアで peak/summit のフィルタ切替が動く
-【依存関係】
-- ISSUE-043（merge.py 改修）完了後に着手するのが自然
-【参照】
-- SRS docs/02_SRS.md FR-013
-- ADR docs/decisions/ADR-007 / ADR-011
-【元 ISSUE】ISSUE-020 から分離（設計フェーズは完結、これは実装フェーズ）</t>
+          <t>【2026-05-22 追記】output_geojson.py + merged_viewer.html 改修スコープに以下を追加: (1) 名称修正 UI 廃止（matched ピークの入力フィールドを削除）。(2) 変更行自動エクスポート（is_band_change_candidate=true の matched ピークを申請書の変更行として自動生成、FR-011 ※5フォーマット準拠）。</t>
         </is>
       </c>
       <c r="N45" s="7" t="inlineStr"/>
@@ -3928,18 +3897,75 @@
       <c r="N46" s="4" t="inlineStr"/>
       <c r="O46" s="4" t="inlineStr"/>
     </row>
+    <row r="47" ht="40" customHeight="1">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-046</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>SRS: 変更申請判定を Points バンド遷移基準に変更（URD/SRS/GLOSSARY 改訂）</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>SOTA 申請「変更」の定義を「山岳名の変更」から「matched ペアで Points バンドをまたぐ標高差があるケース（is_band_change_candidate=true）」に再定義。山岳名変更は申請対象外（ピーク解析と無関係）。URD UR-003・6.スコープ外、SRS FR-007/009/011/012/013・9.スコープ外、GLOSSARY（標高バンド表追加）、ref/SOURCES.md を改訂。ISSUE-025（標高バンド境界値の規定）を本タスクに統合。</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="I47" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J47" s="7" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="K47" s="7" t="inlineStr"/>
+      <c r="L47" s="7" t="inlineStr"/>
+      <c r="M47" s="7" t="inlineStr"/>
+      <c r="N47" s="7" t="inlineStr"/>
+      <c r="O47" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation sqref="J2:J46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3975,7 +4001,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3">
@@ -3985,7 +4011,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
@@ -3995,7 +4021,7 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -4006,7 +4032,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>28.9%</t>
+          <t>32.6%</t>
         </is>
       </c>
     </row>
@@ -4025,7 +4051,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9">
@@ -4055,7 +4081,7 @@
         </is>
       </c>
       <c r="B11" s="11" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
@@ -4093,7 +4119,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17">
@@ -4151,7 +4177,7 @@
         </is>
       </c>
       <c r="B23" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -4179,7 +4205,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
@@ -4189,7 +4215,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -4209,7 +4235,7 @@
         </is>
       </c>
       <c r="B30" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32">
@@ -4237,7 +4263,7 @@
         </is>
       </c>
       <c r="B34" s="11" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35">
@@ -4281,7 +4307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4712,6 +4738,22 @@
         <v>17</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>46</v>
+      </c>
+      <c r="C27" t="n">
+        <v>19</v>
+      </c>
+      <c r="D27" t="n">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
mgmt: ISSUE-047 対応完了（phase1.drawio FR-002/003 除去）
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -4006,7 +4006,7 @@
       </c>
       <c r="J48" s="4" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="K48" s="4" t="inlineStr"/>
@@ -4016,7 +4016,11 @@
         </is>
       </c>
       <c r="M48" s="4" t="inlineStr"/>
-      <c r="N48" s="4" t="inlineStr"/>
+      <c r="N48" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
       <c r="O48" s="4" t="inlineStr"/>
     </row>
     <row r="49" ht="40" customHeight="1">
@@ -4287,7 +4291,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
@@ -4307,7 +4311,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -4984,7 +4988,7 @@
         <v>50</v>
       </c>
       <c r="C27" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D27" t="n">
         <v>20</v>

</xml_diff>

<commit_message>
mgmt: ISSUE-047 解決済・ISSUE-048/049 対応完了
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -4071,7 +4071,7 @@
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
-          <t>対応中</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="K49" s="7" t="inlineStr"/>
@@ -4081,7 +4081,11 @@
         </is>
       </c>
       <c r="M49" s="7" t="inlineStr"/>
-      <c r="N49" s="7" t="inlineStr"/>
+      <c r="N49" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
       <c r="O49" s="7" t="inlineStr"/>
     </row>
     <row r="50" ht="40" customHeight="1">
@@ -4128,7 +4132,7 @@
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>対応中</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="K50" s="4" t="inlineStr"/>
@@ -4138,7 +4142,11 @@
         </is>
       </c>
       <c r="M50" s="4" t="inlineStr"/>
-      <c r="N50" s="4" t="inlineStr"/>
+      <c r="N50" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
       <c r="O50" s="4" t="inlineStr"/>
     </row>
     <row r="51" ht="40" customHeight="1">
@@ -4305,7 +4313,7 @@
         </is>
       </c>
       <c r="B9" s="11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -4315,7 +4323,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -4992,7 +5000,7 @@
         <v>50</v>
       </c>
       <c r="C27" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D27" t="n">
         <v>21</v>

</xml_diff>

<commit_message>
mgmt: plan.md 更新・issues_export.xlsx 再生成（2026-05-23）
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -279,12 +279,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$27</f>
+              <f>'収束グラフ'!$A$2:$A$28</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$B$2:$B$27</f>
+              <f>'収束グラフ'!$B$2:$B$28</f>
             </numRef>
           </val>
         </ser>
@@ -314,12 +314,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$27</f>
+              <f>'収束グラフ'!$A$2:$A$28</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$C$2:$C$27</f>
+              <f>'収束グラフ'!$C$2:$C$28</f>
             </numRef>
           </val>
         </ser>
@@ -349,12 +349,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$27</f>
+              <f>'収束グラフ'!$A$2:$A$28</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$D$2:$D$27</f>
+              <f>'収束グラフ'!$D$2:$D$28</f>
             </numRef>
           </val>
         </ser>
@@ -3762,7 +3762,8 @@
       <c r="L44" s="4" t="inlineStr"/>
       <c r="M44" s="4" t="inlineStr">
         <is>
-          <t>【2026-05-22 追記】merge.py 改修スコープに以下を追加: points/sota_points/is_band_change_candidate 列の計算・追加（FR-009 変更申請判定セクション参照）。バンド定義は GLOSSARY 標高バンド（Points 算出表）に従う。peak_elev は切り捨て（floor）した整数 m でバンド判定（例: 1499.5m → 1499m → 8pt）、sota_alt_m はそのまま判定。</t>
+          <t>【2026-05-22 追記】merge.py 改修スコープに以下を追加: points/sota_points/is_band_change_candidate 列の計算・追加（FR-009 変更申請判定セクション参照）。バンド定義は GLOSSARY 標高バンド（Points 算出表）に従う。peak_elev は切り捨て（floor）した整数 m でバンド判定（例: 1499.5m → 1499m → 8pt）、sota_alt_m はそのまま判定。
+【2026-05-23 補正】merge.py の出力は merged.csv（ピーク台帳・ステータス・不備フラグ）と merged_activation.geojson（AZ・delete判定ゾーンポリゴンの per-mesh 統合）の2系統（SRS FR-018 参照）。AZ/delete-zone PIP 判定の素材は per-mesh activation GeoJSON。不備フラグ・exit code 判定は merged.csv 側で完結する。</t>
         </is>
       </c>
       <c r="N44" s="4" t="inlineStr"/>
@@ -3823,7 +3824,8 @@
       <c r="L45" s="7" t="inlineStr"/>
       <c r="M45" s="7" t="inlineStr">
         <is>
-          <t>【2026-05-22 追記】output_geojson.py + merged_viewer.html 改修スコープに以下を追加: (1) 名称修正 UI 廃止（matched ピークの入力フィールドを削除）。(2) 変更行自動エクスポート（is_band_change_candidate=true の matched ピークを申請書の変更行として自動生成、FR-011 ※5フォーマット準拠）。</t>
+          <t>【2026-05-22 追記】output_geojson.py + merged_viewer.html 改修スコープに以下を追加: (1) 名称修正 UI 廃止（matched ピークの入力フィールドを削除）。(2) 変更行自動エクスポート（is_band_change_candidate=true の matched ピークを申請書の変更行として自動生成、FR-011 ※5フォーマット準拠）。
+【2026-05-23 補正】output_geojson.py の入力は merged.csv + merged_activation.geojson の2系統（SRS FR-013 参照）。ポリゴン情報（AZ・delete判定ゾーン）は merged_activation.geojson から取り込む。出力は merged.geojson（Point + LineString + Polygon の可視化集約）と merged_viewer.html。</t>
         </is>
       </c>
       <c r="N45" s="7" t="inlineStr"/>
@@ -4567,7 +4569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5014,6 +5016,22 @@
         <v>23</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>50</v>
+      </c>
+      <c r="C28" t="n">
+        <v>23</v>
+      </c>
+      <c r="D28" t="n">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
chore: ISSUE-050 クローズ・課題 Excel 更新
機能関連図は不要と判断、ISSUE-050 を対応完了とした。

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -4203,7 +4203,7 @@
       </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="K51" s="7" t="inlineStr"/>
@@ -4213,7 +4213,11 @@
         </is>
       </c>
       <c r="M51" s="7" t="inlineStr"/>
-      <c r="N51" s="7" t="inlineStr"/>
+      <c r="N51" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
       <c r="O51" s="7" t="inlineStr"/>
     </row>
   </sheetData>
@@ -4313,7 +4317,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9">
@@ -4333,7 +4337,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -5026,7 +5030,7 @@
         <v>50</v>
       </c>
       <c r="C28" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D28" t="n">
         <v>23</v>

</xml_diff>

<commit_message>
chore: ISSUE-043/044/045 発生ステージを COD → SRS に修正
現在は SRS ステージのため、merge.py・GeoJSON出力・config.ini.example 改修課題の
発生ステージを実態に合わせて修正。

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -3750,7 +3750,7 @@
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>SRS</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
@@ -3812,7 +3812,7 @@
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>SRS</t>
         </is>
       </c>
       <c r="J45" s="7" t="inlineStr">
@@ -3874,7 +3874,7 @@
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>SRS</t>
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr">
@@ -4545,7 +4545,7 @@
         </is>
       </c>
       <c r="B34" s="11" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="35">
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B36" s="11" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">

</xml_diff>

<commit_message>
chore: 課題整理・SRS/URD/GLOSSARY 補完・tracker 機能追加
【課題整理】
- ISSUE-003（output_xlsx.py）: 却下（URD/SRS 再設計に伴い廃止）
- ISSUE-005（九州・四国統合テスト）: 却下（同上）
- ISSUE-009/013: 担当者 Claude・対応方針を記入
- ISSUE-022/023/027/028/030/034/035/036: 対応完了
- 未対応課題 16 件に対応予定ステージを設定
- ISSUE-043/044/045: 発生ステージ COD → SRS に修正

【SRS/URD/GLOSSARY 補完】
- FR-017: 北方領土タイル判定基準（タイル中心点）を明示（ISSUE-022）
- NFR-003: timestamp 除外規定を追記（ISSUE-023）
- GLOSSARY: 「削除候補サミット」を独立項目として追加（ISSUE-027）
- SRS: フォールバック規定を FR-017 に集約（ISSUE-028）
- URD UR-006: HTML ビューア 2 層構造を明記（ISSUE-030）
- SRS: 竹島除外方針を前提・制約・スコープ外・FR-003 に追記（ISSUE-035）
- params/mesh_list_japan.txt: 5531 をコメントアウト形式で除外（ISSUE-036）

【tracker 機能追加】
- issue に「対応予定ステージ」フィールドを追加
- 却下時に verified_date を自動設定するよう修正

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -67,17 +67,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EBF3FB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFFBE0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF3FB"/>
       </patternFill>
     </fill>
     <fill>
@@ -133,13 +133,13 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O51"/>
+  <dimension ref="A1:P51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -753,12 +753,13 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
     <col width="30" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -809,30 +810,35 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>対応予定ステージ</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>ステータス</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>担当者</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>対応方針</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>備考</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>対応完了日</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>解決確認日</t>
         </is>
@@ -884,32 +890,33 @@
           <t>IT</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>python3 scripts/merge.py --mesh-list params/mesh_5339_neighbors.txt を実行して結果確認</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>ステップ1（prefetch）・ステップ2（findsummits 9メッシュ解析）は完了済み</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -961,50 +968,51 @@
           <t>COD</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>却下</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>ISSUE-001（ステップ3検証）の後に着手。突合列: match_status, summit_code, summit_name, peak_lat, peak_lon, peak_elev, col_lat, col_lon, col_elev, prominence, orig_lat, orig_lon, orig_elev</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>ISSUE-003</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>output_xlsx.py 新規作成（申請用XLSX生成）</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>openpyxl で SOTA申請用 XLSX を生成するスクリプト。新規シート(NEW)・変更シート(MOVED/ELEV_CHANGE)・削除シート(DELETED)・変更なしシート(MATCH)の4シート構成。prominence &lt; 150m の行は黄色ハイライト。</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>機能追加</t>
         </is>
@@ -1014,44 +1022,53 @@
           <t>高</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>その他</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>2026-04-27</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>COD</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>未対応</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>却下</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr"/>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>URD/SRS 再設計に伴い廃止。output_xlsx.py の仕様は SRS 確定後に改めて起票する。元の説明にあった4シート構成はテンプレート未確認のまま Claude が設計した誤り（実際は1シート縦並び）。</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>【2026-05-22 更新】MOVED/ELEV_CHANGE シート言及は廃止。最新仕様: 変更行 = is_band_change_candidate=true の matched ピーク（FR-011）。変更前標高=sota_alt_m、変更後標高=round(peak_elev)、山岳名は変更前後同値。根拠文は自動生成（FR-011 ※5参照）。名称変更申請は廃止されたため変更シートは標高バンド遷移のみ対象。</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr"/>
-      <c r="O4" s="4" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -1074,7 +1091,7 @@
           <t>機能追加</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -1099,97 +1116,107 @@
           <t>COD</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>SOTA スコア別色（MATCHのみ）: 10点=赤, 8点=黄, 6点=緑, 4点=シアン, 2点=青, 1点=紫</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>2026-04-27</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>2026-04-27</t>
         </is>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>ISSUE-005</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>九州・四国メッシュでの統合テスト</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>フルパイプ検証（9メッシュ）が通った後、九州・四国メッシュで end-to-end テストを実施。findsummits4sotaja の過去結果（sotaJA_SummitPeakCol_All5.xlsx）と比較。許容差: ピーク座標 ±100m、標高 ±5m、プロミネンス ±20m。</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>調査</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>解析エンジン</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>2026-04-27</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>ST</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>未対応</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>却下</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr"/>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>URD/SRS 再設計に伴い廃止。</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>複数メッシュ境界付近の既知の山が GeoJSON で正しく1件表示されることも確認。DEM5なしメッシュの DEM10 フォールバック結果の妥当性も確認。</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr"/>
-      <c r="O6" s="4" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -1212,7 +1239,7 @@
           <t>改善</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -1237,28 +1264,29 @@
           <t>IT</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>却下</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>ISSUE-001 完了後に着手</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -1285,7 +1313,7 @@
           <t>改善</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>低</t>
         </is>
@@ -1310,28 +1338,29 @@
           <t>OPS</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>却下</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>フルパイプ検証前に仕様を詰めても実行時の問題で仕様変更になりやすいため後回し</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -1383,97 +1412,107 @@
           <t>HLD</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>却下</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>plan_v1.md: .claude/mgmt/plan_v1.md</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="O9" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="P9" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>ISSUE-009</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>新規サミット仮コードへの地域コード自動付与</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>現在は仮コードが ZZ/ZZ-001 形式の連番。座標から都道府県を判定し、SOTA JA のアソシエーション/リージョンコード（北海道・本州・四国・九州）を仮コードに反映できるか実装を検討する。</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>機能追加</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>merge.py</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>2026-04-27</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>HLD</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
         <is>
           <t>未対応</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>JJ1XGO</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr"/>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>SRS FR-009 に仕様記述済み。COD ステージで preprocess_pref_boundaries.py を実行して N03 GeoJSON を生成後に実装する。</t>
+        </is>
+      </c>
+      <c r="N10" s="6" t="inlineStr">
         <is>
           <t>将来実装候補。フルパイプ検証・申請用出力フェーズ完了後に検討。</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr"/>
-      <c r="O10" s="4" t="inlineStr"/>
+      <c r="O10" s="6" t="inlineStr"/>
+      <c r="P10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -1496,7 +1535,7 @@
           <t>改善</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -1517,28 +1556,29 @@
           <t>OPS</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>requirements.txt・.gitignore・CLAUDE.md は小規模な編集。README.md は現状に合わせて内容を整理してから更新する</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr"/>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr">
+      <c r="P11" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -1565,7 +1605,7 @@
           <t>改善</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -1586,24 +1626,25 @@
           <t>OPS</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>CLAUDE.mdのルールと制約セクションに追記</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="P12" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -1630,7 +1671,7 @@
           <t>設計</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -1651,81 +1692,91 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>スコープ外として対応しない。matched サミットの座標・標高変更は本プロジェクトでは自動識別しない。既存登録情報は概ね正しいと判断。URD UR-003・スコープ外セクションに反映済み。</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr"/>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr">
         <is>
           <t>2026-05-10</t>
         </is>
       </c>
-      <c r="O13" s="2" t="inlineStr">
+      <c r="P13" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
     </row>
     <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>ISSUE-013</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>prefetch_tiles.py の取得範囲を各メッシュの最小範囲に修正</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>現在の enumerate_jobs() は隣接メッシュが mesh_set に含まれる場合にタイル取得範囲を拡張しているが、正しい仕様は各メッシュをカバーする最小範囲（mesh_to_tile_range(meshcode) のみ）のタイルを取得すること。隣接メッシュ拡張ロジック（nb not in mesh_set の分岐）を削除し、各メッシュ単独の範囲のみを取得するよう修正する。全176メッシュを一括取得する運用では境界付近のタイルが複数メッシュから重複取得されるが問題ない。</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>改善</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr"/>
-      <c r="G14" s="4" t="inlineStr"/>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>COD</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>未対応</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>JJ1XGO</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr"/>
-      <c r="M14" s="4" t="inlineStr"/>
-      <c r="N14" s="4" t="inlineStr"/>
-      <c r="O14" s="4" t="inlineStr"/>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>scripts/prefetch_tiles.py の enumerate_jobs() から隣接メッシュ拡張ロジック（nb not in mesh_set の分岐）を削除し、各メッシュ単独の mesh_to_tile_range(meshcode) のみを取得するよう修正する。</t>
+        </is>
+      </c>
+      <c r="N14" s="6" t="inlineStr"/>
+      <c r="O14" s="6" t="inlineStr"/>
+      <c r="P14" s="6" t="inlineStr"/>
     </row>
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -1748,7 +1799,7 @@
           <t>機能追加</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -1765,28 +1816,29 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>ADR-008 の dominant peak 特定アルゴリズムを全面改訂。タイブレーク: Haversine 最近接 → 最小プロミネンスに変更。フォールバック廃止（包含なし時はログ警告 + 処理中止）。SRS FR-009 の主ピーク特定ロジックも同様に更新。フラグ名 is_tile_top → key_col_unresolved にリネーム（SRS 全体・ADR-004・ADR-008・GLOSSARY の全箇所を更新）。実装コード（src/*.c 等）への追従は別タスク（本 ISSUE のスコープ外）。</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>【設計変更 2026-05-19】タイブレーク「Haversine 最近接」を「最小プロミネンス」に変更。最小プロミネンスのピークが地形学的に delete 候補サミットと同一の局所的な隆起を表すため。フォールバック廃止: フェーズ3.5 広域再解析後に包含なしが残るのは陸地最高峰のみと想定され稀少なため、自動処理せず中止 + 個別対応とする。フラグ名 is_tile_top はタイル（256×256px）の最頂点と誤読されやすいため key_col_unresolved に改名。【追加変更 2026-05-19】さらに肯定形に統一するため key_col_unresolved → key_col_resolved、並列フラグ area_truncated → area_complete に再リネーム（共に true=正常 で真偽値方向を揃えた）。実装コード追従 ISSUE は今後起票予定。</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="O15" s="2" t="inlineStr">
         <is>
           <t>2026-05-10</t>
         </is>
       </c>
-      <c r="O15" s="2" t="inlineStr">
+      <c r="P15" s="2" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -1813,7 +1865,7 @@
           <t>機能追加</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -1830,24 +1882,25 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>GitHub Pages 公開ツールからローカル用HTMLビューア（docs/mockup/viewer_mockup.html）に方針変更。山岳名JP/EN入力フォームとlocalStorage保存を実装。FR-013に仕様として取り込み済み。</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr">
         <is>
           <t>2026-05-13</t>
         </is>
       </c>
-      <c r="O16" s="2" t="inlineStr">
+      <c r="P16" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -1870,7 +1923,7 @@
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr"/>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -1893,18 +1946,27 @@
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
           <t>未対応</t>
         </is>
       </c>
-      <c r="K17" s="7" t="inlineStr">
+      <c r="L17" s="7" t="inlineStr">
         <is>
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="L17" s="7" t="inlineStr"/>
-      <c r="M17" s="7" t="inlineStr"/>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>scripts/merge.py の load_peaks() に --mesh-list 指定時の絞り込みロジックを追加する。指定メッシュコードのセットを受け取り、csv_dir 配下から {meshcode}.csv のみを対象にする。省略時は現行の glob 全読み込みを維持する。</t>
+        </is>
+      </c>
       <c r="N17" s="7" t="inlineStr"/>
       <c r="O17" s="7" t="inlineStr"/>
+      <c r="P17" s="7" t="inlineStr"/>
     </row>
     <row r="18" ht="40" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -1923,7 +1985,7 @@
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -1944,24 +2006,25 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>SRS に FR-018（activation.geojson 統合ステップ）を新設。フェーズ3を FR-008 → FR-018 → FR-014 の構成に再設計し、FR-009 の前に統合済み activation.geojson が参照できるよう仕様化。コミット 5b633f5（2026-05-09）で対応完了。</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr"/>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr">
         <is>
           <t>2026-05-09</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
+      <c r="P18" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -2012,31 +2075,25 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>FR-009 に以下を追記:
-(1) 判定順序を明示: ①AZ 内に SOTA → matched, ②コル等高線内に SOTA → dominant, ③それ以外 → new
-(2) sota_summit feature の match_status を独立定義:
-   matched = FR-010 スコープ内で AZ にマッチ
-   deleted = FR-010 スコープ内で AZ にマッチせず
-(3) ADR-008 フォールバック時の peak.match_status と sota_summit の対応関係を明確化。案A（peak も dominant に昇格）または案B（peak の match_status は変えず sota_summit を独立扱い・FR-013 フィーチャ構成テーブルを更新）から選定。
-(4) GLOSSARY に '削除候補（deleted）' を追加。
-(5) ADR-007 / ADR-008 とも整合チェック。</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr"/>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>案 B（peak.match_status は変更せず、summit.dominant_peak_code で紐付けのみ）を採用。peak は常に match_status=new のまま、delete サミットが従属する dominant peak を dominant_peak_code で参照する形で実装。SRS FR-009・ADR-008 L29 参照。</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr">
         <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="O19" s="2" t="inlineStr">
+      <c r="P19" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -2084,13 +2141,14 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>FR-009 に追記:
 (1) 採番順序を明示（推奨: peak_lat 降順 → peak_lon 昇順タイブレーク、または (peak_lat, peak_lon) 昇順タプル）
@@ -2098,7 +2156,7 @@
 (3) NFR-003 とのトレース確認</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>【Opus相談推奨】複数の独立した設計判断と副次的影響の整理が必要。
 相談ポイント:
@@ -2109,12 +2167,12 @@
 【2026-05-20 訂正】対応完了コメントに記載した『プロミネンス降順 → peak_lat 降順 → peak_lon 昇順』は Claude の解釈ミス。正しくは『標高降順 → プロミネンス降順 → peak_lat 降順 → peak_lon 昇順』（標高が 1 次キー、プロミネンスは標高同値時のタイブレーク）。SRS FR-009 / NFR-003 も訂正済（commit にて反映）。</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="O20" s="2" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr">
+      <c r="P20" s="2" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2165,13 +2223,14 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>delete判定ゾーンポリゴン方式（max(col_elev, peak_elev - delete_zone_max_drop) 以上の Flood Fill）を採用し、コル等高線ポリゴンを廃止。実装可能な仕様レベルまで確定。
 Phase A 完了（SRS / ADR / GLOSSARY 改修）:
@@ -2191,7 +2250,7 @@
 - ISSUE-045: params/config.ini.example に delete_zone_max_drop = 250 追加</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>【議論結論 2026-05-21】
 - 旧3案（A/B/C）は破棄。delete判定ゾーンポリゴン方式を採用。
@@ -2223,12 +2282,12 @@
 - HTML ビューア（merged_viewer.html）実装範囲</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="O21" s="2" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="P21" s="2" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
@@ -2255,7 +2314,7 @@
           <t>改善</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -2276,20 +2335,21 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr">
         <is>
           <t>FR-014 出力節に以下のいずれかを明示:
 案A: 'per-mesh ファイルは更新せず、merged.csv / merged_activation.geojson のみ更新'
 案B: '中間ファイルも更新する'（再現性向上のため）</t>
         </is>
       </c>
-      <c r="M22" s="2" t="inlineStr">
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>【最終決定】FR-014 は縮小版パイプライン構造を採用:
 - 広域 per-mesh CSV/GeoJSON を新規出力するのみ
@@ -2299,12 +2359,12 @@
 反映先: SRS FR-014 / FR-008 / FR-018、ADR-004 Decision「出力スコープ」</t>
         </is>
       </c>
-      <c r="N22" s="2" t="inlineStr">
+      <c r="O22" s="2" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="O22" s="2" t="inlineStr">
+      <c r="P22" s="2" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -2331,7 +2391,7 @@
           <t>改善</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -2352,77 +2412,95 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J23" s="7" t="inlineStr">
-        <is>
-          <t>未対応</t>
-        </is>
-      </c>
-      <c r="K23" s="7" t="inlineStr"/>
+      <c r="J23" s="7" t="inlineStr"/>
+      <c r="K23" s="7" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
       <c r="L23" s="7" t="inlineStr">
         <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
           <t>FR-017 に 'タイル中心点が北方領土6村ポリゴンに含まれるタイルを列挙' と明示し、ADR-005 と同じ規定を SRS に転記する。</t>
         </is>
       </c>
-      <c r="M23" s="7" t="inlineStr"/>
       <c r="N23" s="7" t="inlineStr"/>
-      <c r="O23" s="7" t="inlineStr"/>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="P23" s="7" t="inlineStr"/>
     </row>
     <row r="24" ht="40" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>ISSUE-023</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>NFR-003: 決定論性スコープから timestamp 除外を明記</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>URD/SRS レビュー指摘 M-3。NFR-003 L527-529 で 'すべての出力が同一の内容になること' とあるが、merged.geojson の metadata.generated_at は実行時刻に依存するため完全な同一性は不可能。</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>改善</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>その他</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr"/>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="I24" s="6" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>未対応</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr"/>
-      <c r="L24" s="4" t="inlineStr">
+      <c r="J24" s="6" t="inlineStr"/>
+      <c r="K24" s="6" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L24" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="M24" s="6" t="inlineStr">
         <is>
           <t>NFR-003 に 'metadata.generated_at 等の実行時タイムスタンプを除き、ピーク座標・標高・突合結果・採番が同一であること' と除外規定を明記。</t>
         </is>
       </c>
-      <c r="M24" s="4" t="inlineStr"/>
-      <c r="N24" s="4" t="inlineStr"/>
-      <c r="O24" s="4" t="inlineStr"/>
+      <c r="N24" s="6" t="inlineStr"/>
+      <c r="O24" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="P24" s="6" t="inlineStr"/>
     </row>
     <row r="25" ht="40" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
@@ -2445,7 +2523,7 @@
           <t>改善</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -2468,18 +2546,23 @@
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="K25" s="7" t="inlineStr">
+        <is>
           <t>未対応</t>
         </is>
       </c>
-      <c r="K25" s="7" t="inlineStr"/>
-      <c r="L25" s="7" t="inlineStr">
+      <c r="L25" s="7" t="inlineStr"/>
+      <c r="M25" s="7" t="inlineStr">
         <is>
           <t>FR-015 に縮小方式を明示する（推奨: max pooling でダウンサンプル、NODATA は除外）。もしくは HLD で規定する旨を SRS に明記。</t>
         </is>
       </c>
-      <c r="M25" s="7" t="inlineStr"/>
       <c r="N25" s="7" t="inlineStr"/>
       <c r="O25" s="7" t="inlineStr"/>
+      <c r="P25" s="7" t="inlineStr"/>
     </row>
     <row r="26" ht="40" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -2502,7 +2585,7 @@
           <t>設計</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -2523,28 +2606,29 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>FR-009 の用語定義または GLOSSARY で標高バンド境界表を提示する（SOTA 日本支部の正式表を出典として引用）。緯度区分がある場合は区分も含めて表で記述。</t>
         </is>
       </c>
-      <c r="M26" s="2" t="inlineStr">
+      <c r="N26" s="2" t="inlineStr">
         <is>
           <t>【2026-05-22 対応完了】GLOSSARY に SOTA 日本支部参照マニュアル（2025年7月改定版）に基づく標高バンド表を追加（全国統一・地域依存なし）。SRS FR-009 に変更申請判定（Points バンド遷移）セクションを追加し、GLOSSARY への参照リンクで出典を明示。ref/SOURCES.md にも出典エントリを追加。本 ISSUE は ISSUE-046（変更申請判定スコープ変更）に統合。</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr">
+      <c r="O26" s="2" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="O26" s="2" t="inlineStr">
+      <c r="P26" s="2" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
@@ -2574,7 +2658,7 @@
           <t>改善</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>低</t>
         </is>
@@ -2595,13 +2679,14 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>表記ルールを SRS 冒頭または GLOSSARY に明示し、全文を統一:
 (1) 本文表記: 'Keyコル'、プロパティ名 / feature_type 値: 'key_col_boundary' に統一
@@ -2609,76 +2694,85 @@
 (3) 'dominant peak' は本文・GLOSSARY 見出しとも英語表記に統一</t>
         </is>
       </c>
-      <c r="M27" s="2" t="inlineStr"/>
-      <c r="N27" s="2" t="inlineStr">
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="O27" s="2" t="inlineStr">
+      <c r="P27" s="2" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
     </row>
     <row r="28" ht="40" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>ISSUE-027</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>GLOSSARY 補完（削除候補・dominant peak 見出し統一）</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>URD/SRS レビュー指摘 L-4。'削除候補（deleted）' が用語集に独立項目として未定義。dominant peak の説明文で言及されるのみ。</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>改善</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>その他</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr"/>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr"/>
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="I28" s="6" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
-          <t>未対応</t>
-        </is>
-      </c>
-      <c r="K28" s="4" t="inlineStr"/>
-      <c r="L28" s="4" t="inlineStr">
+      <c r="J28" s="6" t="inlineStr"/>
+      <c r="K28" s="6" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L28" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="M28" s="6" t="inlineStr">
         <is>
           <t>GLOSSARY に以下を追加:
 (1) '削除候補（deleted サミット）' を独立項目として追加（ISSUE-018 の sota_summit.match_status=deleted 定義と整合）
 (2) ISSUE-026 と協調して 'dominant peak' 見出しを英語表記に統一</t>
         </is>
       </c>
-      <c r="M28" s="4" t="inlineStr"/>
-      <c r="N28" s="4" t="inlineStr"/>
-      <c r="O28" s="4" t="inlineStr"/>
+      <c r="N28" s="6" t="inlineStr"/>
+      <c r="O28" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="P28" s="6" t="inlineStr"/>
     </row>
     <row r="29" ht="40" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
@@ -2701,7 +2795,7 @@
           <t>改善</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>低</t>
         </is>
@@ -2722,33 +2816,42 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J29" s="7" t="inlineStr">
-        <is>
-          <t>未対応</t>
-        </is>
-      </c>
-      <c r="K29" s="7" t="inlineStr"/>
+      <c r="J29" s="7" t="inlineStr"/>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
       <c r="L29" s="7" t="inlineStr">
         <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="inlineStr">
+        <is>
           <t>フォールバック規定を 1 箇所（推奨: FR-017 のみ）に集約し、他箇所からは '詳細は FR-017 参照' とリンクする。</t>
         </is>
       </c>
-      <c r="M29" s="7" t="inlineStr"/>
       <c r="N29" s="7" t="inlineStr"/>
-      <c r="O29" s="7" t="inlineStr"/>
+      <c r="O29" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="P29" s="7" t="inlineStr"/>
     </row>
     <row r="30" ht="40" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>ISSUE-029</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>UR-008 / UR-009 の要件性検討（NFR への再マップ）</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>URD/SRS レビュー指摘 U-1。
 UR-008: 'ドキュメントに従って環境構築から成果物生成まで実行できること'
@@ -2756,39 +2859,44 @@
 両者ともユーザーニーズというよりプロセス品質目標。トレース対象として残すなら扱いを確定したい。現状 NFR-003 / NFR-007 が部分的に対応しているが対応関係が暗黙的。</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>設計</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>その他</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr"/>
-      <c r="H30" s="4" t="inlineStr">
+      <c r="G30" s="6" t="inlineStr"/>
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr">
+      <c r="I30" s="6" t="inlineStr">
         <is>
           <t>URD</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr">
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="K30" s="6" t="inlineStr">
         <is>
           <t>未対応</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr"/>
-      <c r="L30" s="4" t="inlineStr">
+      <c r="L30" s="6" t="inlineStr"/>
+      <c r="M30" s="6" t="inlineStr">
         <is>
           <t>以下のいずれかに整理:
 案A: UR-008 / UR-009 を URD に残しつつ '(品質要件)' と明示し、SRS で NFR-XXX に明示マップ
@@ -2796,7 +2904,7 @@
 案C: URD に残し、トレース確認のための専用節を新設</t>
         </is>
       </c>
-      <c r="M30" s="4" t="inlineStr">
+      <c r="N30" s="6" t="inlineStr">
         <is>
           <t>【Opus相談推奨】URD/SRS構造に関わる設計哲学的判断。後から変更すると影響範囲が大きい。
 相談ポイント:
@@ -2807,8 +2915,8 @@
 (5) ISSUE-031（UR↔FR/NFRトレース調査）・ISSUE-032（RTM作成）の進め方への影響</t>
         </is>
       </c>
-      <c r="N30" s="4" t="inlineStr"/>
-      <c r="O30" s="4" t="inlineStr"/>
+      <c r="O30" s="6" t="inlineStr"/>
+      <c r="P30" s="6" t="inlineStr"/>
     </row>
     <row r="31" ht="40" customHeight="1">
       <c r="A31" s="7" t="inlineStr">
@@ -2831,7 +2939,7 @@
           <t>改善</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>低</t>
         </is>
@@ -2852,40 +2960,49 @@
           <t>URD</t>
         </is>
       </c>
-      <c r="J31" s="7" t="inlineStr">
-        <is>
-          <t>未対応</t>
-        </is>
-      </c>
-      <c r="K31" s="7" t="inlineStr"/>
+      <c r="J31" s="7" t="inlineStr"/>
+      <c r="K31" s="7" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
       <c r="L31" s="7" t="inlineStr">
         <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="M31" s="7" t="inlineStr">
+        <is>
           <t>URD UR-006 の要件文または前提・制約に '作業用ビューア（山岳名入力・XLSX エクスポート）と公開用 HTML（閲覧専用）の 2 層構造' を反映する。</t>
         </is>
       </c>
-      <c r="M31" s="7" t="inlineStr"/>
       <c r="N31" s="7" t="inlineStr"/>
-      <c r="O31" s="7" t="inlineStr"/>
+      <c r="O31" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="P31" s="7" t="inlineStr"/>
     </row>
     <row r="32" ht="40" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>ISSUE-031</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>SRS: 各 UR に対する FR/NFR の対応漏れ調査と『対応 UR』記述の補完</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>ユーザー指摘: 各 FR / NFR の '対応 UR' が記載されているが漏れがある感触あり。本 issue で逆方向（各 UR ← 対応 FR/NFR）をトレースし、漏れている箇所を補完する。
 依存: ISSUE-018〜ISSUE-030 の改訂結果（特に H-1〜H-3 や U-1 によって UR ↔ FR の対応関係が変わる可能性）。
 このため第4段（URD 改訂後）に着手するのが効率的。</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>調査</t>
         </is>
@@ -2895,38 +3012,43 @@
           <t>高</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>その他</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr"/>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr"/>
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="I32" s="6" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr">
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="inlineStr">
         <is>
           <t>未対応</t>
         </is>
       </c>
-      <c r="K32" s="4" t="inlineStr"/>
-      <c r="L32" s="4" t="inlineStr">
+      <c r="L32" s="6" t="inlineStr"/>
+      <c r="M32" s="6" t="inlineStr">
         <is>
           <t>(1) UR-001 〜 UR-010 を縦軸、現状の対応 FR/NFR を横軸に整理した一覧表を作成し漏れを抽出
 (2) 漏れている対応関係を該当 FR / NFR の '対応 UR' フィールドに追記
 (3) ISSUE-031（RTM）作成の前提データとして提供</t>
         </is>
       </c>
-      <c r="M32" s="4" t="inlineStr"/>
-      <c r="N32" s="4" t="inlineStr"/>
-      <c r="O32" s="4" t="inlineStr"/>
+      <c r="N32" s="6" t="inlineStr"/>
+      <c r="O32" s="6" t="inlineStr"/>
+      <c r="P32" s="6" t="inlineStr"/>
     </row>
     <row r="33" ht="40" customHeight="1">
       <c r="A33" s="7" t="inlineStr">
@@ -2979,11 +3101,16 @@
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
           <t>未対応</t>
         </is>
       </c>
-      <c r="K33" s="7" t="inlineStr"/>
-      <c r="L33" s="7" t="inlineStr">
+      <c r="L33" s="7" t="inlineStr"/>
+      <c r="M33" s="7" t="inlineStr">
         <is>
           <t>SRS に '10. 要求トレーサビリティ・マトリックス' を新章として追加。
 - FR セクションと NFR セクションを 2 つの表に分割するか、1 つにまとめるかは可読性で判断
@@ -2991,9 +3118,9 @@
 - ISSUE-031 の調査結果を反映</t>
         </is>
       </c>
-      <c r="M33" s="7" t="inlineStr"/>
       <c r="N33" s="7" t="inlineStr"/>
       <c r="O33" s="7" t="inlineStr"/>
+      <c r="P33" s="7" t="inlineStr"/>
     </row>
     <row r="34" ht="40" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -3040,13 +3167,14 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr"/>
-      <c r="L34" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>(1) L291 の括弧書き「（いずれも FR-014 で後処理される）」を削除またはフェーズ2 完了済み前提の表現に修正
 (2) L294 を削除または FR-009 入力として使う旨に修正
@@ -3054,7 +3182,7 @@
 (4) フェーズ2 内の FR-016 → FR-014 → FR-007 の処理順序が SRS から読み取れるかも合わせて確認</t>
         </is>
       </c>
-      <c r="M34" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr">
         <is>
           <t>当初方針（フェーズ2 配置前提の参照記述整合化）から大幅に範囲拡大。
 FR-014 をフェーズ3.5（新設）に移し、縮小版パイプラインのループ構造
@@ -3065,12 +3193,12 @@
 関連 commit: 8f273a8（暫定・却下）→ 282f427（確定）</t>
         </is>
       </c>
-      <c r="N34" s="2" t="inlineStr">
+      <c r="O34" s="2" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="O34" s="2" t="inlineStr">
+      <c r="P34" s="2" t="inlineStr">
         <is>
           <t>2026-05-19</t>
         </is>
@@ -3097,7 +3225,7 @@
           <t>改善</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="E35" s="5" t="inlineStr">
         <is>
           <t>低</t>
         </is>
@@ -3114,65 +3242,90 @@
         </is>
       </c>
       <c r="I35" s="7" t="inlineStr"/>
-      <c r="J35" s="7" t="inlineStr">
-        <is>
-          <t>未対応</t>
-        </is>
-      </c>
-      <c r="K35" s="7" t="inlineStr"/>
+      <c r="J35" s="7" t="inlineStr"/>
+      <c r="K35" s="7" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
       <c r="L35" s="7" t="inlineStr">
         <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="M35" s="7" t="inlineStr">
+        <is>
           <t>tracker のレコード編集機能で ISSUE-018 の resolution フィールドを書き換え、「案 B（peak.match_status は変更せず、summit.dominant_peak_code で紐付けのみ）を採用」と明記する。</t>
         </is>
       </c>
-      <c r="M35" s="7" t="inlineStr"/>
       <c r="N35" s="7" t="inlineStr"/>
-      <c r="O35" s="7" t="inlineStr"/>
+      <c r="O35" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="P35" s="7" t="inlineStr"/>
     </row>
     <row r="36" ht="40" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>ISSUE-035</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>SRS: 竹島除外方針の記述追加・ADR-009 リンク</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>URD UR-001・ADR-009 に竹島除外方針を追加済み。SRS の前提・制約・スコープ外・FR-003 関連箇所に竹島の記述を追加し、ADR-009 へのリンクを貼る。北方領土の記述（ADR-005 参照）に準じた形で記載すること。</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr"/>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="D36" s="6" t="inlineStr"/>
+      <c r="E36" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr"/>
-      <c r="G36" s="4" t="inlineStr"/>
-      <c r="H36" s="4" t="inlineStr">
+      <c r="F36" s="6" t="inlineStr"/>
+      <c r="G36" s="6" t="inlineStr"/>
+      <c r="H36" s="6" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="I36" s="4" t="inlineStr">
+      <c r="I36" s="6" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="J36" s="4" t="inlineStr">
-        <is>
-          <t>未対応</t>
-        </is>
-      </c>
-      <c r="K36" s="4" t="inlineStr"/>
-      <c r="L36" s="4" t="inlineStr"/>
-      <c r="M36" s="4" t="inlineStr"/>
-      <c r="N36" s="4" t="inlineStr"/>
-      <c r="O36" s="4" t="inlineStr"/>
+      <c r="J36" s="6" t="inlineStr"/>
+      <c r="K36" s="6" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="M36" s="6" t="inlineStr">
+        <is>
+          <t>北方領土の記述（ADR-005 参照）に準じて以下3箇所に竹島の記述を追加する:
+(1) 8.前提・制約（877行目）: 北方領土の記述の直後に「竹島（島根県）が含まれるメッシュ 5531 は mesh_list_japan.txt から除外済み（ADR-009 参照）」を追加
+(2) 9.スコープ外（892行目）: 北方領土の行の直後に「竹島に所在するピーク（韓国 SOTA サミット HL/GB-430 として登録済み。SOTA 日本支部の管轄外のため。除外方法は ADR-009 で規定）」を追加
+(3) FR-003（202行目付近）: 北方領土タイル除外の記述の後に「竹島はメッシュ除外（ADR-009）で対応するため FR-003 での追加処理はない」旨を注記</t>
+        </is>
+      </c>
+      <c r="N36" s="6" t="inlineStr"/>
+      <c r="O36" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="P36" s="6" t="inlineStr"/>
     </row>
     <row r="37" ht="40" customHeight="1">
       <c r="A37" s="7" t="inlineStr">
@@ -3191,7 +3344,7 @@
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr"/>
-      <c r="E37" s="5" t="inlineStr">
+      <c r="E37" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -3208,33 +3361,42 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J37" s="7" t="inlineStr">
-        <is>
-          <t>未対応</t>
-        </is>
-      </c>
+      <c r="J37" s="7" t="inlineStr"/>
       <c r="K37" s="7" t="inlineStr">
         <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L37" s="7" t="inlineStr">
+        <is>
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="L37" s="7" t="inlineStr"/>
-      <c r="M37" s="7" t="inlineStr"/>
+      <c r="M37" s="7" t="inlineStr">
+        <is>
+          <t>5531 を削除ではなくコメントアウト形式（# 5531 竹島のみのため除外（ADR-009））で除外。理由と根拠が履歴として残る。main.c は # 始まり行をスキップ済みのため動作上の変更なし。</t>
+        </is>
+      </c>
       <c r="N37" s="7" t="inlineStr"/>
-      <c r="O37" s="7" t="inlineStr"/>
+      <c r="O37" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="P37" s="7" t="inlineStr"/>
     </row>
     <row r="38" ht="40" customHeight="1">
-      <c r="A38" s="4" t="inlineStr">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>ISSUE-037</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>ADR-010 Phase 1: ビルド基盤 + elevation.c の C++/OpenCV 化（標高値同値性検証含む）</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C38" s="6" t="inlineStr">
         <is>
           <t>ADR-010（C++/OpenCV 全面移行）の Phase 1 として、ビルド基盤の C++ 化と elevation.c の C++ + cv::imread 化を行う。
 【作業範囲】
@@ -3253,7 +3415,7 @@
 - 検討資料 docs/decisions/research/cpp-opencv-migration-research.md（§3 同値性検証手順、§6 ビルド基盤変更）</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>改善</t>
         </is>
@@ -3263,40 +3425,45 @@
           <t>高</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>解析エンジン</t>
         </is>
       </c>
-      <c r="G38" s="4" t="inlineStr">
+      <c r="G38" s="6" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="H38" s="4" t="inlineStr">
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="I38" s="4" t="inlineStr">
+      <c r="I38" s="6" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="J38" s="4" t="inlineStr">
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>LLD</t>
+        </is>
+      </c>
+      <c r="K38" s="6" t="inlineStr">
         <is>
           <t>未対応</t>
         </is>
       </c>
-      <c r="K38" s="4" t="inlineStr">
+      <c r="L38" s="6" t="inlineStr">
         <is>
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="L38" s="4" t="inlineStr"/>
-      <c r="M38" s="4" t="inlineStr"/>
-      <c r="N38" s="4" t="inlineStr"/>
-      <c r="O38" s="4" t="inlineStr"/>
+      <c r="M38" s="6" t="inlineStr"/>
+      <c r="N38" s="6" t="inlineStr"/>
+      <c r="O38" s="6" t="inlineStr"/>
+      <c r="P38" s="6" t="inlineStr"/>
     </row>
     <row r="39" ht="40" customHeight="1">
       <c r="A39" s="7" t="inlineStr">
@@ -3366,31 +3533,36 @@
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
+          <t>LLD</t>
+        </is>
+      </c>
+      <c r="K39" s="7" t="inlineStr">
+        <is>
           <t>未対応</t>
         </is>
       </c>
-      <c r="K39" s="7" t="inlineStr">
+      <c r="L39" s="7" t="inlineStr">
         <is>
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="L39" s="7" t="inlineStr"/>
       <c r="M39" s="7" t="inlineStr"/>
       <c r="N39" s="7" t="inlineStr"/>
       <c r="O39" s="7" t="inlineStr"/>
+      <c r="P39" s="7" t="inlineStr"/>
     </row>
     <row r="40" ht="40" customHeight="1">
-      <c r="A40" s="4" t="inlineStr">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>ISSUE-039</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>ADR-010 Phase 3: FR-015 標高地形図出力の OpenCV 化</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>ADR-010 Phase 3: FR-015（標高地形図 PNG 出力）の実装を OpenCV ベースに書き直す。
 【作業範囲】
@@ -3407,50 +3579,55 @@
 - SRS 6.7 標高地形図（Terrain-RGB PNG）</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>改善</t>
         </is>
       </c>
-      <c r="E40" s="5" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>解析エンジン</t>
         </is>
       </c>
-      <c r="G40" s="4" t="inlineStr">
+      <c r="G40" s="6" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="H40" s="4" t="inlineStr">
+      <c r="H40" s="6" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="I40" s="4" t="inlineStr">
+      <c r="I40" s="6" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="J40" s="4" t="inlineStr">
+      <c r="J40" s="6" t="inlineStr">
+        <is>
+          <t>LLD</t>
+        </is>
+      </c>
+      <c r="K40" s="6" t="inlineStr">
         <is>
           <t>未対応</t>
         </is>
       </c>
-      <c r="K40" s="4" t="inlineStr">
+      <c r="L40" s="6" t="inlineStr">
         <is>
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="L40" s="4" t="inlineStr"/>
-      <c r="M40" s="4" t="inlineStr"/>
-      <c r="N40" s="4" t="inlineStr"/>
-      <c r="O40" s="4" t="inlineStr"/>
+      <c r="M40" s="6" t="inlineStr"/>
+      <c r="N40" s="6" t="inlineStr"/>
+      <c r="O40" s="6" t="inlineStr"/>
+      <c r="P40" s="6" t="inlineStr"/>
     </row>
     <row r="41" ht="40" customHeight="1">
       <c r="A41" s="7" t="inlineStr">
@@ -3500,16 +3677,21 @@
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
+          <t>LLD</t>
+        </is>
+      </c>
+      <c r="K41" s="7" t="inlineStr">
+        <is>
           <t>未対応</t>
         </is>
       </c>
-      <c r="K41" s="7" t="inlineStr">
+      <c r="L41" s="7" t="inlineStr">
         <is>
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="L41" s="7" t="inlineStr"/>
-      <c r="M41" s="7" t="inlineStr">
+      <c r="M41" s="7" t="inlineStr"/>
+      <c r="N41" s="7" t="inlineStr">
         <is>
           <t>【ADR-011 適用 2026-05-21】仕様を delete判定ゾーン方式に更新。
 【作業範囲】
@@ -3549,21 +3731,21 @@
 (7) GeoJSON シリアライズ時の座標精度（小数点何桁）と、形状再現性への影響</t>
         </is>
       </c>
-      <c r="N41" s="7" t="inlineStr"/>
       <c r="O41" s="7" t="inlineStr"/>
+      <c r="P41" s="7" t="inlineStr"/>
     </row>
     <row r="42" ht="40" customHeight="1">
-      <c r="A42" s="4" t="inlineStr">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>ISSUE-041</t>
         </is>
       </c>
-      <c r="B42" s="4" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>実装側のフラグ命名追従（is_tile_top → key_col_resolved + 真偽値反転）</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>ISSUE-014 関連の仕様変更（commit 633e54b / ea6bbbe）で、SRS/ADR/GLOSSARY のフラグ名と真偽値方向を以下に統一した。実装側はまだ旧名のままなので、仕様と整合させる追従が必要。
 【リネーム + 真偽値反転】
@@ -3590,44 +3772,49 @@
 - output_geojson.py 実行 → GeoJSON プロパティが新名で出力されること</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>改善</t>
         </is>
       </c>
-      <c r="E42" s="5" t="inlineStr">
+      <c r="E42" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F42" s="4" t="inlineStr">
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <t>その他</t>
         </is>
       </c>
-      <c r="G42" s="4" t="inlineStr"/>
-      <c r="H42" s="4" t="inlineStr">
+      <c r="G42" s="6" t="inlineStr"/>
+      <c r="H42" s="6" t="inlineStr">
         <is>
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="I42" s="4" t="inlineStr">
+      <c r="I42" s="6" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="J42" s="4" t="inlineStr">
+      <c r="J42" s="6" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="K42" s="6" t="inlineStr">
         <is>
           <t>未対応</t>
         </is>
       </c>
-      <c r="K42" s="4" t="inlineStr">
+      <c r="L42" s="6" t="inlineStr">
         <is>
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="L42" s="4" t="inlineStr"/>
-      <c r="M42" s="4" t="inlineStr">
+      <c r="M42" s="6" t="inlineStr"/>
+      <c r="N42" s="6" t="inlineStr">
         <is>
           <t>【背景】commit 633e54b (is_tile_top → key_col_unresolved) + commit ea6bbbe (key_col_unresolved → key_col_resolved + area_truncated → area_complete) で仕様側を更新済み。実装側はまだ旧名のまま。仕様優先原則のため仕様変更が先行している。
 【関連 ISSUE】
@@ -3637,8 +3824,8 @@
 - ISSUE-040 (ADR-010 Phase 4): FR-016 (area_complete を含む) C++ 新規実装</t>
         </is>
       </c>
-      <c r="N42" s="4" t="inlineStr"/>
-      <c r="O42" s="4" t="inlineStr"/>
+      <c r="O42" s="6" t="inlineStr"/>
+      <c r="P42" s="6" t="inlineStr"/>
     </row>
     <row r="43" ht="40" customHeight="1">
       <c r="A43" s="7" t="inlineStr">
@@ -3667,7 +3854,7 @@
           <t>改善</t>
         </is>
       </c>
-      <c r="E43" s="5" t="inlineStr">
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -3694,36 +3881,41 @@
       </c>
       <c r="J43" s="7" t="inlineStr">
         <is>
+          <t>HLD</t>
+        </is>
+      </c>
+      <c r="K43" s="7" t="inlineStr">
+        <is>
           <t>未対応</t>
         </is>
       </c>
-      <c r="K43" s="7" t="inlineStr"/>
       <c r="L43" s="7" t="inlineStr"/>
-      <c r="M43" s="7" t="inlineStr">
+      <c r="M43" s="7" t="inlineStr"/>
+      <c r="N43" s="7" t="inlineStr">
         <is>
           <t>ISSUE-019 のクローズ時にユーザーから登録要望が出た案件。</t>
         </is>
       </c>
-      <c r="N43" s="7" t="inlineStr"/>
       <c r="O43" s="7" t="inlineStr"/>
+      <c r="P43" s="7" t="inlineStr"/>
     </row>
     <row r="44" ht="40" customHeight="1">
-      <c r="A44" s="4" t="inlineStr">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>ISSUE-043</t>
         </is>
       </c>
-      <c r="B44" s="4" t="inlineStr">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>merge.py: delete判定ゾーン対応（AZ/delete-zone PIP、不備フラグ列、exit code、dominant 改名）</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C44" s="6" t="inlineStr">
         <is>
           <t>ADR-011（delete判定ゾーンポリゴン）採用に伴う merge.py の改修。SRS FR-009 / ADR-007 / ADR-008 / ADR-011 の仕様を実装に反映する。</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>改善</t>
         </is>
@@ -3733,41 +3925,46 @@
           <t>高</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr">
+      <c r="F44" s="6" t="inlineStr">
         <is>
           <t>merge.py</t>
         </is>
       </c>
-      <c r="G44" s="4" t="inlineStr">
+      <c r="G44" s="6" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="H44" s="4" t="inlineStr">
+      <c r="H44" s="6" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="I44" s="4" t="inlineStr">
+      <c r="I44" s="6" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="J44" s="4" t="inlineStr">
+      <c r="J44" s="6" t="inlineStr">
+        <is>
+          <t>LLD</t>
+        </is>
+      </c>
+      <c r="K44" s="6" t="inlineStr">
         <is>
           <t>未対応</t>
         </is>
       </c>
-      <c r="K44" s="4" t="inlineStr"/>
-      <c r="L44" s="4" t="inlineStr"/>
-      <c r="M44" s="4" t="inlineStr">
+      <c r="L44" s="6" t="inlineStr"/>
+      <c r="M44" s="6" t="inlineStr"/>
+      <c r="N44" s="6" t="inlineStr">
         <is>
           <t>【2026-05-22 追記】merge.py 改修スコープに以下を追加: points/sota_points/is_band_change_candidate 列の計算・追加（FR-009 変更申請判定セクション参照）。バンド定義は GLOSSARY 標高バンド（Points 算出表）に従う。peak_elev は切り捨て（floor）した整数 m でバンド判定（例: 1499.5m → 1499m → 8pt）、sota_alt_m はそのまま判定。
 【2026-05-23 補正】merge.py の出力は merged.csv（ピーク台帳・ステータス・不備フラグ）と merged_activation.geojson（AZ・delete判定ゾーンポリゴンの per-mesh 統合）の2系統（SRS FR-018 参照）。AZ/delete-zone PIP 判定の素材は per-mesh activation GeoJSON。不備フラグ・exit code 判定は merged.csv 側で完結する。</t>
         </is>
       </c>
-      <c r="N44" s="4" t="inlineStr"/>
-      <c r="O44" s="4" t="inlineStr"/>
+      <c r="O44" s="6" t="inlineStr"/>
+      <c r="P44" s="6" t="inlineStr"/>
     </row>
     <row r="45" ht="40" customHeight="1">
       <c r="A45" s="7" t="inlineStr">
@@ -3817,74 +4014,84 @@
       </c>
       <c r="J45" s="7" t="inlineStr">
         <is>
+          <t>LLD</t>
+        </is>
+      </c>
+      <c r="K45" s="7" t="inlineStr">
+        <is>
           <t>未対応</t>
         </is>
       </c>
-      <c r="K45" s="7" t="inlineStr"/>
       <c r="L45" s="7" t="inlineStr"/>
-      <c r="M45" s="7" t="inlineStr">
+      <c r="M45" s="7" t="inlineStr"/>
+      <c r="N45" s="7" t="inlineStr">
         <is>
           <t>【2026-05-22 追記】output_geojson.py + merged_viewer.html 改修スコープに以下を追加: (1) 名称修正 UI 廃止（matched ピークの入力フィールドを削除）。(2) 変更行自動エクスポート（is_band_change_candidate=true の matched ピークを申請書の変更行として自動生成、FR-011 ※5フォーマット準拠）。
 【2026-05-23 補正】output_geojson.py の入力は merged.csv + merged_activation.geojson の2系統（SRS FR-013 参照）。ポリゴン情報（AZ・delete判定ゾーン）は merged_activation.geojson から取り込む。出力は merged.geojson（Point + LineString + Polygon の可視化集約）と merged_viewer.html。</t>
         </is>
       </c>
-      <c r="N45" s="7" t="inlineStr"/>
       <c r="O45" s="7" t="inlineStr"/>
+      <c r="P45" s="7" t="inlineStr"/>
     </row>
     <row r="46" ht="40" customHeight="1">
-      <c r="A46" s="4" t="inlineStr">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>ISSUE-045</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>params/config.ini.example: delete_zone_max_drop = 250 パラメータ追加</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>ADR-011 で確定した delete_zone_max_drop（実測値 250m）を config.ini.example に記載し、ユーザー環境への展開を可能にする。</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>改善</t>
         </is>
       </c>
-      <c r="E46" s="5" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr">
+      <c r="F46" s="6" t="inlineStr">
         <is>
           <t>設定</t>
         </is>
       </c>
-      <c r="G46" s="4" t="inlineStr">
+      <c r="G46" s="6" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="H46" s="4" t="inlineStr">
+      <c r="H46" s="6" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="I46" s="4" t="inlineStr">
+      <c r="I46" s="6" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="J46" s="4" t="inlineStr">
+      <c r="J46" s="6" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="K46" s="6" t="inlineStr">
         <is>
           <t>未対応</t>
         </is>
       </c>
-      <c r="K46" s="4" t="inlineStr"/>
-      <c r="L46" s="4" t="inlineStr"/>
-      <c r="M46" s="4" t="inlineStr">
+      <c r="L46" s="6" t="inlineStr"/>
+      <c r="M46" s="6" t="inlineStr"/>
+      <c r="N46" s="6" t="inlineStr">
         <is>
           <t>【作業範囲】
 - params/config.ini.example の [analysis] セクション（または相当箇所）に delete_zone_max_drop = 250 を追加
@@ -3896,8 +4103,8 @@
 【元 ISSUE】ISSUE-020 から分離</t>
         </is>
       </c>
-      <c r="N46" s="4" t="inlineStr"/>
-      <c r="O46" s="4" t="inlineStr"/>
+      <c r="O46" s="6" t="inlineStr"/>
+      <c r="P46" s="6" t="inlineStr"/>
     </row>
     <row r="47" ht="40" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
@@ -3945,20 +4152,21 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J47" s="2" t="inlineStr">
+      <c r="J47" s="2" t="inlineStr"/>
+      <c r="K47" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K47" s="2" t="inlineStr"/>
       <c r="L47" s="2" t="inlineStr"/>
       <c r="M47" s="2" t="inlineStr"/>
-      <c r="N47" s="2" t="inlineStr">
+      <c r="N47" s="2" t="inlineStr"/>
+      <c r="O47" s="2" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="O47" s="2" t="inlineStr">
+      <c r="P47" s="2" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
@@ -3985,7 +4193,7 @@
           <t>改善</t>
         </is>
       </c>
-      <c r="E48" s="5" t="inlineStr">
+      <c r="E48" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -4006,24 +4214,25 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="J48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K48" s="2" t="inlineStr"/>
-      <c r="L48" s="2" t="inlineStr">
+      <c r="L48" s="2" t="inlineStr"/>
+      <c r="M48" s="2" t="inlineStr">
         <is>
           <t>drawio で FR-002/FR-003 のボックスを FR-001 の外に移動し、SVG を再エクスポートして docs/figures/ を更新する</t>
         </is>
       </c>
-      <c r="M48" s="2" t="inlineStr"/>
-      <c r="N48" s="2" t="inlineStr">
+      <c r="N48" s="2" t="inlineStr"/>
+      <c r="O48" s="2" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="O48" s="2" t="inlineStr">
+      <c r="P48" s="2" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
@@ -4050,7 +4259,7 @@
           <t>機能追加</t>
         </is>
       </c>
-      <c r="E49" s="5" t="inlineStr">
+      <c r="E49" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
@@ -4071,24 +4280,25 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J49" s="2" t="inlineStr">
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K49" s="2" t="inlineStr"/>
-      <c r="L49" s="2" t="inlineStr">
+      <c r="L49" s="2" t="inlineStr"/>
+      <c r="M49" s="2" t="inlineStr">
         <is>
           <t>drawio でコンテキスト図を作成し、docs/figures/context.drawio.svg として保存。SRS 3.1 のプレースホルダーを図参照に置き換えてコミット</t>
         </is>
       </c>
-      <c r="M49" s="2" t="inlineStr"/>
-      <c r="N49" s="2" t="inlineStr">
+      <c r="N49" s="2" t="inlineStr"/>
+      <c r="O49" s="2" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="O49" s="2" t="inlineStr">
+      <c r="P49" s="2" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
@@ -4115,7 +4325,7 @@
           <t>機能追加</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="E50" s="5" t="inlineStr">
         <is>
           <t>低</t>
         </is>
@@ -4136,24 +4346,25 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J50" s="2" t="inlineStr">
+      <c r="J50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K50" s="2" t="inlineStr"/>
-      <c r="L50" s="2" t="inlineStr">
+      <c r="L50" s="2" t="inlineStr"/>
+      <c r="M50" s="2" t="inlineStr">
         <is>
           <t>drawio でフェーズ俯瞰図を作成し、docs/figures/phases_overview.drawio.svg として保存。SRS 3.3 のプレースホルダーを図参照に置き換えてコミット</t>
         </is>
       </c>
-      <c r="M50" s="2" t="inlineStr"/>
-      <c r="N50" s="2" t="inlineStr">
+      <c r="N50" s="2" t="inlineStr"/>
+      <c r="O50" s="2" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="O50" s="2" t="inlineStr">
+      <c r="P50" s="2" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
@@ -4180,7 +4391,7 @@
           <t>機能追加</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr">
+      <c r="E51" s="5" t="inlineStr">
         <is>
           <t>低</t>
         </is>
@@ -4205,40 +4416,41 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J51" s="2" t="inlineStr">
+      <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr">
         <is>
           <t>解決済</t>
         </is>
       </c>
-      <c r="K51" s="2" t="inlineStr">
+      <c r="L51" s="2" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="L51" s="2" t="inlineStr">
+      <c r="M51" s="2" t="inlineStr">
         <is>
           <t>drawio で各フェーズの機能関連図を作成し、docs/figures/phase2.drawio.svg 等として保存。SRS の各フェーズ節冒頭に図参照を追加してコミット</t>
         </is>
       </c>
-      <c r="M51" s="2" t="inlineStr">
+      <c r="N51" s="2" t="inlineStr">
         <is>
           <t>【本日の決定事項】フェーズ別機能関連図（phase2〜4）の個別作成は中止し、phases_overview.drawio.svg（フェーズ俯瞰図）で代替する方針を確定。フェーズ1の機能関連図（phase1.drawio.svg）もSRSの参照削除済み（commit 12e2a45）のうえファイル削除。俯瞰図はフェーズ3出力ラベルをmerged_activation.geojsonに修正（SRS FR-018と整合）し、誤字「見つらない→見つからない」も修正してcommit ca09554でコミット済み。</t>
         </is>
       </c>
-      <c r="N51" s="2" t="inlineStr">
+      <c r="O51" s="2" t="inlineStr">
         <is>
           <t>2026-05-23</t>
         </is>
       </c>
-      <c r="O51" s="2" t="inlineStr">
+      <c r="P51" s="2" t="inlineStr">
         <is>
           <t>2026-05-23</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
-    <dataValidation sqref="J2:J51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="5">
+    <dataValidation sqref="K2:K51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -4248,6 +4460,9 @@
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4261,7 +4476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4293,7 +4508,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -4333,7 +4548,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -4353,7 +4568,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -4373,7 +4588,7 @@
         </is>
       </c>
       <c r="B12" s="11" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -4391,7 +4606,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
@@ -4401,7 +4616,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
@@ -4429,7 +4644,7 @@
         </is>
       </c>
       <c r="B20" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
@@ -4449,7 +4664,7 @@
         </is>
       </c>
       <c r="B22" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -4477,7 +4692,7 @@
         </is>
       </c>
       <c r="B26" s="11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27">
@@ -4517,7 +4732,7 @@
         </is>
       </c>
       <c r="B30" s="11" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="32">
@@ -4565,17 +4780,7 @@
         </is>
       </c>
       <c r="B36" s="11" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="B37" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -5046,10 +5251,10 @@
         <v>50</v>
       </c>
       <c r="C28" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="D28" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(URD/SRS/CLAUDE.md): ISSUE-029 UR-009 を開発プロセス目標として CLAUDE.md に移動
UR-009「仕様書・設計書と実装の整合性」はユーザー要件ではなく開発プロセス品質目標であるため、
URD から削除して CLAUDE.md「ドキュメント・実装整合性原則」セクションに移動した。

- UR-008 は URD に残置（NFR-006 マップ維持）
- NFR-003 の対応 UR を UR-009 → UR-004/005 に振り替え（申請書・エビデンスの信頼性）
- NFR-007 の対応 UR を UR-009 → UR-008 に振り替え（実行可能性のログ担保）
- ISSUE-031 の備考に UR-009 削除・NFR 振り替え済みを記録

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -279,12 +279,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$28</f>
+              <f>'収束グラフ'!$A$2:$A$29</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$B$2:$B$28</f>
+              <f>'収束グラフ'!$B$2:$B$29</f>
             </numRef>
           </val>
         </ser>
@@ -314,12 +314,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$28</f>
+              <f>'収束グラフ'!$A$2:$A$29</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$C$2:$C$28</f>
+              <f>'収束グラフ'!$C$2:$C$29</f>
             </numRef>
           </val>
         </ser>
@@ -349,12 +349,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$28</f>
+              <f>'収束グラフ'!$A$2:$A$29</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$D$2:$D$28</f>
+              <f>'収束グラフ'!$D$2:$D$29</f>
             </numRef>
           </val>
         </ser>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr"/>
@@ -2935,7 +2935,11 @@
 (5) ISSUE-031（UR↔FR/NFRトレース調査）・ISSUE-032（RTM作成）の進め方への影響</t>
         </is>
       </c>
-      <c r="O30" s="6" t="inlineStr"/>
+      <c r="O30" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
       <c r="P30" s="6" t="inlineStr"/>
     </row>
     <row r="31" ht="40" customHeight="1">
@@ -3070,7 +3074,11 @@
 (3) ISSUE-031（RTM）作成の前提データとして提供</t>
         </is>
       </c>
-      <c r="N32" s="6" t="inlineStr"/>
+      <c r="N32" s="6" t="inlineStr">
+        <is>
+          <t>UR-009 削除・NFR-003 対応 UR を UR-004/005 に・NFR-007 対応 UR を UR-008 に振り替え済み（ISSUE-029 対応、2026-05-24）</t>
+        </is>
+      </c>
       <c r="O32" s="6" t="inlineStr"/>
       <c r="P32" s="6" t="inlineStr"/>
     </row>
@@ -4746,7 +4754,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -4766,7 +4774,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -4992,7 +5000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5455,6 +5463,22 @@
         <v>34</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>53</v>
+      </c>
+      <c r="C29" t="n">
+        <v>34</v>
+      </c>
+      <c r="D29" t="n">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
chore(tracker): ISSUE-055 登録（SRS HTMLビューアUI要件追加）
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P55"/>
+  <dimension ref="A1:P56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4701,30 +4701,90 @@
       <c r="J55" s="7" t="inlineStr"/>
       <c r="K55" s="7" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="L55" s="7" t="inlineStr"/>
       <c r="M55" s="7" t="inlineStr"/>
       <c r="N55" s="7" t="inlineStr"/>
-      <c r="O55" s="7" t="inlineStr"/>
+      <c r="O55" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
       <c r="P55" s="7" t="inlineStr"/>
+    </row>
+    <row r="56" ht="40" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-055</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>SRS: GeoJSONビューア（HTMLビュー）のUI要件追加</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr"/>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>機能追加</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr"/>
+      <c r="G56" s="6" t="inlineStr"/>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J56" s="6" t="inlineStr"/>
+      <c r="K56" s="6" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L56" s="6" t="inlineStr"/>
+      <c r="M56" s="6" t="inlineStr"/>
+      <c r="N56" s="6" t="inlineStr">
+        <is>
+          <t>HTMLビューアはユーザーI/Fの1つ（外部I/F）であり、SRSに以下を記載する必要がある。
+- match_status別の視覚的区別表示要件
+- key_col_resolved=falseピークの陸地最高峰/島嶼部最高峰特別表示
+- ポップアップ表示項目と編集可否（山岳名は新規のみ入力可など）
+- 変更の根拠フィールドの入力要件・初期値テンプレート（※2/※4/※5）
+- エクスポート機能の存在と出力内容
+実装手段（Leaflet・HTML単体・localStorage等）はHLDに記載する。</t>
+        </is>
+      </c>
+      <c r="O56" s="6" t="inlineStr"/>
+      <c r="P56" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4760,7 +4820,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3">
@@ -4770,7 +4830,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -4791,7 +4851,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>51.9%</t>
+          <t>50.9%</t>
         </is>
       </c>
     </row>
@@ -4830,7 +4890,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -4878,7 +4938,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17">
@@ -4906,7 +4966,7 @@
         </is>
       </c>
       <c r="B20" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
@@ -5022,7 +5082,7 @@
         </is>
       </c>
       <c r="B34" s="11" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35">
@@ -5526,10 +5586,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C29" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D29" t="n">
         <v>34</v>

</xml_diff>

<commit_message>
chore: handover 2026-05-25_1812 + plan.md・xlsx 更新
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -279,12 +279,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$29</f>
+              <f>'収束グラフ'!$A$2:$A$30</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$B$2:$B$29</f>
+              <f>'収束グラフ'!$B$2:$B$30</f>
             </numRef>
           </val>
         </ser>
@@ -314,12 +314,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$29</f>
+              <f>'収束グラフ'!$A$2:$A$30</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$C$2:$C$29</f>
+              <f>'収束グラフ'!$C$2:$C$30</f>
             </numRef>
           </val>
         </ser>
@@ -349,12 +349,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$29</f>
+              <f>'収束グラフ'!$A$2:$A$30</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$D$2:$D$29</f>
+              <f>'収束グラフ'!$D$2:$D$30</f>
             </numRef>
           </val>
         </ser>
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P56"/>
+  <dimension ref="A1:P57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4770,21 +4770,82 @@
       <c r="O56" s="6" t="inlineStr"/>
       <c r="P56" s="6" t="inlineStr"/>
     </row>
+    <row r="57" ht="40" customHeight="1">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-056</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>prefetch_tiles.py: FR-001 仕様追従（全種別独立取得・404時キャッシュ削除）</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>SRS FR-001 改訂（2026-05-25）に合わせて prefetch_tiles.py の実装を修正する。
+【修正内容】
+1. fetch_dem5_with_fallback() の早期 break を撤廃し、dem5a/b/c を独立ジョブとして列挙・取得する（種別間の条件分岐なし）
+2. enumerate_jobs() で dem5b/dem5c も常に列挙対象に含める
+3. fetch_one() で HTTP 404 受信時に同パスのローカルキャッシュが存在すれば os.unlink(path) で削除し、地理院側と同じ状態に保つ
+【背景】
+旧実装は dem5a 取得成功で break する「タイル単位フォールバック取得」になっており、FR-002 のピクセル単位フォールバックが機能するための前提（全種別のタイルがローカルに揃っていること）を満たしていなかった。また 404 受信時にキャッシュを残すと地理院側で削除されたタイルがローカルに残り続ける問題があった。
+【対象ファイル】
+- scripts/prefetch_tiles.py
+  - fetch_dem5_with_fallback() (185-199行付近): early break 撤廃
+  - enumerate_jobs() : dem5b/dem5c を列挙対象に追加
+  - fetch_one() (131-180行付近): 404時の os.unlink 追加</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr"/>
+      <c r="G57" s="7" t="inlineStr"/>
+      <c r="H57" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="I57" s="7" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="J57" s="7" t="inlineStr"/>
+      <c r="K57" s="7" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L57" s="7" t="inlineStr"/>
+      <c r="M57" s="7" t="inlineStr"/>
+      <c r="N57" s="7" t="inlineStr"/>
+      <c r="O57" s="7" t="inlineStr"/>
+      <c r="P57" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4820,7 +4881,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3">
@@ -4830,7 +4891,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -4851,7 +4912,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>50.9%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
@@ -4870,7 +4931,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9">
@@ -4928,7 +4989,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
@@ -4976,7 +5037,7 @@
         </is>
       </c>
       <c r="B21" s="11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22">
@@ -5102,7 +5163,7 @@
         </is>
       </c>
       <c r="B36" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -5116,7 +5177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5595,6 +5656,22 @@
         <v>34</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>56</v>
+      </c>
+      <c r="C30" t="n">
+        <v>35</v>
+      </c>
+      <c r="D30" t="n">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
docs(srs): merged.csv 命名整理（merged_peak.csv / merged_summit.csv 導入）
- FR-008 出力を merged.csv から merged_peak.csv にリネーム
- FR-009 出力に merged_summit.csv（サミット中心の確認用 CSV）を新規追加
  - ピーク中心→サミット中心の概念切り替わり点を FR-009 概要文に明記
- FR-012 出力名を TBD マーカー化（フェーズ5 レビュー後に確定）
- § 3.3 俯瞰図・FR-014・§ 6 成果物一覧の全参照箇所を新命名に追従
- ISSUE-051 タイトルを「SRS フェーズ3（FR-014）:」に修正
- ISSUE-059/060/061 を起票（実装追従・ドキュメント追従・本タスク）

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P59"/>
+  <dimension ref="A1:P62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4498,7 +4498,7 @@
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>SRS フェーズ3.5: area_complete=false トリガー外しの重複記述整理</t>
+          <t>SRS フェーズ3（FR-014）: area_complete=false トリガー外しの重複記述整理</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -4953,21 +4953,199 @@
       </c>
       <c r="P59" s="7" t="inlineStr"/>
     </row>
+    <row r="60" ht="40" customHeight="1">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-059</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>実装側ファイル名追従: merged_peak.csv / merged_summit.csv リネーム</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>SRS 改訂（merged.csv 命名整理）に伴う実装追従。scripts/merge.py:50 の DEFAULT_OUTPUT を merged_peak.csv に変更、scripts/output_geojson.py:34 の DEFAULT_INPUT を merged_peak.csv に変更。FR-009 から merged_summit.csv 出力ロジックを新規追加（カラム構成は FR-012 と同じ）。</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>merge.py</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="inlineStr"/>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="I60" s="6" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="J60" s="6" t="inlineStr"/>
+      <c r="K60" s="6" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L60" s="6" t="inlineStr"/>
+      <c r="M60" s="6" t="inlineStr">
+        <is>
+          <t>merge.py の DEFAULT_OUTPUT 変更 + output_geojson.py の DEFAULT_INPUT 変更 + output_geojson.py に merged_summit.csv 出力処理追加</t>
+        </is>
+      </c>
+      <c r="N60" s="6" t="inlineStr"/>
+      <c r="O60" s="6" t="inlineStr"/>
+      <c r="P60" s="6" t="inlineStr"/>
+    </row>
+    <row r="61" ht="40" customHeight="1">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-060</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>CLAUDE.md / README.md の merged.csv 言及箇所を新命名に更新</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>SRS 改訂（merged.csv 命名整理）に伴うドキュメント追従。CLAUDE.md L63 他 merged.csv を参照しているドキュメント箇所を merged_peak.csv / merged_summit.csv に更新する。</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G61" s="7" t="inlineStr"/>
+      <c r="H61" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="I61" s="7" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="J61" s="7" t="inlineStr"/>
+      <c r="K61" s="7" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L61" s="7" t="inlineStr"/>
+      <c r="M61" s="7" t="inlineStr">
+        <is>
+          <t>CLAUDE.md・README.md 内の merged.csv 参照を検索し新命名に置換</t>
+        </is>
+      </c>
+      <c r="N61" s="7" t="inlineStr"/>
+      <c r="O61" s="7" t="inlineStr"/>
+      <c r="P61" s="7" t="inlineStr"/>
+    </row>
+    <row r="62" ht="40" customHeight="1">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-061</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>SRS merged.csv 命名整理（merged_peak.csv / merged_summit.csv 導入）</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>SRS 内で merged.csv というファイル名が FR-008（内部 work CSV）と FR-012（派生エビデンス CSV）で重複していた問題を解消。FR-008 出力を merged_peak.csv にリネーム、FR-009 出力に merged_summit.csv（サミット一覧 CSV・ピーク→サミット概念切り替わり点の確認用）を新規追加。FR-012 出力名は未定のため TBD マーカー化（フェーズ5 レビュー時に確定）。</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>merge.py</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr"/>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="I62" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J62" s="6" t="inlineStr"/>
+      <c r="K62" s="6" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L62" s="6" t="inlineStr"/>
+      <c r="M62" s="6" t="inlineStr">
+        <is>
+          <t>docs/02_SRS.md を改訂。§3.3 俯瞰図・FR-008/FR-009/FR-014/FR-012 出力欄・§6 成果物一覧をすべて新命名に更新</t>
+        </is>
+      </c>
+      <c r="N62" s="6" t="inlineStr"/>
+      <c r="O62" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="P62" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5003,7 +5181,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3">
@@ -5013,7 +5191,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
@@ -5034,7 +5212,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>48.3%</t>
+          <t>45.9%</t>
         </is>
       </c>
     </row>
@@ -5053,7 +5231,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -5073,7 +5251,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -5111,7 +5289,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16">
@@ -5131,7 +5309,7 @@
         </is>
       </c>
       <c r="B17" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
@@ -5159,7 +5337,7 @@
         </is>
       </c>
       <c r="B21" s="11" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22">
@@ -5207,7 +5385,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28">
@@ -5237,7 +5415,7 @@
         </is>
       </c>
       <c r="B30" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32">
@@ -5265,7 +5443,7 @@
         </is>
       </c>
       <c r="B34" s="11" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="35">
@@ -5285,7 +5463,7 @@
         </is>
       </c>
       <c r="B36" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -5849,10 +6027,10 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C34" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D34" t="n">
         <v>34</v>

</xml_diff>

<commit_message>
docs(srs): FR-009/FR-012 出力を xlsx 化・FR-012 呼称変更
- FR-009 出力: merged_summit.csv → merged_summit.xlsx（サミット一覧（突合後））
- FR-012 出力: TBD マーカー → merged_summit_revised.xlsx（サミット一覧（申請内容反映版））
- 「エビデンス CSV」呼称を全廃し「サミット一覧（申請内容反映版）」に統一
- § 6.5 新規追加（サミット一覧（突合後））・§ 6.5〜6.12 → § 6.6〜6.13 へ番号シフト
- § 6.4 タイトル改名・XLSX フォーマット規定追加（エンコーディング/区切り文字行削除）
- ISSUE-059 タイトル更新・notes 追加、ISSUE-060 notes 追加、ISSUE-062 新規起票

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P62"/>
+  <dimension ref="A1:P63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4961,7 +4961,7 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>実装側ファイル名追従: merged_peak.csv / merged_summit.csv リネーム</t>
+          <t>実装側ファイル名追従: merged_peak.csv / merged_summit.xlsx リネーム</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -5007,7 +5007,11 @@
           <t>merge.py の DEFAULT_OUTPUT 変更 + output_geojson.py の DEFAULT_INPUT 変更 + output_geojson.py に merged_summit.csv 出力処理追加</t>
         </is>
       </c>
-      <c r="N60" s="6" t="inlineStr"/>
+      <c r="N60" s="6" t="inlineStr">
+        <is>
+          <t>SRS 改訂（2026-05-29: xlsx 化）に伴い追加スコープ: merged_summit.csv → merged_summit.xlsx（scripts/merge.py の出力変更）、output_geojson.py の DEFAULT_INPUT を merged_peak.csv に変更。FR-012 実装（merged_summit_revised.xlsx 生成）は ISSUE-062 として分離起票のため本 ISSUE のスコープには含めない。</t>
+        </is>
+      </c>
       <c r="O60" s="6" t="inlineStr"/>
       <c r="P60" s="6" t="inlineStr"/>
     </row>
@@ -5065,7 +5069,11 @@
           <t>CLAUDE.md・README.md 内の merged.csv 参照を検索し新命名に置換</t>
         </is>
       </c>
-      <c r="N61" s="7" t="inlineStr"/>
+      <c r="N61" s="7" t="inlineStr">
+        <is>
+          <t>merged.csv 命名整理に加えて、2026-05-29 の xlsx 化により merged_summit.xlsx の言及も追加対象。CLAUDE.md L63 他を更新。</t>
+        </is>
+      </c>
       <c r="O61" s="7" t="inlineStr"/>
       <c r="P61" s="7" t="inlineStr"/>
     </row>
@@ -5131,21 +5139,75 @@
       </c>
       <c r="P62" s="6" t="inlineStr"/>
     </row>
+    <row r="63" ht="40" customHeight="1">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-062</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>FR-012 実装: merged_summit_revised.xlsx 生成スクリプト新規開発</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>SRS FR-012（サミット一覧（申請内容反映版）生成）の実装。merged.geojson の Point フィーチャから FR-019 でのユーザー編集内容を反映した merged_summit_revised.xlsx を生成するスクリプトを新規開発する。HTML ビューアの「エクスポート」ボタン（FR-019 経由）との連携も必要。</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>機能追加</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>GeoJSON出力</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr"/>
+      <c r="H63" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="I63" s="7" t="inlineStr"/>
+      <c r="J63" s="7" t="inlineStr"/>
+      <c r="K63" s="7" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L63" s="7" t="inlineStr"/>
+      <c r="M63" s="7" t="inlineStr">
+        <is>
+          <t>新規スクリプト scripts/export_summit_revised.py 等を作成し、merged.geojson + HTML ビューア編集内容を入力として merged_summit_revised.xlsx を出力するロジックを実装。FR-013 HTML ビューア改修（エクスポートトリガー連携）も別途必要。</t>
+        </is>
+      </c>
+      <c r="N63" s="7" t="inlineStr"/>
+      <c r="O63" s="7" t="inlineStr"/>
+      <c r="P63" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5181,7 +5243,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3">
@@ -5191,7 +5253,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
@@ -5212,7 +5274,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>45.9%</t>
+          <t>45.2%</t>
         </is>
       </c>
     </row>
@@ -5231,7 +5293,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -5289,7 +5351,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16">
@@ -5327,7 +5389,7 @@
         </is>
       </c>
       <c r="B20" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -5395,7 +5457,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
@@ -6027,7 +6089,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C34" t="n">
         <v>39</v>

</xml_diff>

<commit_message>
chore(tracker): ISSUE-067 対応完了クローズ・xlsx 更新
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P67"/>
+  <dimension ref="A1:P68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5405,21 +5405,71 @@
       <c r="O67" s="7" t="inlineStr"/>
       <c r="P67" s="7" t="inlineStr"/>
     </row>
+    <row r="68" ht="40" customHeight="1">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-067</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>国土地理院タイル出典表示の整備</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr"/>
+      <c r="D68" s="6" t="inlineStr"/>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="inlineStr"/>
+      <c r="G68" s="6" t="inlineStr"/>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J68" s="6" t="inlineStr"/>
+      <c r="K68" s="6" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L68" s="6" t="inlineStr"/>
+      <c r="M68" s="6" t="inlineStr"/>
+      <c r="N68" s="6" t="inlineStr">
+        <is>
+          <t>UR-011 新設（URD）、FR-013/FR-012/FR-021 出典要件追加（SRS）、ADR-014 作成済み。実装対象: README / output_geojson.py / merge.py / viewer_mockup.html XLSX出力。ADR-014 参照: docs/decisions/ADR-014-gsi-tile-attribution-policy.md</t>
+        </is>
+      </c>
+      <c r="O68" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="P68" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5455,7 +5505,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3">
@@ -5465,7 +5515,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4">
@@ -5486,7 +5536,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>42.4%</t>
+          <t>41.8%</t>
         </is>
       </c>
     </row>
@@ -5525,7 +5575,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -5573,7 +5623,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
@@ -5717,7 +5767,7 @@
         </is>
       </c>
       <c r="B34" s="11" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="35">
@@ -6333,10 +6383,10 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C36" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D36" t="n">
         <v>34</v>

</xml_diff>

<commit_message>
chore(mgmt): handover 2026-06-02 および issues_export 更新
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -279,12 +279,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$37</f>
+              <f>'収束グラフ'!$A$2:$A$38</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$B$2:$B$37</f>
+              <f>'収束グラフ'!$B$2:$B$38</f>
             </numRef>
           </val>
         </ser>
@@ -314,12 +314,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$37</f>
+              <f>'収束グラフ'!$A$2:$A$38</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$C$2:$C$37</f>
+              <f>'収束グラフ'!$C$2:$C$38</f>
             </numRef>
           </val>
         </ser>
@@ -349,12 +349,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$37</f>
+              <f>'収束グラフ'!$A$2:$A$38</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$D$2:$D$37</f>
+              <f>'収束グラフ'!$D$2:$D$38</f>
             </numRef>
           </val>
         </ser>
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P70"/>
+  <dimension ref="A1:P74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5579,21 +5579,221 @@
       </c>
       <c r="P70" s="6" t="inlineStr"/>
     </row>
+    <row r="71" ht="40" customHeight="1">
+      <c r="A71" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-070</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>等高線レイヤー描画パラメータ確定（HLD）</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr"/>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>機能追加</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr"/>
+      <c r="G71" s="7" t="inlineStr"/>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="I71" s="7" t="inlineStr">
+        <is>
+          <t>HLD</t>
+        </is>
+      </c>
+      <c r="J71" s="7" t="inlineStr"/>
+      <c r="K71" s="7" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L71" s="7" t="inlineStr"/>
+      <c r="M71" s="7" t="inlineStr"/>
+      <c r="N71" s="7" t="inlineStr">
+        <is>
+          <t>【HLD で詰める内容】ADR-SRS-015 の実装詳細。モックアップ(viewer_mockup.html)での確認値を起点として最終確定する。(1) ズーム別計曲線/主曲線間隔（暫定: z≤11: 500/100m、z≤13: 200/50m、z≤14: 100/20m、z≥15: 50/10m）。(2) 線色・透明度（暫定: 計曲線 #a04020 alpha=120、主曲線 #c87850 alpha=70。OSM・地理院淡色との合成可読性で微調整）。(3) 描画アルゴリズム（現状: 隣接セル比較、257×257拡張グリッドでタイル境界を解消済み）。(4) 本番 HTML 実装時はモックアップの ContourLayer コードを参照すること。</t>
+        </is>
+      </c>
+      <c r="O71" s="7" t="inlineStr"/>
+      <c r="P71" s="7" t="inlineStr"/>
+    </row>
+    <row r="72" ht="40" customHeight="1">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-071</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>標高タイル選択・フォールバック実装方針（HLD）</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr"/>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>機能追加</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="inlineStr"/>
+      <c r="G72" s="6" t="inlineStr"/>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="I72" s="6" t="inlineStr">
+        <is>
+          <t>HLD</t>
+        </is>
+      </c>
+      <c r="J72" s="6" t="inlineStr"/>
+      <c r="K72" s="6" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L72" s="6" t="inlineStr"/>
+      <c r="M72" s="6" t="inlineStr"/>
+      <c r="N72" s="6" t="inlineStr">
+        <is>
+          <t>【HLD で詰める内容】ADR-SRS-015 の実装詳細。(1) ズーム別優先タイル（dem10b/dem5a/dem1a）の選択ロジック確定。(2) 404 時フォールバック順序（dem5a→dem5b→dem5c→dem_png z14 縮小補完）の本番実装。(3) dem1a（z=17、1m メッシュ）採用可否の再評価（ADR-SRS-015 で現状見送り）。(4) 取得失敗時の Canvas タイル扱い（透明 or 「等高線なし」表示）。(5) GSI 規約上問題のない並列リクエスト数の上限確認。(6) fetch + blob URL 方式（CORS canvas taint 回避）の維持確認。</t>
+        </is>
+      </c>
+      <c r="O72" s="6" t="inlineStr"/>
+      <c r="P72" s="6" t="inlineStr"/>
+    </row>
+    <row r="73" ht="40" customHeight="1">
+      <c r="A73" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-072</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>Leaflet pane 構成と重ね順の整理（HLD）</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr"/>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr"/>
+      <c r="G73" s="7" t="inlineStr"/>
+      <c r="H73" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="I73" s="7" t="inlineStr">
+        <is>
+          <t>HLD</t>
+        </is>
+      </c>
+      <c r="J73" s="7" t="inlineStr"/>
+      <c r="K73" s="7" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L73" s="7" t="inlineStr"/>
+      <c r="M73" s="7" t="inlineStr"/>
+      <c r="N73" s="7" t="inlineStr">
+        <is>
+          <t>【HLD で詰める内容】(1) contourPane（z-index=250、pointerEvents=none）の正式採用（モックアップで実装済み・検証必要）。(2) 既存オーバーレイ（基準点 cpLayer z=400、1次メッシュ meshGrid z=400）との z-index 整合性確認。(3) 等高線レイヤーのレイヤーコントロール配置（overlay 欄・デフォルト OFF）の確認。(4) 公開用 HTML（FR-020）への等高線レイヤー引き継ぎ方針。</t>
+        </is>
+      </c>
+      <c r="O73" s="7" t="inlineStr"/>
+      <c r="P73" s="7" t="inlineStr"/>
+    </row>
+    <row r="74" ht="40" customHeight="1">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-073</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>attribution 制御方式の確定（HLD）</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr"/>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="inlineStr"/>
+      <c r="G74" s="6" t="inlineStr"/>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="I74" s="6" t="inlineStr">
+        <is>
+          <t>HLD</t>
+        </is>
+      </c>
+      <c r="J74" s="6" t="inlineStr"/>
+      <c r="K74" s="6" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L74" s="6" t="inlineStr"/>
+      <c r="M74" s="6" t="inlineStr"/>
+      <c r="N74" s="6" t="inlineStr">
+        <is>
+          <t>【HLD で詰める内容】(1) map.attributionControl.addAttribution() による固定 attribution 追加方式の本番実装（モックアップで確認済み）。(2) 基図の GSI 系タイル（地理院標準・淡色）自体の attribution と固定 attribution の重複表示の扱い（現状: 2つの GSI リンクが並ぶ。許容するか整理するか）。(3) 公開用 HTML エクスポート（FR-020）への引き継ぎ確認。</t>
+        </is>
+      </c>
+      <c r="O74" s="6" t="inlineStr"/>
+      <c r="P74" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5629,7 +5829,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3">
@@ -5639,7 +5839,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4">
@@ -5660,7 +5860,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>40.6%</t>
+          <t>38.4%</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5879,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
@@ -5737,7 +5937,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16">
@@ -5747,7 +5947,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17">
@@ -5775,7 +5975,7 @@
         </is>
       </c>
       <c r="B20" s="11" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
@@ -5785,7 +5985,7 @@
         </is>
       </c>
       <c r="B21" s="11" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22">
@@ -5901,7 +6101,7 @@
         </is>
       </c>
       <c r="B35" s="11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36">
@@ -5925,7 +6125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6532,6 +6732,22 @@
         <v>34</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>73</v>
+      </c>
+      <c r="C38" t="n">
+        <v>42</v>
+      </c>
+      <c r="D38" t="n">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
chore(tracker): issues_export.xlsx を ISSUE-074/075/076 登録後に再生成
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -279,12 +279,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$38</f>
+              <f>'収束グラフ'!$A$2:$A$40</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$B$2:$B$38</f>
+              <f>'収束グラフ'!$B$2:$B$40</f>
             </numRef>
           </val>
         </ser>
@@ -314,12 +314,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$38</f>
+              <f>'収束グラフ'!$A$2:$A$40</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$C$2:$C$38</f>
+              <f>'収束グラフ'!$C$2:$C$40</f>
             </numRef>
           </val>
         </ser>
@@ -349,12 +349,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$38</f>
+              <f>'収束グラフ'!$A$2:$A$40</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$D$2:$D$38</f>
+              <f>'収束グラフ'!$D$2:$D$40</f>
             </numRef>
           </val>
         </ser>
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P74"/>
+  <dimension ref="A1:P77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5779,21 +5779,171 @@
       <c r="O74" s="6" t="inlineStr"/>
       <c r="P74" s="6" t="inlineStr"/>
     </row>
+    <row r="75" ht="40" customHeight="1">
+      <c r="A75" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-074</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>Phase構造の再編: Phase 2-1/2-2/3 → Phase 2/3 フェーズ単位ループへ変更</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Phase 2-1/2-2/3 の3区分構造を Phase 2/3 のフェーズ単位ループへ変更する。Phase 3 のループ構造を明示し、3.3.2 俯瞰図と関連 FR 本文を更新する。3.3.1 マトリクスの横軸も Phase 1/2/3/4/5 に再編する。</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="inlineStr"/>
+      <c r="G75" s="7" t="inlineStr"/>
+      <c r="H75" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="I75" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J75" s="7" t="inlineStr"/>
+      <c r="K75" s="7" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L75" s="7" t="inlineStr"/>
+      <c r="M75" s="7" t="inlineStr"/>
+      <c r="N75" s="7" t="inlineStr"/>
+      <c r="O75" s="7" t="inlineStr"/>
+      <c r="P75" s="7" t="inlineStr"/>
+    </row>
+    <row r="76" ht="40" customHeight="1">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-075</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>FR-004/FR-014 責務分担変更 + ADR-SRS-004 更新</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>FR-004 を「3x3メッシュ結合解析オーケストレーション」に改名・3x3 専用に純化（N≥4 モード削除）。FR-014 を「広域結合解析オーケストレーション」に格上げし、4 コーナー配置（NW/NE/SW/SE）生成を内部化。ADR-SRS-004 を本方針に合わせて再更新する。</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="inlineStr"/>
+      <c r="G76" s="6" t="inlineStr"/>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="I76" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J76" s="6" t="inlineStr"/>
+      <c r="K76" s="6" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L76" s="6" t="inlineStr"/>
+      <c r="M76" s="6" t="inlineStr"/>
+      <c r="N76" s="6" t="inlineStr"/>
+      <c r="O76" s="6" t="inlineStr"/>
+      <c r="P76" s="6" t="inlineStr"/>
+    </row>
+    <row r="77" ht="40" customHeight="1">
+      <c r="A77" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-076</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>FR-022 出力明示 + フェーズ遷移制御の所在</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>FR-022 出力テーブルに「未解決ピーク座標リスト」「次の N 値」「次のアクション (Phase 3 起動 / Phase 4 移行)」を明示する。フェーズ遷移制御を SRS のどこまで規定し HLD に何を委ねるかを決定する。</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F77" s="7" t="inlineStr"/>
+      <c r="G77" s="7" t="inlineStr"/>
+      <c r="H77" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="I77" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J77" s="7" t="inlineStr"/>
+      <c r="K77" s="7" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L77" s="7" t="inlineStr"/>
+      <c r="M77" s="7" t="inlineStr"/>
+      <c r="N77" s="7" t="inlineStr"/>
+      <c r="O77" s="7" t="inlineStr"/>
+      <c r="P77" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5829,7 +5979,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3">
@@ -5839,7 +5989,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4">
@@ -5860,7 +6010,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>38.4%</t>
+          <t>36.8%</t>
         </is>
       </c>
     </row>
@@ -5879,7 +6029,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9">
@@ -5947,7 +6097,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17">
@@ -5985,7 +6135,7 @@
         </is>
       </c>
       <c r="B21" s="11" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22">
@@ -6091,7 +6241,7 @@
         </is>
       </c>
       <c r="B34" s="11" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="35">
@@ -6125,7 +6275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6748,6 +6898,38 @@
         <v>34</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>73</v>
+      </c>
+      <c r="C39" t="n">
+        <v>42</v>
+      </c>
+      <c r="D39" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>76</v>
+      </c>
+      <c r="C40" t="n">
+        <v>42</v>
+      </c>
+      <c r="D40" t="n">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
chore: tracker の issues.json / xlsx を更新（ISSUE-077 対応完了）
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -279,12 +279,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$40</f>
+              <f>'収束グラフ'!$A$2:$A$41</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$B$2:$B$40</f>
+              <f>'収束グラフ'!$B$2:$B$41</f>
             </numRef>
           </val>
         </ser>
@@ -314,12 +314,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$40</f>
+              <f>'収束グラフ'!$A$2:$A$41</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$C$2:$C$40</f>
+              <f>'収束グラフ'!$C$2:$C$41</f>
             </numRef>
           </val>
         </ser>
@@ -349,12 +349,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$40</f>
+              <f>'収束グラフ'!$A$2:$A$41</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$D$2:$D$40</f>
+              <f>'収束グラフ'!$D$2:$D$41</f>
             </numRef>
           </val>
         </ser>
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P77"/>
+  <dimension ref="A1:P78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5929,21 +5929,75 @@
       <c r="O77" s="7" t="inlineStr"/>
       <c r="P77" s="7" t="inlineStr"/>
     </row>
+    <row r="78" ht="40" customHeight="1">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-077</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>外部I/F・ユーザ入力・内部データの三分類規約とSRS再編</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr"/>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="inlineStr"/>
+      <c r="G78" s="6" t="inlineStr"/>
+      <c r="H78" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="I78" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J78" s="6" t="inlineStr"/>
+      <c r="K78" s="6" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L78" s="6" t="inlineStr"/>
+      <c r="M78" s="6" t="inlineStr"/>
+      <c r="N78" s="6" t="inlineStr">
+        <is>
+          <t>CLAUDE.md・GLOSSARY・SRS・ADR-SRS-016 を更新。2.2.2廃止→7.2、6.10/6.14/6.16/6.17移設、7→8/8→9/9→10リナンバリング</t>
+        </is>
+      </c>
+      <c r="O78" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="P78" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5979,7 +6033,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3">
@@ -5989,7 +6043,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4">
@@ -6010,7 +6064,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>36.8%</t>
+          <t>36.4%</t>
         </is>
       </c>
     </row>
@@ -6049,7 +6103,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -6087,7 +6141,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16">
@@ -6155,7 +6209,7 @@
         </is>
       </c>
       <c r="B23" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -6241,7 +6295,7 @@
         </is>
       </c>
       <c r="B34" s="11" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="35">
@@ -6275,7 +6329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6930,6 +6984,22 @@
         <v>34</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>77</v>
+      </c>
+      <c r="C41" t="n">
+        <v>43</v>
+      </c>
+      <c r="D41" t="n">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
chore(tracker): ISSUE-081 対応完了に更新・issues_export.xlsx 再生成
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -279,12 +279,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$42</f>
+              <f>'収束グラフ'!$A$2:$A$43</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$B$2:$B$42</f>
+              <f>'収束グラフ'!$B$2:$B$43</f>
             </numRef>
           </val>
         </ser>
@@ -314,12 +314,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$42</f>
+              <f>'収束グラフ'!$A$2:$A$43</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$C$2:$C$42</f>
+              <f>'収束グラフ'!$C$2:$C$43</f>
             </numRef>
           </val>
         </ser>
@@ -349,12 +349,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$42</f>
+              <f>'収束グラフ'!$A$2:$A$43</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$D$2:$D$42</f>
+              <f>'収束グラフ'!$D$2:$D$43</f>
             </numRef>
           </val>
         </ser>
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P81"/>
+  <dimension ref="A1:P82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4845,7 +4845,11 @@
       </c>
       <c r="L57" s="7" t="inlineStr"/>
       <c r="M57" s="7" t="inlineStr"/>
-      <c r="N57" s="7" t="inlineStr"/>
+      <c r="N57" s="7" t="inlineStr">
+        <is>
+          <t>【ADR-SRS-018 反映】北方領土除外タイルリストの読み込みと取得スキップ処理が追加変更点として加わった。enumerate_jobs() または fetch() の段階で、北方領土除外タイルリスト（テキスト: x y ペア）を読み込み、リスト内のタイルはジョブに含めない（HTTP リクエストを発行しない）。既存ローカルキャッシュが存在する場合は削除して地理院側と同じ状態に保つこと（取得しない = リストに入れないのと同義）。</t>
+        </is>
+      </c>
       <c r="O57" s="7" t="inlineStr"/>
       <c r="P57" s="7" t="inlineStr"/>
     </row>
@@ -6155,7 +6159,7 @@
       <c r="M80" s="6" t="inlineStr"/>
       <c r="N80" s="6" t="inlineStr">
         <is>
-          <t>SRS 確定（コミット予定）後に着手する。実装側 ISSUE。</t>
+          <t>【ADR-SRS-018 反映】4.1/4.2 の章順序入れ替え自体には実装上の影響なし。出力ファイル仕様（3 種類）は変更なし。</t>
         </is>
       </c>
       <c r="O80" s="6" t="inlineStr"/>
@@ -6219,21 +6223,81 @@
         </is>
       </c>
     </row>
+    <row r="82" ht="40" customHeight="1">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-081</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>SRS: 北方領土除外をタイル取得段階に前倒し・4.1/4.2 入れ替え・3.2/3.3.1/3.3.2 修正</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>FR-001/FR-017 の順序入れ替えに伴う SRS 改訂。
+主な変更:
+1. 4.1/4.2 セクション番号入れ替え（行政区域前処理→タイル取得の順）
+2. 3.2/3.3.1/3.3.2 もそれに合わせて修正
+3. FR-001 入力: 北方領土除外タイルリスト（必須）追加・1次メッシュコードリストを任意（デフォルト=日本全土）に変更
+4. FR-017 概要修正（FR-004→FR-001）・フォールバック節削除
+5. FR-004 から北方領土タイル除外段落削除
+6. データ辞書 7.2/7.2.1 の参照先を FR-004→FR-001 に変更
+7. ADR-SRS-018 新規作成
+8. ISSUE-056/ISSUE-079 説明文追記
+仕様詳細: mgmt/plan.md</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr"/>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr"/>
+      <c r="G82" s="6" t="inlineStr"/>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="I82" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J82" s="6" t="inlineStr"/>
+      <c r="K82" s="6" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L82" s="6" t="inlineStr"/>
+      <c r="M82" s="6" t="inlineStr"/>
+      <c r="N82" s="6" t="inlineStr"/>
+      <c r="O82" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="P82" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6269,7 +6333,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3">
@@ -6279,7 +6343,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
@@ -6300,7 +6364,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>51.2%</t>
+          <t>50.6%</t>
         </is>
       </c>
     </row>
@@ -6339,7 +6403,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -6377,7 +6441,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16">
@@ -6511,7 +6575,7 @@
         </is>
       </c>
       <c r="B32" s="11" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="33">
@@ -6545,7 +6609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7232,6 +7296,22 @@
         <v>47</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>81</v>
+      </c>
+      <c r="C43" t="n">
+        <v>45</v>
+      </c>
+      <c r="D43" t="n">
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
chore(tracker): ISSUE-079 todo 移行・ISSUE-062 以降のステージ情報補正
- ISSUE-079 (preprocess_pref_boundaries.py FR-017 追従) を todo.md へ移行
- ISSUE-062 以降の未対応 Issue 10 件の発生ステージを SRS に統一
- 各 Issue に対応予定ステージを設定（HTML ビューア系/HLD 確定系=HLD、SRS 改訂系=SRS）

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -5240,8 +5240,16 @@
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="I63" s="7" t="inlineStr"/>
-      <c r="J63" s="7" t="inlineStr"/>
+      <c r="I63" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J63" s="7" t="inlineStr">
+        <is>
+          <t>HLD</t>
+        </is>
+      </c>
       <c r="K63" s="7" t="inlineStr">
         <is>
           <t>未対応</t>
@@ -5294,8 +5302,16 @@
           <t>2026-05-31</t>
         </is>
       </c>
-      <c r="I64" s="6" t="inlineStr"/>
-      <c r="J64" s="6" t="inlineStr"/>
+      <c r="I64" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J64" s="6" t="inlineStr">
+        <is>
+          <t>HLD</t>
+        </is>
+      </c>
       <c r="K64" s="6" t="inlineStr">
         <is>
           <t>未対応</t>
@@ -5460,8 +5476,16 @@
           <t>2026-05-31</t>
         </is>
       </c>
-      <c r="I67" s="7" t="inlineStr"/>
-      <c r="J67" s="7" t="inlineStr"/>
+      <c r="I67" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J67" s="7" t="inlineStr">
+        <is>
+          <t>HLD</t>
+        </is>
+      </c>
       <c r="K67" s="7" t="inlineStr">
         <is>
           <t>未対応</t>
@@ -5694,10 +5718,14 @@
       </c>
       <c r="I71" s="7" t="inlineStr">
         <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J71" s="7" t="inlineStr">
+        <is>
           <t>HLD</t>
         </is>
       </c>
-      <c r="J71" s="7" t="inlineStr"/>
       <c r="K71" s="7" t="inlineStr">
         <is>
           <t>未対応</t>
@@ -5744,10 +5772,14 @@
       </c>
       <c r="I72" s="6" t="inlineStr">
         <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J72" s="6" t="inlineStr">
+        <is>
           <t>HLD</t>
         </is>
       </c>
-      <c r="J72" s="6" t="inlineStr"/>
       <c r="K72" s="6" t="inlineStr">
         <is>
           <t>未対応</t>
@@ -5794,10 +5826,14 @@
       </c>
       <c r="I73" s="7" t="inlineStr">
         <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J73" s="7" t="inlineStr">
+        <is>
           <t>HLD</t>
         </is>
       </c>
-      <c r="J73" s="7" t="inlineStr"/>
       <c r="K73" s="7" t="inlineStr">
         <is>
           <t>未対応</t>
@@ -5844,10 +5880,14 @@
       </c>
       <c r="I74" s="6" t="inlineStr">
         <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J74" s="6" t="inlineStr">
+        <is>
           <t>HLD</t>
         </is>
       </c>
-      <c r="J74" s="6" t="inlineStr"/>
       <c r="K74" s="6" t="inlineStr">
         <is>
           <t>未対応</t>
@@ -5901,7 +5941,11 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J75" s="7" t="inlineStr"/>
+      <c r="J75" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
       <c r="K75" s="7" t="inlineStr">
         <is>
           <t>未対応</t>
@@ -5951,7 +5995,11 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J76" s="6" t="inlineStr"/>
+      <c r="J76" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
       <c r="K76" s="6" t="inlineStr">
         <is>
           <t>未対応</t>
@@ -6001,7 +6049,11 @@
           <t>SRS</t>
         </is>
       </c>
-      <c r="J77" s="7" t="inlineStr"/>
+      <c r="J77" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
       <c r="K77" s="7" t="inlineStr">
         <is>
           <t>未対応</t>
@@ -6140,17 +6192,17 @@
       </c>
     </row>
     <row r="80" ht="40" customHeight="1">
-      <c r="A80" s="6" t="inlineStr">
+      <c r="A80" s="2" t="inlineStr">
         <is>
           <t>ISSUE-079</t>
         </is>
       </c>
-      <c r="B80" s="6" t="inlineStr">
+      <c r="B80" s="2" t="inlineStr">
         <is>
           <t>scripts/preprocess_pref_boundaries.py を FR-017 改訂版仕様に追従</t>
         </is>
       </c>
-      <c r="C80" s="6" t="inlineStr">
+      <c r="C80" s="2" t="inlineStr">
         <is>
           <t>FR-017 SRS 改訂（2026-06-05）に伴う実装変更。
 主な変更点:
@@ -6163,7 +6215,7 @@
 仕様詳細: docs/02_SRS.md FR-017・7.1.3・7.2.1・ADR-URD-005</t>
         </is>
       </c>
-      <c r="D80" s="6" t="inlineStr">
+      <c r="D80" s="2" t="inlineStr">
         <is>
           <t>改善</t>
         </is>
@@ -6173,37 +6225,41 @@
           <t>高</t>
         </is>
       </c>
-      <c r="F80" s="6" t="inlineStr">
+      <c r="F80" s="2" t="inlineStr">
         <is>
           <t>その他</t>
         </is>
       </c>
-      <c r="G80" s="6" t="inlineStr"/>
-      <c r="H80" s="6" t="inlineStr">
+      <c r="G80" s="2" t="inlineStr"/>
+      <c r="H80" s="2" t="inlineStr">
         <is>
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="I80" s="6" t="inlineStr">
+      <c r="I80" s="2" t="inlineStr">
         <is>
           <t>COD</t>
         </is>
       </c>
-      <c r="J80" s="6" t="inlineStr"/>
-      <c r="K80" s="6" t="inlineStr">
-        <is>
-          <t>未対応</t>
-        </is>
-      </c>
-      <c r="L80" s="6" t="inlineStr"/>
-      <c r="M80" s="6" t="inlineStr"/>
-      <c r="N80" s="6" t="inlineStr">
+      <c r="J80" s="2" t="inlineStr"/>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>却下</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="inlineStr"/>
+      <c r="M80" s="2" t="inlineStr"/>
+      <c r="N80" s="2" t="inlineStr">
         <is>
           <t>【ADR-SRS-018 反映】4.1/4.2 の章順序入れ替え自体には実装上の影響なし。出力ファイル仕様（3 種類）は変更なし。</t>
         </is>
       </c>
-      <c r="O80" s="6" t="inlineStr"/>
-      <c r="P80" s="6" t="inlineStr"/>
+      <c r="O80" s="2" t="inlineStr"/>
+      <c r="P80" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="40" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
@@ -6355,7 +6411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6387,7 +6443,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -6427,7 +6483,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
@@ -6467,7 +6523,7 @@
         </is>
       </c>
       <c r="B12" s="11" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14">
@@ -6485,7 +6541,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16">
@@ -6533,7 +6589,7 @@
         </is>
       </c>
       <c r="B21" s="11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22">
@@ -6591,7 +6647,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
@@ -6609,7 +6665,7 @@
         </is>
       </c>
       <c r="B31" s="11" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="32">
@@ -6619,16 +6675,6 @@
         </is>
       </c>
       <c r="B32" s="11" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>COD</t>
-        </is>
-      </c>
-      <c r="B33" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7343,7 +7389,7 @@
         <v>45</v>
       </c>
       <c r="D43" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(plan): FR-005 レビュー保留・ISSUE-087 起票・ISSUE-075 先行着手プラン
FR-005「ピーク候補検出」のレビュー観点 A〜N を整理した結果、観点 L（制御フロー・
オーケストレーション所在の明示）が浮上。L の改善方向は FR-004 のオーケストレー
ション役割集約を含むため、ISSUE-075（FR-004/FR-014 責務再編）と一体作業になる。

ISSUE-075 完了を待ってから FR-005 レビューに戻る方針とし、観点リスト A〜N を
ISSUE-087 として永続化。ISSUE-075 notes にも「完了後 ISSUE-087 着手」を記録。
mgmt/plan.md は ISSUE-075 着手プランで上書きした。

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -279,12 +279,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$44</f>
+              <f>'収束グラフ'!$A$2:$A$45</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$B$2:$B$44</f>
+              <f>'収束グラフ'!$B$2:$B$45</f>
             </numRef>
           </val>
         </ser>
@@ -314,12 +314,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$44</f>
+              <f>'収束グラフ'!$A$2:$A$45</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$C$2:$C$44</f>
+              <f>'収束グラフ'!$C$2:$C$45</f>
             </numRef>
           </val>
         </ser>
@@ -349,12 +349,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$44</f>
+              <f>'収束グラフ'!$A$2:$A$45</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$D$2:$D$44</f>
+              <f>'収束グラフ'!$D$2:$D$45</f>
             </numRef>
           </val>
         </ser>
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P87"/>
+  <dimension ref="A1:P88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6007,7 +6007,11 @@
       </c>
       <c r="L76" s="6" t="inlineStr"/>
       <c r="M76" s="6" t="inlineStr"/>
-      <c r="N76" s="6" t="inlineStr"/>
+      <c r="N76" s="6" t="inlineStr">
+        <is>
+          <t>完了後、ISSUE-087（SRS FR-005 ピーク候補検出のレビュー反映）に着手すること。FR-005 観点 L（制御フロー・オーケストレーション所在）の確定は本 ISSUE の再編結果に依存する。</t>
+        </is>
+      </c>
       <c r="O76" s="6" t="inlineStr"/>
       <c r="P76" s="6" t="inlineStr"/>
     </row>
@@ -6653,21 +6657,110 @@
       <c r="O87" s="7" t="inlineStr"/>
       <c r="P87" s="7" t="inlineStr"/>
     </row>
+    <row r="88" ht="40" customHeight="1">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-087</t>
+        </is>
+      </c>
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>SRS FR-005 ピーク候補検出のレビュー反映</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="inlineStr">
+        <is>
+          <t>SRS FR-005「ピーク候補検出」のレビュー結果を反映する。
+## 前提条件
+ISSUE-075（FR-004/FR-014 責務再編 + ADR-SRS-004 更新）完了が前提。
+観点 L/M/N の確定は ISSUE-075 の再編結果に依存するため、ISSUE-075 完了後に着手すること。
+## レビュー観点リスト
+| 観点 | 内容 | 優先度 | 備考 |
+|---|---|---|---|
+| L | 制御フロー・オーケストレーション所在の明示 | 最重要 | ISSUE-075 完了後に確定 |
+| M | FR-005/006 単一走査の明示（C から発展） | 高 | ISSUE-075 完了後に確定 |
+| N | FR-007/016 への遷移条件 | 高 | ISSUE-075 完了後に確定 |
+| A | 対応 UR（UR-002 除外検討） | 中 | 独立に判断可 |
+| B | 概要の中粒度化 | 中 | 独立に判断可 |
+| D | 説明の仕様抜け（NODATA・0m・決定論・1px ボーダー） | 中 | 独立に判断可 |
+| E | 出力テーブル形式欄整理（CLAUDE.md 観点 I 違反） | 低 | 独立に判断可 |
+| F | 「ピーク候補」と「ピーク」の使い分け | 中 | 独立に判断可 |
+| G | 「山塊グループ」用語定義 | 低 | 独立に判断可 |
+| H | 異常系セクションの有無 | 低 | 独立に判断可 |
+| I | 広域モード言及 | 低 | ISSUE-075 完了後に整合確認 |
+| J | アルゴリズム説明の SRS/HLD 所在 | 中 | 独立に判断可 |
+| K | 内部データ分類見直し | — | ISSUE-084 既登録・本件対象外 |
+## 観点 L の現状認識
+- SRS では各 FR の責務は書かれているが、全体の制御がどう流れるかが見えない
+- FR-004 概要「per-mesh パイプライン（FR-005〜FR-007・FR-016）に引き渡す」の「引き渡す」が曖昧
+- FR-005 説明はピクセル単位の動作のみで、ループの主体（誰が回すか）が不明
+- FR-006 説明「FR-005 の処理中に…」で走査共有が暗黙
+- per-mesh パイプライン全体の処理フロー俯瞰図が SRS にない
+## 改善方向（ISSUE-075 完了後に確定）
+1. FR-004 に「per-mesh オーケストレーション役割」を明示（結合画像生成 → FR-005/006 走査 → FR-007 出力 → FR-016 ポリゴン生成）
+2. FR-005/FR-006 を「同一の単一ピクセル走査ループ内で機能分担して実行」と明示
+3. 4.3 セクション冒頭 or FR-004 説明末尾に per-mesh パイプライン処理フロー図を追加
+## 議論経緯（2026-06-09 セッション）
+FR-005 レビュー観点を整理する中で、ユーザーから「全体との関連がよくわからない。FR-004 と FR-005 の制御所在が不明」との指摘があり観点 L が浮上。L の改善方向は FR-004 のオーケストレーション役割明示を含み、ISSUE-075 の再編と一体作業になるため、ISSUE-075 完了後に本 ISSUE 着手とした。</t>
+        </is>
+      </c>
+      <c r="D88" s="6" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F88" s="6" t="inlineStr"/>
+      <c r="G88" s="6" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="I88" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J88" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="K88" s="6" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L88" s="6" t="inlineStr"/>
+      <c r="M88" s="6" t="inlineStr"/>
+      <c r="N88" s="6" t="inlineStr"/>
+      <c r="O88" s="6" t="inlineStr"/>
+      <c r="P88" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6703,7 +6796,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3">
@@ -6713,7 +6806,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
@@ -6734,7 +6827,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>48.8%</t>
+          <t>48.3%</t>
         </is>
       </c>
     </row>
@@ -6753,7 +6846,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
@@ -6821,7 +6914,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
@@ -6859,7 +6952,7 @@
         </is>
       </c>
       <c r="B21" s="11" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22">
@@ -6945,7 +7038,7 @@
         </is>
       </c>
       <c r="B32" s="11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33">
@@ -6979,7 +7072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7698,6 +7791,22 @@
         <v>59</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>87</v>
+      </c>
+      <c r="C45" t="n">
+        <v>45</v>
+      </c>
+      <c r="D45" t="n">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
chore(tracker): issues_export.xlsx 再生成 (ISSUE-075 対応完了反映)
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -6002,7 +6002,7 @@
       </c>
       <c r="K76" s="6" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="L76" s="6" t="inlineStr"/>
@@ -6012,7 +6012,11 @@
           <t>完了後、ISSUE-087（SRS FR-005 ピーク候補検出のレビュー反映）に着手すること。FR-005 観点 L（制御フロー・オーケストレーション所在）の確定は本 ISSUE の再編結果に依存する。</t>
         </is>
       </c>
-      <c r="O76" s="6" t="inlineStr"/>
+      <c r="O76" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="P76" s="6" t="inlineStr"/>
     </row>
     <row r="77" ht="40" customHeight="1">
@@ -6846,7 +6850,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9">
@@ -6866,7 +6870,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -7801,7 +7805,7 @@
         <v>87</v>
       </c>
       <c r="C45" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D45" t="n">
         <v>59</v>

</xml_diff>

<commit_message>
chore(tracker): issues_export.xlsx 再生成 (ISSUE-088 登録・対応完了反映)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -279,12 +279,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$45</f>
+              <f>'収束グラフ'!$A$2:$A$47</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$B$2:$B$45</f>
+              <f>'収束グラフ'!$B$2:$B$47</f>
             </numRef>
           </val>
         </ser>
@@ -314,12 +314,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$45</f>
+              <f>'収束グラフ'!$A$2:$A$47</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$C$2:$C$45</f>
+              <f>'収束グラフ'!$C$2:$C$47</f>
             </numRef>
           </val>
         </ser>
@@ -349,12 +349,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$45</f>
+              <f>'収束グラフ'!$A$2:$A$47</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$D$2:$D$45</f>
+              <f>'収束グラフ'!$D$2:$D$47</f>
             </numRef>
           </val>
         </ser>
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P88"/>
+  <dimension ref="A1:P89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6750,21 +6750,110 @@
       <c r="O88" s="6" t="inlineStr"/>
       <c r="P88" s="6" t="inlineStr"/>
     </row>
+    <row r="89" ht="40" customHeight="1">
+      <c r="A89" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-088</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>SRS FR-004 メッシュ結合解析のレビュー反映</t>
+        </is>
+      </c>
+      <c r="C89" s="7" t="inlineStr">
+        <is>
+          <t>FR-004（メッシュ結合解析）のレビュー結果（観点 A〜J）を SRS / ADR-SRS-003 に反映する。
+## レビュー観点リスト
+| 観点 | 内容 | 重要度 |
+|---|---|---|
+| A | ADR-SRS-003 との矛盾: ADR「出力は中心メッシュ内のピークのみ」vs SRS「解析対象メッシュ全体の地理的範囲内のピークを出力」。SRS が正（analysis_count 最大9回・FR-008 重複排除と整合）。ADR の Decision を更新 | 高 |
+| B | 入力テーブル不足: 「標高タイル（ローカルキャッシュ）」が FR-004 入力に無い（7.2 一覧・FR-002 入力と不整合）→ 追加 | 高 |
+| C | 誤参照: 「安定性を評価する（FR-009 参照）」→ stability の定義・算出は FR-008 → 修正 | 中 |
+| D | ピーク出力範囲（地理的範囲フィルタ＝フリンジ除外）の記述所在: FR-007 の責務だが FR-007 に記述なし → 整理 | 中 |
+| E | FR-015 呼び出しがオーケストレーション記述から漏れ → タイミング含め明示 | 中 |
+| F | 出力備考「解析対象メッシュ範囲情報を伴う」が未定義 → 定義明文化 | 中 |
+| G | 結合画像範囲の曖昧さ: リスト外メッシュの NODATA 扱いと範囲定義（bounding box）を明文化 | 中 |
+| H | 「全176メッシュ」ハードコード → 「メッシュコードリストの全メッシュ」表現に修正 | 低 |
+| I | 入力備考: 1次メッシュコードリストに [7.1.1 参照] 付与 | 低 |
+| J | オーケストレーション役割の明示 + per-mesh パイプライン処理フロー図追加（ISSUE-087 観点 L の FR-004 側作業を本 ISSUE に取り込み） | 高 |
+## 運用合意（2026-06-11）
+観点 A〜J は個別確認を省略し Fable 提案通りに一括修正。次回セッションで修正後の FR-004 を再レビューする（実質の verify）。ISSUE-075・ISSUE-087 への注記・verify は FR-004 と FR-014 両方のレビュー完了後に行う。</t>
+        </is>
+      </c>
+      <c r="D89" s="7" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F89" s="7" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G89" s="7" t="inlineStr">
+        <is>
+          <t>JJ1XGO</t>
+        </is>
+      </c>
+      <c r="H89" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="I89" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J89" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="K89" s="7" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L89" s="7" t="inlineStr">
+        <is>
+          <t>Fable</t>
+        </is>
+      </c>
+      <c r="M89" s="7" t="inlineStr">
+        <is>
+          <t>SRS FR-004 セクション・FR-007（観点 D）・ADR-SRS-003（観点 A）を修正し、処理フロー図を追加する</t>
+        </is>
+      </c>
+      <c r="N89" s="7" t="inlineStr"/>
+      <c r="O89" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="P89" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J89" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6800,7 +6889,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3">
@@ -6810,7 +6899,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -6831,7 +6920,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>48.3%</t>
+          <t>47.7%</t>
         </is>
       </c>
     </row>
@@ -6870,7 +6959,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -6918,7 +7007,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17">
@@ -6956,7 +7045,7 @@
         </is>
       </c>
       <c r="B21" s="11" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22">
@@ -7024,7 +7113,7 @@
         </is>
       </c>
       <c r="B29" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31">
@@ -7042,7 +7131,7 @@
         </is>
       </c>
       <c r="B32" s="11" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="33">
@@ -7076,7 +7165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7811,6 +7900,38 @@
         <v>59</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>87</v>
+      </c>
+      <c r="C46" t="n">
+        <v>46</v>
+      </c>
+      <c r="D46" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>88</v>
+      </c>
+      <c r="C47" t="n">
+        <v>47</v>
+      </c>
+      <c r="D47" t="n">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
chore(tracker): ISSUE-090 notes にレビュー論点を転記・issues_export.xlsx 再生成
次セッションでの第2回レビュー用に「Fable の判断で直した点」4件と
持ち越し議論（解析範囲サイズ N の種別等）を ISSUE-090 の notes に全文記録。

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -6959,7 +6959,20 @@
           <t>docs/20_SRS.md（FR-014/007/015/022・俯瞰図）と ADR-SRS-004 を改訂。修正後にユーザーレビューを実施し第2回反映を行う。持ち越し議論: 解析範囲サイズ N の種別・B群推奨案の妥当性。</t>
         </is>
       </c>
-      <c r="N91" s="7" t="inlineStr"/>
+      <c r="N91" s="7" t="inlineStr">
+        <is>
+          <t>【次セッションでユーザーレビュー予定。以下、修正完了報告の該当部をそのまま転記】
+■ Fable の判断で直した点（ここがレビューの中心です）
+1. 無効パターンスキップの再定義（最重要）: 旧規則「存在しないメッシュを含むパターンはスキップ」だと、日本海沿岸の鳥海山（広域解析の本命ターゲット）はウィンドウに海域メッシュをほぼ必ず含むため全パターンスキップ＝広域解析が一切走らない、という矛盾がありました。「存在しないメッシュは NODATA 充填で続行し、存在メッシュが 3×3 解析済み範囲から 1 枚も増えないパターンだけスキップ」に変更しました
+2. 所属メッシュ単位のグルーピング: 同一メッシュに複数の未確定ピークがあると、ファイル名（4-5239-NW.csv）が衝突し同じウィンドウを二度解析する問題があったため、メッシュ単位でまとめて解析し「所属ピーク全部が解決したら早期終了」としました
+3. L15 座標の維持: 広域は L14（max pooling）で解析しますが、座標が L14 になると FR-008 の重複排除（L15 座標一致）が壊れるため、「pooling で採用した最大値ピクセルの L15 座標を保持して出力する」と明記しました
+4. 異常系: 3×3 相当範囲のタイルゼロは処理中止（FR-004 と同じ）、広域で初めて触れる範囲のタイル欠如は NODATA 続行、と区別しました
+（ついでに直したもの: 根拠式の誤記（2√2≒2.8倍）、コーナー表記の方角ベース統一（ADR の例示テーブルは範囲計算自体が誤っていたので再計算）、FR-007 に対象ピーク座標リスト入力と zoom_level カラム追加、ISSUE-051/052 も本対応に取り込みクローズ）
+■ 持ち越し議論（ご意見ください）
+- 「解析範囲サイズ N」の種別: 現状「ユーザー入力」のままですが、実際は FR-022 が自動で渡す値です。また、データ辞書 2.2.1 の「通常解析の N×N（デフォルト3）」という記述とも意味がずれています
+- 上記 1〜4 の判断の妥当性</t>
+        </is>
+      </c>
       <c r="O91" s="7" t="inlineStr"/>
       <c r="P91" s="7" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
chore(tracker): ISSUE-087 対応完了でクローズ・issues_export.xlsx 再生成
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -6777,13 +6777,17 @@
       </c>
       <c r="K88" s="6" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="L88" s="6" t="inlineStr"/>
       <c r="M88" s="6" t="inlineStr"/>
       <c r="N88" s="6" t="inlineStr"/>
-      <c r="O88" s="6" t="inlineStr"/>
+      <c r="O88" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
       <c r="P88" s="6" t="inlineStr"/>
     </row>
     <row r="89" ht="40" customHeight="1">
@@ -7174,7 +7178,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
@@ -7194,7 +7198,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -8193,7 +8197,7 @@
         <v>91</v>
       </c>
       <c r="C49" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D49" t="n">
         <v>68</v>

</xml_diff>

<commit_message>
chore(tracker): ISSUE-084 対応完了でクローズ・issues_export.xlsx 再生成
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -279,12 +279,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$49</f>
+              <f>'収束グラフ'!$A$2:$A$50</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$B$2:$B$49</f>
+              <f>'収束グラフ'!$B$2:$B$50</f>
             </numRef>
           </val>
         </ser>
@@ -314,12 +314,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$49</f>
+              <f>'収束グラフ'!$A$2:$A$50</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$C$2:$C$49</f>
+              <f>'収束グラフ'!$C$2:$C$50</f>
             </numRef>
           </val>
         </ser>
@@ -349,12 +349,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$49</f>
+              <f>'収束グラフ'!$A$2:$A$50</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$D$2:$D$49</f>
+              <f>'収束グラフ'!$D$2:$D$50</f>
             </numRef>
           </val>
         </ser>
@@ -6568,7 +6568,7 @@
       <c r="J85" s="7" t="inlineStr"/>
       <c r="K85" s="7" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="L85" s="7" t="inlineStr"/>
@@ -6578,7 +6578,11 @@
           <t>FR-015 レビュー（観点 H）の別 ISSUE として登録。解析範囲結合画像の内部トランザクション化（ISSUE-083 相当修正）との一貫性検討として登録</t>
         </is>
       </c>
-      <c r="O85" s="7" t="inlineStr"/>
+      <c r="O85" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
       <c r="P85" s="7" t="inlineStr"/>
     </row>
     <row r="86" ht="40" customHeight="1">
@@ -7178,7 +7182,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -7198,7 +7202,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -7404,7 +7408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8203,6 +8207,22 @@
         <v>68</v>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>91</v>
+      </c>
+      <c r="C50" t="n">
+        <v>56</v>
+      </c>
+      <c r="D50" t="n">
+        <v>68</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
chore(tracker): ISSUE-084・087 解決済に更新・issues_export.xlsx 再生成
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -6528,22 +6528,22 @@
       <c r="P84" s="6" t="inlineStr"/>
     </row>
     <row r="85" ht="40" customHeight="1">
-      <c r="A85" s="7" t="inlineStr">
+      <c r="A85" s="2" t="inlineStr">
         <is>
           <t>ISSUE-084</t>
         </is>
       </c>
-      <c r="B85" s="7" t="inlineStr">
+      <c r="B85" s="2" t="inlineStr">
         <is>
           <t>ピーク候補リスト・コル情報の内部トランザクション化検討</t>
         </is>
       </c>
-      <c r="C85" s="7" t="inlineStr">
+      <c r="C85" s="2" t="inlineStr">
         <is>
           <t>解析範囲結合画像と同様に、ピーク候補リスト・コル情報も内部トランザクションとして分類すべきかを検討する。FR-005 出力のピーク候補リストと FR-006 出力のコル情報は独立した中央データ構造として保持されるか（内部データ）、FR 間の一時的な受け渡し値に過ぎないか（内部トランザクション）を ADR-SRS-017 の基準で判定する。</t>
         </is>
       </c>
-      <c r="D85" s="7" t="inlineStr">
+      <c r="D85" s="2" t="inlineStr">
         <is>
           <t>設計</t>
         </is>
@@ -6553,37 +6553,41 @@
           <t>低</t>
         </is>
       </c>
-      <c r="F85" s="7" t="inlineStr"/>
-      <c r="G85" s="7" t="inlineStr"/>
-      <c r="H85" s="7" t="inlineStr">
+      <c r="F85" s="2" t="inlineStr"/>
+      <c r="G85" s="2" t="inlineStr"/>
+      <c r="H85" s="2" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="I85" s="7" t="inlineStr">
+      <c r="I85" s="2" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="J85" s="7" t="inlineStr"/>
-      <c r="K85" s="7" t="inlineStr">
-        <is>
-          <t>対応完了</t>
-        </is>
-      </c>
-      <c r="L85" s="7" t="inlineStr"/>
-      <c r="M85" s="7" t="inlineStr"/>
-      <c r="N85" s="7" t="inlineStr">
+      <c r="J85" s="2" t="inlineStr"/>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L85" s="2" t="inlineStr"/>
+      <c r="M85" s="2" t="inlineStr"/>
+      <c r="N85" s="2" t="inlineStr">
         <is>
           <t>FR-015 レビュー（観点 H）の別 ISSUE として登録。解析範囲結合画像の内部トランザクション化（ISSUE-083 相当修正）との一貫性検討として登録</t>
         </is>
       </c>
-      <c r="O85" s="7" t="inlineStr">
+      <c r="O85" s="2" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="P85" s="7" t="inlineStr"/>
+      <c r="P85" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="40" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
@@ -6702,17 +6706,17 @@
       </c>
     </row>
     <row r="88" ht="40" customHeight="1">
-      <c r="A88" s="6" t="inlineStr">
+      <c r="A88" s="2" t="inlineStr">
         <is>
           <t>ISSUE-087</t>
         </is>
       </c>
-      <c r="B88" s="6" t="inlineStr">
+      <c r="B88" s="2" t="inlineStr">
         <is>
           <t>SRS FR-005 ピーク候補検出のレビュー反映</t>
         </is>
       </c>
-      <c r="C88" s="6" t="inlineStr">
+      <c r="C88" s="2" t="inlineStr">
         <is>
           <t>SRS FR-005「ピーク候補検出」のレビュー結果を反映する。
 ## 前提条件
@@ -6748,7 +6752,7 @@
 FR-005 レビュー観点を整理する中で、ユーザーから「全体との関連がよくわからない。FR-004 と FR-005 の制御所在が不明」との指摘があり観点 L が浮上。L の改善方向は FR-004 のオーケストレーション役割明示を含み、ISSUE-075 の再編と一体作業になるため、ISSUE-075 完了後に本 ISSUE 着手とした。</t>
         </is>
       </c>
-      <c r="D88" s="6" t="inlineStr">
+      <c r="D88" s="2" t="inlineStr">
         <is>
           <t>改善</t>
         </is>
@@ -6758,41 +6762,45 @@
           <t>中</t>
         </is>
       </c>
-      <c r="F88" s="6" t="inlineStr"/>
-      <c r="G88" s="6" t="inlineStr">
+      <c r="F88" s="2" t="inlineStr"/>
+      <c r="G88" s="2" t="inlineStr">
         <is>
           <t>JJ1XGO</t>
         </is>
       </c>
-      <c r="H88" s="6" t="inlineStr">
+      <c r="H88" s="2" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="I88" s="6" t="inlineStr">
+      <c r="I88" s="2" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="J88" s="6" t="inlineStr">
+      <c r="J88" s="2" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="K88" s="6" t="inlineStr">
-        <is>
-          <t>対応完了</t>
-        </is>
-      </c>
-      <c r="L88" s="6" t="inlineStr"/>
-      <c r="M88" s="6" t="inlineStr"/>
-      <c r="N88" s="6" t="inlineStr"/>
-      <c r="O88" s="6" t="inlineStr">
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="inlineStr"/>
+      <c r="M88" s="2" t="inlineStr"/>
+      <c r="N88" s="2" t="inlineStr"/>
+      <c r="O88" s="2" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="P88" s="6" t="inlineStr"/>
+      <c r="P88" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="40" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
@@ -7110,7 +7118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7142,7 +7150,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -7152,7 +7160,7 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5">
@@ -7163,7 +7171,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>56.0%</t>
+          <t>58.2%</t>
         </is>
       </c>
     </row>
@@ -7202,7 +7210,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -7212,7 +7220,7 @@
         </is>
       </c>
       <c r="B11" s="11" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12">
@@ -7250,7 +7258,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
@@ -7260,7 +7268,7 @@
         </is>
       </c>
       <c r="B17" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -7288,7 +7296,7 @@
         </is>
       </c>
       <c r="B21" s="11" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="22">
@@ -7301,99 +7309,89 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>設計</t>
-        </is>
-      </c>
-      <c r="B23" s="11" t="n">
-        <v>1</v>
-      </c>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>カテゴリ別（未解決）</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>カテゴリ別（未解決）</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="n"/>
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>解析エンジン</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>解析エンジン</t>
+          <t>merge.py</t>
         </is>
       </c>
       <c r="B26" s="11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>merge.py</t>
+          <t>GeoJSON出力</t>
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>GeoJSON出力</t>
+          <t>その他</t>
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>その他</t>
-        </is>
-      </c>
-      <c r="B29" s="11" t="n">
         <v>4</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>ステージ別（未解決）</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="n"/>
+    </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>ステージ別（未解決）</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="n"/>
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>SRS</t>
+          <t>HLD</t>
         </is>
       </c>
       <c r="B32" s="11" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>HLD</t>
+          <t>COD</t>
         </is>
       </c>
       <c r="B33" s="11" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>COD</t>
-        </is>
-      </c>
-      <c r="B34" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8220,7 +8218,7 @@
         <v>56</v>
       </c>
       <c r="D50" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(tracker): ISSUE-083 解決済に更新・issues_export.xlsx 再生成
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -6474,22 +6474,22 @@
       </c>
     </row>
     <row r="84" ht="40" customHeight="1">
-      <c r="A84" s="6" t="inlineStr">
+      <c r="A84" s="2" t="inlineStr">
         <is>
           <t>ISSUE-083</t>
         </is>
       </c>
-      <c r="B84" s="6" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr">
         <is>
           <t>SRS 全 FR の入出力テーブル形式欄の一括見直し</t>
         </is>
       </c>
-      <c r="C84" s="6" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
         <is>
           <t>SRS の全 FR 入出力テーブルの「形式」欄を見直し、ファイル形式・データ型のみに統一する。特性記述（解像度・色分け・データ範囲等）は「備考」欄に移動する。CLAUDE.md ドキュメントフォーマット標準に方針を追記済み（FR-015 レビュー観点 I 対応時に追記）。FR-015 出力テーブルは観点 I の対応で修正済み。残りの全 FR 分が対象。</t>
         </is>
       </c>
-      <c r="D84" s="6" t="inlineStr">
+      <c r="D84" s="2" t="inlineStr">
         <is>
           <t>改善</t>
         </is>
@@ -6499,37 +6499,41 @@
           <t>低</t>
         </is>
       </c>
-      <c r="F84" s="6" t="inlineStr"/>
-      <c r="G84" s="6" t="inlineStr"/>
-      <c r="H84" s="6" t="inlineStr">
+      <c r="F84" s="2" t="inlineStr"/>
+      <c r="G84" s="2" t="inlineStr"/>
+      <c r="H84" s="2" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="I84" s="6" t="inlineStr">
+      <c r="I84" s="2" t="inlineStr">
         <is>
           <t>SRS</t>
         </is>
       </c>
-      <c r="J84" s="6" t="inlineStr"/>
-      <c r="K84" s="6" t="inlineStr">
-        <is>
-          <t>対応完了</t>
-        </is>
-      </c>
-      <c r="L84" s="6" t="inlineStr"/>
-      <c r="M84" s="6" t="inlineStr"/>
-      <c r="N84" s="6" t="inlineStr">
+      <c r="J84" s="2" t="inlineStr"/>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L84" s="2" t="inlineStr"/>
+      <c r="M84" s="2" t="inlineStr"/>
+      <c r="N84" s="2" t="inlineStr">
         <is>
           <t>FR-015 レビュー（観点 I）の別 ISSUE として登録。CLAUDE.md のフォーマット標準『入出力テーブルの形式欄はファイル形式・データ型のみを記載する』が根拠</t>
         </is>
       </c>
-      <c r="O84" s="6" t="inlineStr">
+      <c r="O84" s="2" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="P84" s="6" t="inlineStr"/>
+      <c r="P84" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="40" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
@@ -7278,7 +7282,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -7288,7 +7292,7 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5">
@@ -7299,7 +7303,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>57.0%</t>
+          <t>58.1%</t>
         </is>
       </c>
     </row>
@@ -7338,7 +7342,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -7348,7 +7352,7 @@
         </is>
       </c>
       <c r="B11" s="11" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12">
@@ -7396,7 +7400,7 @@
         </is>
       </c>
       <c r="B17" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -7424,7 +7428,7 @@
         </is>
       </c>
       <c r="B21" s="11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22">
@@ -7500,7 +7504,7 @@
         </is>
       </c>
       <c r="B31" s="11" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="32">
@@ -8346,7 +8350,7 @@
         <v>57</v>
       </c>
       <c r="D50" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(srs): FR-016 レビュー反映（完了）— FR-018/009/008空行・GLOSSARY・ADR-SRS-022作成・ISSUE登録
- FR-008: 出力テーブル末尾の空行を挿入（**説明**: との混入解消）
- FR-018: 出力テーブル末尾の空行を挿入・統合キー=peak_lat/peak_lon を明記（ADR-SRS-022）
- FR-009: 出力テーブル末尾の空行を挿入・merged_peak.csv と merged_activation.geojson の
  join キー=peak_lat/peak_lon を突合説明に明記（ADR-SRS-022）
- GLOSSARY: アクティベーションゾーンにデータ辞書リンク追記・delete判定ゾーンの
  「SRS 3.4.1」→「SRS 2.2.1」修正（論点4）
- ADR-SRS-022 作成: per-mesh GeoJSON join方式＋FR-007→FR-016データフロー決定
- ISSUE-100/101/102 登録・対応完了（論点1・論点3・指摘2）
- todo.md: ADR-SRS-022コード追従タスク・GeoJSON命名整理タスクを追加（論点5）

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P99"/>
+  <dimension ref="A1:P102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7552,21 +7552,207 @@
         </is>
       </c>
     </row>
+    <row r="100" ht="40" customHeight="1">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-100</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>FR-016 per-mesh GeoJSON プロパティ設計（join 方式）</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr">
+        <is>
+          <t>FR-016 出力プロパティが未定義のまま FR-009 が merged_activation.geojson と merged_peak.csv を突合する設計だった。プロパティを peak_lat/peak_lon（join キー）+ feature_type + area_complete の4フィールドに限定し、属性は CSV に集約する join 方式を採用（ADR-SRS-022）。</t>
+        </is>
+      </c>
+      <c r="D100" s="6" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F100" s="6" t="inlineStr"/>
+      <c r="G100" s="6" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H100" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="I100" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J100" s="6" t="inlineStr"/>
+      <c r="K100" s="6" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L100" s="6" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="M100" s="6" t="inlineStr">
+        <is>
+          <t>SRS FR-016/018/009 を join 方式に整合して更新。ADR-SRS-022 作成済み。</t>
+        </is>
+      </c>
+      <c r="N100" s="6" t="inlineStr"/>
+      <c r="O100" s="6" t="inlineStr"/>
+      <c r="P100" s="6" t="inlineStr"/>
+    </row>
+    <row r="101" ht="40" customHeight="1">
+      <c r="A101" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-101</t>
+        </is>
+      </c>
+      <c r="B101" s="7" t="inlineStr">
+        <is>
+          <t>FR-016 delete_zone 再生成不要の根拠明記</t>
+        </is>
+      </c>
+      <c r="C101" s="7" t="inlineStr">
+        <is>
+          <t>key_col_resolved=false のピークはコル確定後も delete_zone を再生成しない。理由が SRS に記載されていなかった。</t>
+        </is>
+      </c>
+      <c r="D101" s="7" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E101" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F101" s="7" t="inlineStr"/>
+      <c r="G101" s="7" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H101" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="I101" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J101" s="7" t="inlineStr"/>
+      <c r="K101" s="7" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L101" s="7" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="M101" s="7" t="inlineStr">
+        <is>
+          <t>FR-016 の詳細説明に許容根拠（3×3 でコル未検出＝実質プロミネンス大で max_drop キャップが実効的、過大化しない）を追記済み。</t>
+        </is>
+      </c>
+      <c r="N101" s="7" t="inlineStr"/>
+      <c r="O101" s="7" t="inlineStr"/>
+      <c r="P101" s="7" t="inlineStr"/>
+    </row>
+    <row r="102" ht="40" customHeight="1">
+      <c r="A102" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-102</t>
+        </is>
+      </c>
+      <c r="B102" s="6" t="inlineStr">
+        <is>
+          <t>アクティベーションゾーン標高差の設定可能項目化</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>AZ Flood Fill の標高差閾値 25m がハードコードされていた。プロミネンス最終フィルタと同様に設定可能項目としてデータ辞書（SRS 2.2.1）で管理するべきとのユーザー指摘。</t>
+        </is>
+      </c>
+      <c r="D102" s="6" t="inlineStr">
+        <is>
+          <t>機能追加</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F102" s="6" t="inlineStr"/>
+      <c r="G102" s="6" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H102" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="I102" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J102" s="6" t="inlineStr"/>
+      <c r="K102" s="6" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L102" s="6" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="M102" s="6" t="inlineStr">
+        <is>
+          <t>SRS 2.2.1 データ辞書に「アクティベーションゾーン標高差」を追加（デフォルト 25m・SOTA 規定値）。FR-016 の 25m 記述をデータ辞書参照化済み。GLOSSARY のアクティベーションゾーン定義にもデータ辞書リンクを追記済み。</t>
+        </is>
+      </c>
+      <c r="N102" s="6" t="inlineStr"/>
+      <c r="O102" s="6" t="inlineStr"/>
+      <c r="P102" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7580,7 +7766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7602,7 +7788,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3">
@@ -7612,7 +7798,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -7633,7 +7819,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>60.2%</t>
+          <t>58.4%</t>
         </is>
       </c>
     </row>
@@ -7672,7 +7858,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -7710,7 +7896,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16">
@@ -7720,7 +7906,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
@@ -7748,7 +7934,7 @@
         </is>
       </c>
       <c r="B20" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
@@ -7771,89 +7957,99 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>カテゴリ別（未解決）</t>
         </is>
       </c>
-      <c r="B24" s="9" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>解析エンジン</t>
-        </is>
-      </c>
-      <c r="B25" s="11" t="n">
-        <v>4</v>
-      </c>
+      <c r="B25" s="9" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>merge.py</t>
+          <t>解析エンジン</t>
         </is>
       </c>
       <c r="B26" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>GeoJSON出力</t>
+          <t>merge.py</t>
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
+          <t>GeoJSON出力</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
           <t>その他</t>
         </is>
       </c>
-      <c r="B28" s="11" t="n">
+      <c r="B29" s="11" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>ステージ別（未解決）</t>
         </is>
       </c>
-      <c r="B30" s="9" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="10" t="inlineStr">
-        <is>
-          <t>SRS</t>
-        </is>
-      </c>
-      <c r="B31" s="11" t="n">
-        <v>20</v>
-      </c>
+      <c r="B31" s="9" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>HLD</t>
+          <t>SRS</t>
         </is>
       </c>
       <c r="B32" s="11" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
+          <t>HLD</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
           <t>COD</t>
         </is>
       </c>
-      <c r="B33" s="11" t="n">
+      <c r="B34" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8690,7 +8886,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C51" t="n">
         <v>62</v>

</xml_diff>

<commit_message>
chore: tracker export update（ISSUE-114/115登録・対応完了）
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P113"/>
+  <dimension ref="A1:P115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8500,21 +8500,161 @@
       <c r="O113" s="7" t="inlineStr"/>
       <c r="P113" s="7" t="inlineStr"/>
     </row>
+    <row r="114" ht="40" customHeight="1">
+      <c r="A114" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-114</t>
+        </is>
+      </c>
+      <c r="B114" s="6" t="inlineStr">
+        <is>
+          <t>FR-009中心成果物GeoJSONのリネーム・和名整理（merged.geojson → merged_summit.geojson）</t>
+        </is>
+      </c>
+      <c r="C114" s="6" t="inlineStr">
+        <is>
+          <t>FR-009の中心成果物merged.geojsonの和名「統合ピーク候補」が中間ファイルmerged_peak.geojson（和名「統合ピーク候補 GeoJSON」）と重複しており、FR-009の概念（ピーク中心→サミット中心の節目）とも乖離。ファイル名をmerged_summit.geojsonへ変更し、和名を「突合済み統合 GeoJSON」へ整理する。</t>
+        </is>
+      </c>
+      <c r="D114" s="6" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E114" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F114" s="6" t="inlineStr">
+        <is>
+          <t>GeoJSON出力</t>
+        </is>
+      </c>
+      <c r="G114" s="6" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H114" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I114" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J114" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="K114" s="6" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L114" s="6" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="M114" s="6" t="inlineStr">
+        <is>
+          <t>ファイル名をmerged_summit.geojsonに変更（merged_summit.xlsxとペア）。和名を「突合済み統合 GeoJSON」に統一。ADR-SRS-030作成・SRS本文反映・関連ADR整合更新で対応。</t>
+        </is>
+      </c>
+      <c r="N114" s="6" t="inlineStr"/>
+      <c r="O114" s="6" t="inlineStr"/>
+      <c r="P114" s="6" t="inlineStr"/>
+    </row>
+    <row r="115" ht="40" customHeight="1">
+      <c r="A115" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-115</t>
+        </is>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>仮サミットコード連番上限の設定可能化・00始まり化（A99固定 → 設定項目化）</t>
+        </is>
+      </c>
+      <c r="C115" s="7" t="inlineStr">
+        <is>
+          <t>仮サミットコードの連番上限がA99固定のため、初年度に1エリア100件超となる可能性がある。上限を2.2.1設定可能項目へ追加し運用年度で切り替えられるようにする。あわせて連番を00始まりへ変更（A00〜A99で1prefix100件）。</t>
+        </is>
+      </c>
+      <c r="D115" s="7" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E115" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F115" s="7" t="inlineStr">
+        <is>
+          <t>設定</t>
+        </is>
+      </c>
+      <c r="G115" s="7" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H115" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I115" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J115" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="K115" s="7" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L115" s="7" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="M115" s="7" t="inlineStr">
+        <is>
+          <t>2.2.1設定可能項目に「仮サミットコード連番上限」を追加（デフォルトA・許容A〜Z）。連番を01始まり→00始まりへ変更。フォーマット例をA01→A00へ全更新。ADR-SRS-031作成・SRS本文反映で対応。</t>
+        </is>
+      </c>
+      <c r="N115" s="7" t="inlineStr"/>
+      <c r="O115" s="7" t="inlineStr"/>
+      <c r="P115" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K115" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E115" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D115" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"機能追加,改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I115" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J115" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8528,7 +8668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8550,7 +8690,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3">
@@ -8560,7 +8700,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
@@ -8581,7 +8721,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>59.8%</t>
+          <t>58.8%</t>
         </is>
       </c>
     </row>
@@ -8620,7 +8760,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -8668,7 +8808,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17">
@@ -8706,7 +8846,7 @@
         </is>
       </c>
       <c r="B21" s="11" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22">
@@ -8764,54 +8904,64 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
+          <t>設定</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
           <t>その他</t>
         </is>
       </c>
-      <c r="B29" s="11" t="n">
+      <c r="B30" s="11" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>ステージ別（未解決）</t>
         </is>
       </c>
-      <c r="B31" s="9" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>SRS</t>
-        </is>
-      </c>
-      <c r="B32" s="11" t="n">
-        <v>26</v>
-      </c>
+      <c r="B32" s="9" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>HLD</t>
+          <t>SRS</t>
         </is>
       </c>
       <c r="B33" s="11" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
+          <t>HLD</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
           <t>COD</t>
         </is>
       </c>
-      <c r="B34" s="11" t="n">
+      <c r="B35" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9696,7 +9846,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C54" t="n">
         <v>73</v>

</xml_diff>

<commit_message>
docs(tracker): spec-panel FR-013 レビュー指摘を登録（issue6件＋todo3件）
- ISSUE-121〜126 を登録（merged_summit.geojson スキーマ正本のFR-009移設・
  FR-013↔FR-019役割境界・metadataキー重複・area_complete死に仕様・
  prominence値未規定・dominant複数削除候補の対応識別）
- todo.md に文言修正3件追記（summit_name_jp取得元・feature_type用語ゆれ・概要明記）
- spec-panel FR-013 の指摘10（summitslist_date UTC表記）は取り下げ

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P120"/>
+  <dimension ref="A1:P126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8982,21 +8982,393 @@
       <c r="O120" s="6" t="inlineStr"/>
       <c r="P120" s="6" t="inlineStr"/>
     </row>
+    <row r="121" ht="40" customHeight="1">
+      <c r="A121" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-121</t>
+        </is>
+      </c>
+      <c r="B121" s="7" t="inlineStr">
+        <is>
+          <t>merged_summit.geojson スキーマ正本を生成者 FR-009 へ移設（消費者 FR-013 から）</t>
+        </is>
+      </c>
+      <c r="C121" s="7" t="inlineStr">
+        <is>
+          <t>merged_summit.geojson のフィーチャ構成・プロパティスキーマ正本が消費者である FR-013(SRS L959-1045) に定義されている。生成者は FR-009(L848・L917)。スキーマを消費側に置くと FR-009 との乖離リスクが構造的に残り、metadata/プロパティ記述が FR-013/FR-019/FR-009 で部分重複する温床になっている（指摘2-4の根因）。</t>
+        </is>
+      </c>
+      <c r="D121" s="7" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F121" s="7" t="inlineStr">
+        <is>
+          <t>GeoJSON出力</t>
+        </is>
+      </c>
+      <c r="G121" s="7" t="inlineStr">
+        <is>
+          <t>Opus</t>
+        </is>
+      </c>
+      <c r="H121" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="I121" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J121" s="7" t="inlineStr"/>
+      <c r="K121" s="7" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L121" s="7" t="inlineStr"/>
+      <c r="M121" s="7" t="inlineStr">
+        <is>
+          <t>スキーマ正本を FR-009（または 7.2 内部データ）へ移設し、FR-013/FR-019 は参照に統一する。</t>
+        </is>
+      </c>
+      <c r="N121" s="7" t="inlineStr"/>
+      <c r="O121" s="7" t="inlineStr"/>
+      <c r="P121" s="7" t="inlineStr"/>
+    </row>
+    <row r="122" ht="40" customHeight="1">
+      <c r="A122" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-122</t>
+        </is>
+      </c>
+      <c r="B122" s="6" t="inlineStr">
+        <is>
+          <t>FR-013↔FR-019 の役割境界整理（生成機構の記述位置）</t>
+        </is>
+      </c>
+      <c r="C122" s="6" t="inlineStr">
+        <is>
+          <t>FR-013 は『生成』と銘打つが、生成機構（テンプレート同梱・JS変数埋め込み・出力パス merged_viewer.html）の記述が FR-019(L1099-1100) 側にある。FR-013(L938)↔FR-019 の役割境界が曖昧。</t>
+        </is>
+      </c>
+      <c r="D122" s="6" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F122" s="6" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G122" s="6" t="inlineStr">
+        <is>
+          <t>Opus</t>
+        </is>
+      </c>
+      <c r="H122" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="I122" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J122" s="6" t="inlineStr"/>
+      <c r="K122" s="6" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L122" s="6" t="inlineStr"/>
+      <c r="M122" s="6" t="inlineStr">
+        <is>
+          <t>生成手順=FR-013、ブラウザ提供機能=FR-019 に責務を整理する。</t>
+        </is>
+      </c>
+      <c r="N122" s="6" t="inlineStr"/>
+      <c r="O122" s="6" t="inlineStr"/>
+      <c r="P122" s="6" t="inlineStr"/>
+    </row>
+    <row r="123" ht="40" customHeight="1">
+      <c r="A123" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-123</t>
+        </is>
+      </c>
+      <c r="B123" s="7" t="inlineStr">
+        <is>
+          <t>viewer 使用 metadata キー列挙の重複・不一致を集約（FR-013/FR-019）</t>
+        </is>
+      </c>
+      <c r="C123" s="7" t="inlineStr">
+        <is>
+          <t>viewer が使う metadata キー列挙が FR-013(L954-958, 6件) と FR-019(L1123-1126, 表示用3件) で重複かつ内容不一致。</t>
+        </is>
+      </c>
+      <c r="D123" s="7" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E123" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F123" s="7" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G123" s="7" t="inlineStr">
+        <is>
+          <t>Opus</t>
+        </is>
+      </c>
+      <c r="H123" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="I123" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J123" s="7" t="inlineStr"/>
+      <c r="K123" s="7" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L123" s="7" t="inlineStr"/>
+      <c r="M123" s="7" t="inlineStr">
+        <is>
+          <t>一方へ集約し他方は参照にする。</t>
+        </is>
+      </c>
+      <c r="N123" s="7" t="inlineStr"/>
+      <c r="O123" s="7" t="inlineStr"/>
+      <c r="P123" s="7" t="inlineStr"/>
+    </row>
+    <row r="124" ht="40" customHeight="1">
+      <c r="A124" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-124</t>
+        </is>
+      </c>
+      <c r="B124" s="6" t="inlineStr">
+        <is>
+          <t>AZ area_complete=false の死に仕様を明確化（viewer 到達データでは常に true）</t>
+        </is>
+      </c>
+      <c r="C124" s="6" t="inlineStr">
+        <is>
+          <t>FR-013(L1016) は AZ プロパティ area_complete を true/false 両値で定義するが、FR-019(L1108) は area_complete=false が上流(FR-009 is_area_incomplete)停止で viewer 非到達とする。viewer 到達 merged_summit.geojson では常に true で false 記述が死に仕様。</t>
+        </is>
+      </c>
+      <c r="D124" s="6" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E124" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F124" s="6" t="inlineStr">
+        <is>
+          <t>GeoJSON出力</t>
+        </is>
+      </c>
+      <c r="G124" s="6" t="inlineStr">
+        <is>
+          <t>Opus</t>
+        </is>
+      </c>
+      <c r="H124" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="I124" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J124" s="6" t="inlineStr"/>
+      <c r="K124" s="6" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L124" s="6" t="inlineStr"/>
+      <c r="M124" s="6" t="inlineStr">
+        <is>
+          <t>merged_summit.geojson 文脈では常に true である旨を注記、または中間データ専用と明確化する。</t>
+        </is>
+      </c>
+      <c r="N124" s="6" t="inlineStr"/>
+      <c r="O124" s="6" t="inlineStr"/>
+      <c r="P124" s="6" t="inlineStr"/>
+    </row>
+    <row r="125" ht="40" customHeight="1">
+      <c r="A125" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-125</t>
+        </is>
+      </c>
+      <c r="B125" s="7" t="inlineStr">
+        <is>
+          <t>key_col_resolved=false ピークの prominence プロパティ値表現を規定</t>
+        </is>
+      </c>
+      <c r="C125" s="7" t="inlineStr">
+        <is>
+          <t>key_col_resolved=false のピークでは col Point と prominence_range LineString は『含めない』と明記される(SRS L988・L1030)が、peak Point の prominence プロパティ値（空文字/センチネル/省略）の表現が未規定(L979)。FR-019(L1132) は表示『未定義』とするが GeoJSON 値が未定義。</t>
+        </is>
+      </c>
+      <c r="D125" s="7" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E125" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F125" s="7" t="inlineStr">
+        <is>
+          <t>GeoJSON出力</t>
+        </is>
+      </c>
+      <c r="G125" s="7" t="inlineStr">
+        <is>
+          <t>Opus</t>
+        </is>
+      </c>
+      <c r="H125" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="I125" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J125" s="7" t="inlineStr"/>
+      <c r="K125" s="7" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L125" s="7" t="inlineStr"/>
+      <c r="M125" s="7" t="inlineStr">
+        <is>
+          <t>未確定時の prominence 値の表現（空文字/省略 等）を SRS に規定する。</t>
+        </is>
+      </c>
+      <c r="N125" s="7" t="inlineStr"/>
+      <c r="O125" s="7" t="inlineStr"/>
+      <c r="P125" s="7" t="inlineStr"/>
+    </row>
+    <row r="126" ht="40" customHeight="1">
+      <c r="A126" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-126</t>
+        </is>
+      </c>
+      <c r="B126" s="6" t="inlineStr">
+        <is>
+          <t>dominant 複数削除候補の対応識別（coord_diff/summit の相手コードプロパティ）</t>
+        </is>
+      </c>
+      <c r="C126" s="6" t="inlineStr">
+        <is>
+          <t>dominant ピークの勢力圏に削除候補サミットが複数入る場合、ピーク→SOTAサミット線(coord_diff)が複数本でき全て同じ summit_code(ピーク仮コード)を持つため、どの線がどの削除候補に対応するかプロパティで判別不可（幾何のみ）。既存サミット点側にも親 dominant ピークを示すプロパティがない(SRS L965・L1037-1045)。実害は限定的（地図描画は幾何で成立）。</t>
+        </is>
+      </c>
+      <c r="D126" s="6" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E126" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F126" s="6" t="inlineStr">
+        <is>
+          <t>GeoJSON出力</t>
+        </is>
+      </c>
+      <c r="G126" s="6" t="inlineStr">
+        <is>
+          <t>Opus</t>
+        </is>
+      </c>
+      <c r="H126" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="I126" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J126" s="6" t="inlineStr"/>
+      <c r="K126" s="6" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L126" s="6" t="inlineStr"/>
+      <c r="M126" s="6" t="inlineStr">
+        <is>
+          <t>推奨方向（非拘束）: 対応づけを summit_code で明示する既存方針に整合させ、線に相手サミットのSOTAコード、サミット点に親ピーク仮コードを新プロパティとして追加。ただし新プロパティ名・付与範囲・FR-009生成ロジック/FR-019(相互ジャンプ)/FR-012/FR-021 への波及を確認のうえ本issue着手時に決定（今は決めない）。必要なら ADR 化。</t>
+        </is>
+      </c>
+      <c r="N126" s="6" t="inlineStr"/>
+      <c r="O126" s="6" t="inlineStr"/>
+      <c r="P126" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K120" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E120" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D120" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I120" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J120" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9032,7 +9404,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3">
@@ -9042,7 +9414,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4">
@@ -9063,7 +9435,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>56.3%</t>
+          <t>53.6%</t>
         </is>
       </c>
     </row>
@@ -9082,7 +9454,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9">
@@ -9140,7 +9512,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16">
@@ -9150,7 +9522,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17">
@@ -9178,7 +9550,7 @@
         </is>
       </c>
       <c r="B20" s="11" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21">
@@ -9198,7 +9570,7 @@
         </is>
       </c>
       <c r="B22" s="11" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24">
@@ -9236,7 +9608,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28">
@@ -9266,7 +9638,7 @@
         </is>
       </c>
       <c r="B30" s="11" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32">
@@ -9284,7 +9656,7 @@
         </is>
       </c>
       <c r="B33" s="11" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="34">
@@ -10236,7 +10608,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="C57" t="n">
         <v>79</v>

</xml_diff>

<commit_message>
docs(srs): FR-013レビュー由来 ISSUE-121〜126 + todo3件を SRS へ反映
- ISSUE-121: merged_summit.geojson スキーマ正本を FR-013 から生成者 FR-009 へ移設
  フィーチャ構成（match_status別）と各フィーチャのプロパティ全表を FR-009 末尾に移動。
  FR-013 は「スキーマ正本は FR-009 参照」に置換。6.6 のフィーチャ構成参照も更新。
- ISSUE-122: 生成機構（テンプレート同梱・JS変数埋め込み）の記述を FR-019 → FR-013 へ移動。
  FR-019 は「FR-013 が生成した HTML をブラウザで開いた際の機能を定義」に集約。
- ISSUE-123: metadata キー列挙の重複解消。FR-013 の6キーリストを削除し FR-009 参照に。
  viewer 表示キー一覧は FR-019 側に一本化。
- ISSUE-124: area_complete=false の位置付け明確化。FR-009 プロパティ表に「不備ゲートが
  false を検査するため両値に意味を持つ。viewer 到達時は常に true」を注記。死に仕様ではない。
- ISSUE-125: key_col_resolved=false 時の prominence を null と確定。スキーマに明記。
- ISSUE-126: dominant 複数削除候補の対応識別は幾何（終点座標）で成立。個別識別プロパティは
  追加しない。coord_diff 表の後に方針を明記。
- TODO 1: summit_name_jp 取得元を「本FR が geojson_v{N} から取得し格納」に修正（FR-009内3箇所）
- TODO 2: FR-019 のマーカー形状説明の `col=▼` → `key_col=▼`、popup見出しも統一。
- TODO 3: FR-013 概要に「作業用ビューアのみ生成。公開用は FR-020 が別途生成」を明記。

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -279,12 +279,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$57</f>
+              <f>'収束グラフ'!$A$2:$A$58</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$B$2:$B$57</f>
+              <f>'収束グラフ'!$B$2:$B$58</f>
             </numRef>
           </val>
         </ser>
@@ -314,12 +314,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$57</f>
+              <f>'収束グラフ'!$A$2:$A$58</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$C$2:$C$57</f>
+              <f>'収束グラフ'!$C$2:$C$58</f>
             </numRef>
           </val>
         </ser>
@@ -349,12 +349,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$57</f>
+              <f>'収束グラフ'!$A$2:$A$58</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$D$2:$D$57</f>
+              <f>'収束グラフ'!$D$2:$D$58</f>
             </numRef>
           </val>
         </ser>
@@ -9031,7 +9031,7 @@
       <c r="J121" s="7" t="inlineStr"/>
       <c r="K121" s="7" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="L121" s="7" t="inlineStr"/>
@@ -9041,7 +9041,11 @@
         </is>
       </c>
       <c r="N121" s="7" t="inlineStr"/>
-      <c r="O121" s="7" t="inlineStr"/>
+      <c r="O121" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
       <c r="P121" s="7" t="inlineStr"/>
     </row>
     <row r="122" ht="40" customHeight="1">
@@ -9093,7 +9097,7 @@
       <c r="J122" s="6" t="inlineStr"/>
       <c r="K122" s="6" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="L122" s="6" t="inlineStr"/>
@@ -9103,7 +9107,11 @@
         </is>
       </c>
       <c r="N122" s="6" t="inlineStr"/>
-      <c r="O122" s="6" t="inlineStr"/>
+      <c r="O122" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
       <c r="P122" s="6" t="inlineStr"/>
     </row>
     <row r="123" ht="40" customHeight="1">
@@ -9155,7 +9163,7 @@
       <c r="J123" s="7" t="inlineStr"/>
       <c r="K123" s="7" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="L123" s="7" t="inlineStr"/>
@@ -9165,7 +9173,11 @@
         </is>
       </c>
       <c r="N123" s="7" t="inlineStr"/>
-      <c r="O123" s="7" t="inlineStr"/>
+      <c r="O123" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
       <c r="P123" s="7" t="inlineStr"/>
     </row>
     <row r="124" ht="40" customHeight="1">
@@ -9217,7 +9229,7 @@
       <c r="J124" s="6" t="inlineStr"/>
       <c r="K124" s="6" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="L124" s="6" t="inlineStr"/>
@@ -9227,7 +9239,11 @@
         </is>
       </c>
       <c r="N124" s="6" t="inlineStr"/>
-      <c r="O124" s="6" t="inlineStr"/>
+      <c r="O124" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
       <c r="P124" s="6" t="inlineStr"/>
     </row>
     <row r="125" ht="40" customHeight="1">
@@ -9279,7 +9295,7 @@
       <c r="J125" s="7" t="inlineStr"/>
       <c r="K125" s="7" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="L125" s="7" t="inlineStr"/>
@@ -9289,7 +9305,11 @@
         </is>
       </c>
       <c r="N125" s="7" t="inlineStr"/>
-      <c r="O125" s="7" t="inlineStr"/>
+      <c r="O125" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
       <c r="P125" s="7" t="inlineStr"/>
     </row>
     <row r="126" ht="40" customHeight="1">
@@ -9341,7 +9361,7 @@
       <c r="J126" s="6" t="inlineStr"/>
       <c r="K126" s="6" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="L126" s="6" t="inlineStr"/>
@@ -9351,7 +9371,11 @@
         </is>
       </c>
       <c r="N126" s="6" t="inlineStr"/>
-      <c r="O126" s="6" t="inlineStr"/>
+      <c r="O126" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
       <c r="P126" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -9454,7 +9478,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -9474,7 +9498,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
@@ -9690,7 +9714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10617,6 +10641,22 @@
         <v>84</v>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>125</v>
+      </c>
+      <c r="C58" t="n">
+        <v>85</v>
+      </c>
+      <c r="D58" t="n">
+        <v>84</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
chore(tracker): ISSUE-127〜130 登録・クローズを Excel に反映
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -279,12 +279,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$59</f>
+              <f>'収束グラフ'!$A$2:$A$61</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$B$2:$B$59</f>
+              <f>'収束グラフ'!$B$2:$B$61</f>
             </numRef>
           </val>
         </ser>
@@ -314,12 +314,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$59</f>
+              <f>'収束グラフ'!$A$2:$A$61</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$C$2:$C$59</f>
+              <f>'収束グラフ'!$C$2:$C$61</f>
             </numRef>
           </val>
         </ser>
@@ -349,12 +349,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$59</f>
+              <f>'収束グラフ'!$A$2:$A$61</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$D$2:$D$59</f>
+              <f>'収束グラフ'!$D$2:$D$61</f>
             </numRef>
           </val>
         </ser>
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P126"/>
+  <dimension ref="A1:P130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9458,21 +9458,285 @@
         </is>
       </c>
     </row>
+    <row r="127" ht="40" customHeight="1">
+      <c r="A127" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-127</t>
+        </is>
+      </c>
+      <c r="B127" s="7" t="inlineStr">
+        <is>
+          <t>FR-020 公開用HTMLに UR-011 帰属表示を反映</t>
+        </is>
+      </c>
+      <c r="C127" s="7" t="inlineStr">
+        <is>
+          <t>公開用HTML(FR-020)は唯一の外部公開成果物だが対応URがUR-006のみで、6.13にattribution記載が無い。FR-019の帰属表示は作業用ビューア向けで別テンプレートの公開用に引き継がれる保証が無い。</t>
+        </is>
+      </c>
+      <c r="D127" s="7" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F127" s="7" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G127" s="7" t="inlineStr">
+        <is>
+          <t>Opus</t>
+        </is>
+      </c>
+      <c r="H127" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="I127" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J127" s="7" t="inlineStr"/>
+      <c r="K127" s="7" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L127" s="7" t="inlineStr"/>
+      <c r="M127" s="7" t="inlineStr">
+        <is>
+          <t>FR-020対応URにUR-011追加。6.13にattribution行(© 国土地理院常時＋OSM/OpenTopoMap各表示＋『加工して作成』)明記。UR紐付けのADR要否を判断。</t>
+        </is>
+      </c>
+      <c r="N127" s="7" t="inlineStr"/>
+      <c r="O127" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="P127" s="7" t="inlineStr"/>
+    </row>
+    <row r="128" ht="40" customHeight="1">
+      <c r="A128" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-128</t>
+        </is>
+      </c>
+      <c r="B128" s="6" t="inlineStr">
+        <is>
+          <t>公開用HTMLの提供機能・公開情報範囲の定義</t>
+        </is>
+      </c>
+      <c r="C128" s="6" t="inlineStr">
+        <is>
+          <t>公開用は除外項目(編集UI/XLSX/localStorage)のみ明示で、FR-019の閲覧系機能(背景切替/検索/フィルター/各レイヤー/全データpopup/相互ジャンプ/metadata基準日表示)のどれを含めるか未定義。全データpopupでの内部フラグ・仮コードの外部露出可否も未決(要1論点ずつ相談)。</t>
+        </is>
+      </c>
+      <c r="D128" s="6" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F128" s="6" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G128" s="6" t="inlineStr">
+        <is>
+          <t>Opus</t>
+        </is>
+      </c>
+      <c r="H128" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="I128" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J128" s="6" t="inlineStr"/>
+      <c r="K128" s="6" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L128" s="6" t="inlineStr"/>
+      <c r="M128" s="6" t="inlineStr">
+        <is>
+          <t>公開用に含める閲覧機能の包含規則をFR-020/6.13に明記。内部値露出ポリシー・metadata基準日表示の要否を順に確定(露出判断はADR候補)。</t>
+        </is>
+      </c>
+      <c r="N128" s="6" t="inlineStr"/>
+      <c r="O128" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="P128" s="6" t="inlineStr"/>
+    </row>
+    <row r="129" ht="40" customHeight="1">
+      <c r="A129" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-129</t>
+        </is>
+      </c>
+      <c r="B129" s="7" t="inlineStr">
+        <is>
+          <t>公開用エクスポート時の localStorage マージ仕様の明確化</t>
+        </is>
+      </c>
+      <c r="C129" s="7" t="inlineStr">
+        <is>
+          <t>FR-020はlocalStorageをマージするとあるが、generated_at不一致(前回実行分)時にどの状態(現在のビューア表示状態 vs localStorage生データ)をマージするか未定義。</t>
+        </is>
+      </c>
+      <c r="D129" s="7" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E129" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F129" s="7" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G129" s="7" t="inlineStr">
+        <is>
+          <t>Opus</t>
+        </is>
+      </c>
+      <c r="H129" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="I129" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J129" s="7" t="inlineStr"/>
+      <c r="K129" s="7" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L129" s="7" t="inlineStr"/>
+      <c r="M129" s="7" t="inlineStr">
+        <is>
+          <t>マージ元を『現在のビューア表示状態のスナップショット』と明記する。</t>
+        </is>
+      </c>
+      <c r="N129" s="7" t="inlineStr"/>
+      <c r="O129" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="P129" s="7" t="inlineStr"/>
+    </row>
+    <row r="130" ht="40" customHeight="1">
+      <c r="A130" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-130</t>
+        </is>
+      </c>
+      <c r="B130" s="6" t="inlineStr">
+        <is>
+          <t>公開用 別テンプレート採用の設計判断記録(ADR要否)</t>
+        </is>
+      </c>
+      <c r="C130" s="6" t="inlineStr">
+        <is>
+          <t>作業用テンプレートを条件分岐させず別ファイルにする設計判断の根拠が未記録。HLDで扱うかADR-SRS化するか未定。</t>
+        </is>
+      </c>
+      <c r="D130" s="6" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E130" s="5" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="F130" s="6" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G130" s="6" t="inlineStr">
+        <is>
+          <t>Opus</t>
+        </is>
+      </c>
+      <c r="H130" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="I130" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J130" s="6" t="inlineStr"/>
+      <c r="K130" s="6" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L130" s="6" t="inlineStr"/>
+      <c r="M130" s="6" t="inlineStr">
+        <is>
+          <t>HLD所掌か ADR-SRS 化かを判断し、ADR化なら作成。</t>
+        </is>
+      </c>
+      <c r="N130" s="6" t="inlineStr"/>
+      <c r="O130" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="P130" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9508,7 +9772,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3">
@@ -9518,7 +9782,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -9539,7 +9803,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>69.6%</t>
+          <t>67.4%</t>
         </is>
       </c>
     </row>
@@ -9578,7 +9842,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -9616,7 +9880,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16">
@@ -9626,7 +9890,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
@@ -9636,7 +9900,7 @@
         </is>
       </c>
       <c r="B17" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
@@ -9654,7 +9918,7 @@
         </is>
       </c>
       <c r="B20" s="11" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21">
@@ -9674,7 +9938,7 @@
         </is>
       </c>
       <c r="B22" s="11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24">
@@ -9722,7 +9986,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="30">
@@ -9740,7 +10004,7 @@
         </is>
       </c>
       <c r="B31" s="11" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="32">
@@ -9774,7 +10038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10733,6 +10997,38 @@
         <v>104</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>125</v>
+      </c>
+      <c r="C60" t="n">
+        <v>85</v>
+      </c>
+      <c r="D60" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>129</v>
+      </c>
+      <c r="C61" t="n">
+        <v>89</v>
+      </c>
+      <c r="D61" t="n">
+        <v>104</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
chore(tracker): ISSUE-135 登録・対応完了（unmatched 要確認扱い）
unmatched サミットの要確認扱い変更（ADR-SRS-037）を ISSUE-135 として登録し、
SRS/ADR 反映完了に伴い対応完了。plan.md・Excel エクスポートを同期。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -279,12 +279,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$62</f>
+              <f>'収束グラフ'!$A$2:$A$63</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$B$2:$B$62</f>
+              <f>'収束グラフ'!$B$2:$B$63</f>
             </numRef>
           </val>
         </ser>
@@ -314,12 +314,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$62</f>
+              <f>'収束グラフ'!$A$2:$A$63</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$C$2:$C$62</f>
+              <f>'収束グラフ'!$C$2:$C$63</f>
             </numRef>
           </val>
         </ser>
@@ -349,12 +349,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$62</f>
+              <f>'収束グラフ'!$A$2:$A$63</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$D$2:$D$62</f>
+              <f>'収束グラフ'!$D$2:$D$63</f>
             </numRef>
           </val>
         </ser>
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P134"/>
+  <dimension ref="A1:P135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9986,21 +9986,91 @@
       </c>
       <c r="P134" s="6" t="inlineStr"/>
     </row>
+    <row r="135" ht="40" customHeight="1">
+      <c r="A135" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-135</t>
+        </is>
+      </c>
+      <c r="B135" s="7" t="inlineStr">
+        <is>
+          <t>地形変化で消滅したサミット（unmatched）の要確認扱い・FR-009 即停止の見直し</t>
+        </is>
+      </c>
+      <c r="C135" s="7" t="inlineStr">
+        <is>
+          <t>現行 FR-009 / ADR-SRS-011 は、既存 SOTA サミットが AZ・delete判定ゾーンのいずれにも入らない場合を summit.match_status=unmatched とし『閾値不備または解析欠落』とみなして処理停止する。しかし噴火・山体崩壊・カルデラ陥没で山が実際に消えた場合、旧サミット座標がどのゾーンにも入らず unmatched になりうる。これはシステム不備ではなく正当な地形変化＝削除候補であり、即停止設計は実態を捉えていない盲点。座標だけでは地形変化と解析不備を機械区別できないため自動削除は誤削除リスクがある。</t>
+        </is>
+      </c>
+      <c r="D135" s="7" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E135" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F135" s="7" t="inlineStr">
+        <is>
+          <t>merge.py</t>
+        </is>
+      </c>
+      <c r="G135" s="7" t="inlineStr">
+        <is>
+          <t>Opus</t>
+        </is>
+      </c>
+      <c r="H135" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="I135" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J135" s="7" t="inlineStr"/>
+      <c r="K135" s="7" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L135" s="7" t="inlineStr"/>
+      <c r="M135" s="7" t="inlineStr">
+        <is>
+          <t>新規 ADR-SRS-037 を作成し以下を確定: (1) unmatched を『要確認』状態として続行扱い（停止トリガーから外す）。申請書の削除行には自動掲載せず merged_summit.xlsx・HTMLビューアのカテゴリで担当者に提示。(2) 件数しきい値（config.ini）で解析バグを防御。少数は続行、しきい値超過は解析異常の疑いで停止。(3) is_area_incomplete / is_key_col_unresolved は従来どおり停止維持。影響文書を同期更新（ADR-SRS-011 / ADR-URD-007 / 20_SRS FR-009・データ辞書 / ADR-SRS-033 / ADR-SRS-035 / GLOSSARY）。</t>
+        </is>
+      </c>
+      <c r="N135" s="7" t="inlineStr">
+        <is>
+          <t>ユーザー確認済み: 要確認続行＋件数しきい値停止。成果物はSRS/ADR文書のみ（ADR-SRS-011 が採用・未実装のためコード変更なし）。</t>
+        </is>
+      </c>
+      <c r="O135" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="P135" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K135" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E135" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D135" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I135" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J135" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10036,7 +10106,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3">
@@ -10046,7 +10116,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
@@ -10067,7 +10137,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>65.4%</t>
+          <t>64.9%</t>
         </is>
       </c>
     </row>
@@ -10106,7 +10176,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -10144,7 +10214,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16">
@@ -10202,7 +10272,7 @@
         </is>
       </c>
       <c r="B22" s="11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24">
@@ -10230,7 +10300,7 @@
         </is>
       </c>
       <c r="B26" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
@@ -10268,7 +10338,7 @@
         </is>
       </c>
       <c r="B31" s="11" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32">
@@ -10302,7 +10372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11309,6 +11379,22 @@
         <v>104</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>134</v>
+      </c>
+      <c r="C63" t="n">
+        <v>94</v>
+      </c>
+      <c r="D63" t="n">
+        <v>104</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
chore(tracker): issue report 最新エクスポート
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -744,7 +744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P139"/>
+  <dimension ref="A1:P143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10399,21 +10399,273 @@
         </is>
       </c>
     </row>
+    <row r="140" ht="40" customHeight="1">
+      <c r="A140" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-140</t>
+        </is>
+      </c>
+      <c r="B140" s="6" t="inlineStr">
+        <is>
+          <t>key_col_unresolved_peaks-N.csv のカラム定義（スキーマ）を FR-022 出力テーブル／§7.2.1 に追加</t>
+        </is>
+      </c>
+      <c r="C140" s="6" t="inlineStr">
+        <is>
+          <t>FR-022 の出力テーブルおよび §7.2.1 No.7 に key_col_unresolved_peaks-N.csv のカラム定義が存在しない。FR-014 入力備考に「key_col_resolved=false のピーク群・緯度経度」と略記されているだけで、公式のカラム一覧定義がない。per-mesh CSV（FR-007 出力参照リンク）・merged_peak.csv（FR-008）と同様の定義レベルが必要。</t>
+        </is>
+      </c>
+      <c r="D140" s="6" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E140" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F140" s="6" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G140" s="6" t="inlineStr"/>
+      <c r="H140" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I140" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J140" s="6" t="inlineStr"/>
+      <c r="K140" s="6" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L140" s="6" t="inlineStr"/>
+      <c r="M140" s="6" t="inlineStr">
+        <is>
+          <t>カラムを確定し（最低限 peak_lat, peak_lon。追加列があれば明示）、FR-022 出力テーブル備考欄か §7.2.2 に定義セクションを追加する。FR-014 入力備考欄も整合させる。</t>
+        </is>
+      </c>
+      <c r="N140" s="6" t="inlineStr"/>
+      <c r="O140" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P140" s="6" t="inlineStr"/>
+    </row>
+    <row r="141" ht="40" customHeight="1">
+      <c r="A141" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-141</t>
+        </is>
+      </c>
+      <c r="B141" s="7" t="inlineStr">
+        <is>
+          <t>FR-022 異常系定義の追加（入力 CSV 不存在・空ピーク時の挙動）</t>
+        </is>
+      </c>
+      <c r="C141" s="7" t="inlineStr">
+        <is>
+          <t>FR-022 に異常系定義がない。FR-014・FR-004 等は「異常系」セクションを持つが FR-022 には存在しない。「merged_peak.csv が存在しない場合」「CSV が空（0件ピーク）の場合」の挙動が未定義。空ピークの場合は「ゼロ件 = 全充足」として正常終了してフェーズ4へ進んでよいかの設計判断も必要。</t>
+        </is>
+      </c>
+      <c r="D141" s="7" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E141" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F141" s="7" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G141" s="7" t="inlineStr"/>
+      <c r="H141" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I141" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J141" s="7" t="inlineStr"/>
+      <c r="K141" s="7" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L141" s="7" t="inlineStr"/>
+      <c r="M141" s="7" t="inlineStr">
+        <is>
+          <t>FR-022 説明に「異常系」セクションを追加。「入力 CSV が存在しない場合はエラー終了（FR-023 に伝播）」「ピーク0件（空 CSV）の場合は「ゼロ」を返し正常終了（フェーズ4へ進む）」の方針を確定して記述する。</t>
+        </is>
+      </c>
+      <c r="N141" s="7" t="inlineStr"/>
+      <c r="O141" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P141" s="7" t="inlineStr"/>
+    </row>
+    <row r="142" ht="40" customHeight="1">
+      <c r="A142" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-142</t>
+        </is>
+      </c>
+      <c r="B142" s="6" t="inlineStr">
+        <is>
+          <t>FR-023 の下位 FR エラー時のエラー伝播方針を SRS に明記</t>
+        </is>
+      </c>
+      <c r="C142" s="6" t="inlineStr">
+        <is>
+          <t>FR-023 の説明に、下位 FR（FR-004・FR-014・FR-008・FR-018・FR-022 等）が異常終了した場合の挙動が記述されていない。シェルスクリプトとして即時終了（エラー伝播）するかどうかの方針が不明。スキップして継続する設計も考えられるが、フェイルファースト原則（lessons.md 参照）に照らせば即時終了が適切と推定される。</t>
+        </is>
+      </c>
+      <c r="D142" s="6" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E142" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F142" s="6" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G142" s="6" t="inlineStr"/>
+      <c r="H142" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I142" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J142" s="6" t="inlineStr"/>
+      <c r="K142" s="6" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L142" s="6" t="inlineStr"/>
+      <c r="M142" s="6" t="inlineStr">
+        <is>
+          <t>方針を確定し（推奨: 即時終了・エラー伝播）、FR-023 説明のループ終了条件周辺に「呼び出した FR がエラー終了した場合は FR-023 も即時終了する」旨を追記する。</t>
+        </is>
+      </c>
+      <c r="N142" s="6" t="inlineStr"/>
+      <c r="O142" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P142" s="6" t="inlineStr"/>
+    </row>
+    <row r="143" ht="40" customHeight="1">
+      <c r="A143" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-143</t>
+        </is>
+      </c>
+      <c r="B143" s="7" t="inlineStr">
+        <is>
+          <t>FR-020: NFR-010（描画応答性）スコープに公開用 HTML を含めるか確認・RTM 更新</t>
+        </is>
+      </c>
+      <c r="C143" s="7" t="inlineStr">
+        <is>
+          <t>spec-panel FR-020 レビュー指摘③。NFR-010（描画応答性・連続操作の滑らかさ）は「本 NFR は HTML ビューア（FR-013）のマーカー描画に適用する」と FR-013 のみに限定されている。公開用 HTML（FR-020）も同規模（最大1万件）のマーカーを表示するビューアであり、60fps の描画応答性要件が同様に適用されるべきかどうかを確認する必要がある。RTM でも FR-020 → UR-014 のマッピングが欠落している。</t>
+        </is>
+      </c>
+      <c r="D143" s="7" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E143" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F143" s="7" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G143" s="7" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H143" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I143" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J143" s="7" t="inlineStr"/>
+      <c r="K143" s="7" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L143" s="7" t="inlineStr"/>
+      <c r="M143" s="7" t="inlineStr">
+        <is>
+          <t>NFR-010 のスコープを FR-020 にも明示的に拡張する（「HTML ビューア（FR-013・FR-020）のマーカー描画に適用する」）か、FR-013 と同等の要件が FR-020 に引き継がれることを NFR-010 本文または ADR に明記するかを選択し、RTM の FR-020 行 UR-014 列に ✅ を追記する。</t>
+        </is>
+      </c>
+      <c r="N143" s="7" t="inlineStr"/>
+      <c r="O143" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P143" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10449,7 +10701,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3">
@@ -10459,7 +10711,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
@@ -10480,7 +10732,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>73.9%</t>
+          <t>71.8%</t>
         </is>
       </c>
     </row>
@@ -10519,7 +10771,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -10557,7 +10809,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
@@ -10567,7 +10819,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
@@ -10615,7 +10867,7 @@
         </is>
       </c>
       <c r="B22" s="11" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24">
@@ -10663,7 +10915,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30">
@@ -10681,7 +10933,7 @@
         </is>
       </c>
       <c r="B31" s="11" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="32">
@@ -11745,10 +11997,10 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C64" t="n">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D64" t="n">
         <v>119</v>

</xml_diff>

<commit_message>
chore(tracker): FR-017 spec-panel 指摘①〜⑧ を tracker・todo に登録
- ISSUE-144: FR-017 生成1（60地域GeoJSON）への北方領土ポリゴン含有の扱いを明示
- ISSUE-145: FR-017 生成1 dissolve の出力形状（MultiPolygon 可否）を明示
- ISSUE-146: FR-017 再実行条件（N03 ZIP 差し替え時）の SRS 記載 vs HLD 委任を判断
- todo: 指摘①③（高）・④（中）・⑦⑧（低）をtodo.mdに追加

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -744,7 +744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P143"/>
+  <dimension ref="A1:P146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10651,21 +10651,207 @@
       </c>
       <c r="P143" s="7" t="inlineStr"/>
     </row>
+    <row r="144" ht="40" customHeight="1">
+      <c r="A144" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-144</t>
+        </is>
+      </c>
+      <c r="B144" s="6" t="inlineStr">
+        <is>
+          <t>FR-017 生成1（60地域GeoJSON）への北方領土ポリゴン含有の扱いを明示</t>
+        </is>
+      </c>
+      <c r="C144" s="6" t="inlineStr">
+        <is>
+          <t>FR-017 §生成1（60地域GeoJSON）を作成する際、北方領土6村（N03_007: 01695〜01700）のポリゴンを dissolve 対象に含めるか除外するかが未定義。生成3（北方領土除外タイルリスト）は同コードを抽出して別途処理するが、生成1の dissolve 処理で除外するか残すかが記述されていない。含めたままにすると FR-009 でのエリアコード付与対象に北方領土のポリゴン範囲が残るが、北方領土のピーク候補は FR-001 タイル取得スキップにより解析結果に流れ込まない設計のため実害はない。ただし設計意図が読み取れない状態であり、実装者が迷う可能性がある。</t>
+        </is>
+      </c>
+      <c r="D144" s="6" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E144" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F144" s="6" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G144" s="6" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H144" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I144" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J144" s="6" t="inlineStr"/>
+      <c r="K144" s="6" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L144" s="6" t="inlineStr"/>
+      <c r="M144" s="6" t="inlineStr">
+        <is>
+          <t>「生成1では北方領土ポリゴンを dissolve 対象に含める（除外は生成3＋FR-001 で完結しているため重複除外は不要）」または「生成3と同一条件で生成1から除外する」どちらかを決定し、FR-017 §生成1 の説明文に明記する。</t>
+        </is>
+      </c>
+      <c r="N144" s="6" t="inlineStr"/>
+      <c r="O144" s="6" t="inlineStr"/>
+      <c r="P144" s="6" t="inlineStr"/>
+    </row>
+    <row r="145" ht="40" customHeight="1">
+      <c r="A145" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-145</t>
+        </is>
+      </c>
+      <c r="B145" s="7" t="inlineStr">
+        <is>
+          <t>FR-017 生成1 dissolve の出力形状（MultiPolygon 可否）を明示</t>
+        </is>
+      </c>
+      <c r="C145" s="7" t="inlineStr">
+        <is>
+          <t>FR-017 §生成1（行282）に「1地域1ポリゴンに集約」と記述されているが、沖縄・鹿児島等の離島は本島と隣接しないため dissolve の自然な結果は MultiPolygon になる。「1ポリゴン」が MultiPolygon 許容なのか厳密に単一 Polygon なのかが未定義。FR-009 での point-in-polygon 処理の実装時（GeoJSON ライブラリの扱い）に影響する。</t>
+        </is>
+      </c>
+      <c r="D145" s="7" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E145" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F145" s="7" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G145" s="7" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H145" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I145" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J145" s="7" t="inlineStr"/>
+      <c r="K145" s="7" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L145" s="7" t="inlineStr"/>
+      <c r="M145" s="7" t="inlineStr">
+        <is>
+          <t>「1フィーチャ（MultiPolygon 許容）に集約」として SRS の記述「1地域1ポリゴン」を「1地域1フィーチャ（MultiPolygon 許容）」に更新することを推奨する。離島を含む都府県は必然的に MultiPolygon になるため単一 Polygon への厳密化は現実的でない。</t>
+        </is>
+      </c>
+      <c r="N145" s="7" t="inlineStr"/>
+      <c r="O145" s="7" t="inlineStr"/>
+      <c r="P145" s="7" t="inlineStr"/>
+    </row>
+    <row r="146" ht="40" customHeight="1">
+      <c r="A146" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-146</t>
+        </is>
+      </c>
+      <c r="B146" s="6" t="inlineStr">
+        <is>
+          <t>FR-017 再実行条件（N03 ZIP 差し替え時）の SRS 記載 vs HLD 委任を判断</t>
+        </is>
+      </c>
+      <c r="C146" s="6" t="inlineStr">
+        <is>
+          <t>FR-017 §実行タイミング（行276）は「初回のみ。出力ファイル群が未生成の場合に起動する」と定義しているが、N03 ZIP を新年版に差し替えた場合の再実行手順が未定義。「出力ファイルを削除してから再実行する」という操作手順を SRS 段階で明記するか、HLD に完全委任するかを決める必要がある。</t>
+        </is>
+      </c>
+      <c r="D146" s="6" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E146" s="5" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="F146" s="6" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G146" s="6" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H146" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I146" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J146" s="6" t="inlineStr"/>
+      <c r="K146" s="6" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L146" s="6" t="inlineStr"/>
+      <c r="M146" s="6" t="inlineStr">
+        <is>
+          <t>SRS に「出力ファイルを手動削除することで再実行できる（詳細は HLD 参照）」程度の一文を追加する方向を推奨する。完全 HLD 委任とする場合は FR-017 §実行タイミングに『再実行はHLD参照』の一文を追記する。</t>
+        </is>
+      </c>
+      <c r="N146" s="6" t="inlineStr"/>
+      <c r="O146" s="6" t="inlineStr"/>
+      <c r="P146" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J143" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10701,7 +10887,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3">
@@ -10711,7 +10897,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4">
@@ -10732,7 +10918,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>71.8%</t>
+          <t>70.3%</t>
         </is>
       </c>
     </row>
@@ -10751,7 +10937,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
@@ -10819,7 +11005,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17">
@@ -10829,7 +11015,7 @@
         </is>
       </c>
       <c r="B17" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
@@ -10867,7 +11053,7 @@
         </is>
       </c>
       <c r="B22" s="11" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24">
@@ -10915,7 +11101,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30">
@@ -10933,7 +11119,7 @@
         </is>
       </c>
       <c r="B31" s="11" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="32">
@@ -11997,7 +12183,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C64" t="n">
         <v>123</v>

</xml_diff>

<commit_message>
docs(srs): FR-017 生成1 dissolve 出力形状を MultiPolygon 許容に明記（ISSUE-145）
「1地域1ポリゴンに集約」→「1地域1フィーチャ（Polygon または MultiPolygon）に集約」に修正。
離島を含む地域（東京・鹿児島・沖縄・北海道離島振興局等）は海峡で分断されるため
MultiPolygon になる旨を追記した。

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -10766,7 +10766,7 @@
       <c r="J145" s="7" t="inlineStr"/>
       <c r="K145" s="7" t="inlineStr">
         <is>
-          <t>未対応</t>
+          <t>対応完了</t>
         </is>
       </c>
       <c r="L145" s="7" t="inlineStr"/>
@@ -10776,7 +10776,11 @@
         </is>
       </c>
       <c r="N145" s="7" t="inlineStr"/>
-      <c r="O145" s="7" t="inlineStr"/>
+      <c r="O145" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
       <c r="P145" s="7" t="inlineStr"/>
     </row>
     <row r="146" ht="40" customHeight="1">
@@ -10941,7 +10945,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -10961,7 +10965,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -12190,7 +12194,7 @@
         <v>145</v>
       </c>
       <c r="C64" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D64" t="n">
         <v>119</v>

</xml_diff>

<commit_message>
chore(mgmt): FR-012 spec-panel レビュー 計画・issue 登録を記録
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -279,12 +279,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$64</f>
+              <f>'収束グラフ'!$A$2:$A$65</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$B$2:$B$64</f>
+              <f>'収束グラフ'!$B$2:$B$65</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -315,12 +315,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$64</f>
+              <f>'収束グラフ'!$A$2:$A$65</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$C$2:$C$64</f>
+              <f>'収束グラフ'!$C$2:$C$65</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -351,12 +351,12 @@
           </marker>
           <cat>
             <strRef>
-              <f>'収束グラフ'!$A$2:$A$64</f>
+              <f>'収束グラフ'!$A$2:$A$65</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'収束グラフ'!$D$2:$D$64</f>
+              <f>'収束グラフ'!$D$2:$D$65</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -744,7 +744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P146"/>
+  <dimension ref="A1:P158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10400,22 +10400,22 @@
       </c>
     </row>
     <row r="140" ht="40" customHeight="1">
-      <c r="A140" s="6" t="inlineStr">
+      <c r="A140" s="2" t="inlineStr">
         <is>
           <t>ISSUE-140</t>
         </is>
       </c>
-      <c r="B140" s="6" t="inlineStr">
+      <c r="B140" s="2" t="inlineStr">
         <is>
           <t>key_col_unresolved_peaks-N.csv のカラム定義（スキーマ）を FR-022 出力テーブル／§7.2.1 に追加</t>
         </is>
       </c>
-      <c r="C140" s="6" t="inlineStr">
+      <c r="C140" s="2" t="inlineStr">
         <is>
           <t>FR-022 の出力テーブルおよび §7.2.1 No.7 に key_col_unresolved_peaks-N.csv のカラム定義が存在しない。FR-014 入力備考に「key_col_resolved=false のピーク群・緯度経度」と略記されているだけで、公式のカラム一覧定義がない。per-mesh CSV（FR-007 出力参照リンク）・merged_peak.csv（FR-008）と同様の定義レベルが必要。</t>
         </is>
       </c>
-      <c r="D140" s="6" t="inlineStr">
+      <c r="D140" s="2" t="inlineStr">
         <is>
           <t>設計</t>
         </is>
@@ -10425,445 +10425,1241 @@
           <t>高</t>
         </is>
       </c>
-      <c r="F140" s="6" t="inlineStr">
+      <c r="F140" s="2" t="inlineStr">
         <is>
           <t>その他</t>
         </is>
       </c>
-      <c r="G140" s="6" t="inlineStr"/>
-      <c r="H140" s="6" t="inlineStr">
+      <c r="G140" s="2" t="inlineStr"/>
+      <c r="H140" s="2" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="I140" s="6" t="inlineStr">
-        <is>
-          <t>SRS</t>
-        </is>
-      </c>
-      <c r="J140" s="6" t="inlineStr"/>
-      <c r="K140" s="6" t="inlineStr">
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="inlineStr"/>
+      <c r="K140" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L140" s="2" t="inlineStr"/>
+      <c r="M140" s="2" t="inlineStr">
+        <is>
+          <t>カラムを確定し（最低限 peak_lat, peak_lon。追加列があれば明示）、FR-022 出力テーブル備考欄か §7.2.2 に定義セクションを追加する。FR-014 入力備考欄も整合させる。</t>
+        </is>
+      </c>
+      <c r="N140" s="2" t="inlineStr"/>
+      <c r="O140" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P140" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="40" customHeight="1">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-141</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>FR-022 異常系定義の追加（入力 CSV 不存在・空ピーク時の挙動）</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>FR-022 に異常系定義がない。FR-014・FR-004 等は「異常系」セクションを持つが FR-022 には存在しない。「merged_peak.csv が存在しない場合」「CSV が空（0件ピーク）の場合」の挙動が未定義。空ピークの場合は「ゼロ件 = 全充足」として正常終了してフェーズ4へ進んでよいかの設計判断も必要。</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E141" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr"/>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J141" s="2" t="inlineStr"/>
+      <c r="K141" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L141" s="2" t="inlineStr"/>
+      <c r="M141" s="2" t="inlineStr">
+        <is>
+          <t>FR-022 説明に「異常系」セクションを追加。「入力 CSV が存在しない場合はエラー終了（FR-023 に伝播）」「ピーク0件（空 CSV）の場合は「ゼロ」を返し正常終了（フェーズ4へ進む）」の方針を確定して記述する。</t>
+        </is>
+      </c>
+      <c r="N141" s="2" t="inlineStr"/>
+      <c r="O141" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P141" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="40" customHeight="1">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-142</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>FR-023 の下位 FR エラー時のエラー伝播方針を SRS に明記</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>FR-023 の説明に、下位 FR（FR-004・FR-014・FR-008・FR-018・FR-022 等）が異常終了した場合の挙動が記述されていない。シェルスクリプトとして即時終了（エラー伝播）するかどうかの方針が不明。スキップして継続する設計も考えられるが、フェイルファースト原則（lessons.md 参照）に照らせば即時終了が適切と推定される。</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E142" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr"/>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J142" s="2" t="inlineStr"/>
+      <c r="K142" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L142" s="2" t="inlineStr"/>
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>方針を確定し（推奨: 即時終了・エラー伝播）、FR-023 説明のループ終了条件周辺に「呼び出した FR がエラー終了した場合は FR-023 も即時終了する」旨を追記する。</t>
+        </is>
+      </c>
+      <c r="N142" s="2" t="inlineStr"/>
+      <c r="O142" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P142" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="40" customHeight="1">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-143</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>FR-020: NFR-010（描画応答性）スコープに公開用 HTML を含めるか確認・RTM 更新</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>spec-panel FR-020 レビュー指摘③。NFR-010（描画応答性・連続操作の滑らかさ）は「本 NFR は HTML ビューア（FR-013）のマーカー描画に適用する」と FR-013 のみに限定されている。公開用 HTML（FR-020）も同規模（最大1万件）のマーカーを表示するビューアであり、60fps の描画応答性要件が同様に適用されるべきかどうかを確認する必要がある。RTM でも FR-020 → UR-014 のマッピングが欠落している。</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E143" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J143" s="2" t="inlineStr"/>
+      <c r="K143" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L143" s="2" t="inlineStr"/>
+      <c r="M143" s="2" t="inlineStr">
+        <is>
+          <t>NFR-010 のスコープを FR-020 にも明示的に拡張する（「HTML ビューア（FR-013・FR-020）のマーカー描画に適用する」）か、FR-013 と同等の要件が FR-020 に引き継がれることを NFR-010 本文または ADR に明記するかを選択し、RTM の FR-020 行 UR-014 列に ✅ を追記する。</t>
+        </is>
+      </c>
+      <c r="N143" s="2" t="inlineStr"/>
+      <c r="O143" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P143" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="40" customHeight="1">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-144</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>FR-017 生成1（60地域GeoJSON）への北方領土ポリゴン含有の扱いを明示</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>FR-017 §生成1（60地域GeoJSON）を作成する際、北方領土6村（N03_007: 01695〜01700）のポリゴンを dissolve 対象に含めるか除外するかが未定義。生成3（北方領土除外タイルリスト）は同コードを抽出して別途処理するが、生成1の dissolve 処理で除外するか残すかが記述されていない。含めたままにすると FR-009 でのエリアコード付与対象に北方領土のポリゴン範囲が残るが、北方領土のピーク候補は FR-001 タイル取得スキップにより解析結果に流れ込まない設計のため実害はない。ただし設計意図が読み取れない状態であり、実装者が迷う可能性がある。</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E144" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J144" s="2" t="inlineStr"/>
+      <c r="K144" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L144" s="2" t="inlineStr"/>
+      <c r="M144" s="2" t="inlineStr">
+        <is>
+          <t>「生成1では北方領土ポリゴンを dissolve 対象に含める（除外は生成3＋FR-001 で完結しているため重複除外は不要）」または「生成3と同一条件で生成1から除外する」どちらかを決定し、FR-017 §生成1 の説明文に明記する。</t>
+        </is>
+      </c>
+      <c r="N144" s="2" t="inlineStr"/>
+      <c r="O144" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P144" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="40" customHeight="1">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-145</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>FR-017 生成1 dissolve の出力形状（MultiPolygon 可否）を明示</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>FR-017 §生成1（行282）に「1地域1ポリゴンに集約」と記述されているが、沖縄・鹿児島等の離島は本島と隣接しないため dissolve の自然な結果は MultiPolygon になる。「1ポリゴン」が MultiPolygon 許容なのか厳密に単一 Polygon なのかが未定義。FR-009 での point-in-polygon 処理の実装時（GeoJSON ライブラリの扱い）に影響する。</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E145" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J145" s="2" t="inlineStr"/>
+      <c r="K145" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L145" s="2" t="inlineStr"/>
+      <c r="M145" s="2" t="inlineStr">
+        <is>
+          <t>「1フィーチャ（MultiPolygon 許容）に集約」として SRS の記述「1地域1ポリゴン」を「1地域1フィーチャ（MultiPolygon 許容）」に更新することを推奨する。離島を含む都府県は必然的に MultiPolygon になるため単一 Polygon への厳密化は現実的でない。</t>
+        </is>
+      </c>
+      <c r="N145" s="2" t="inlineStr"/>
+      <c r="O145" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P145" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="40" customHeight="1">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-146</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>FR-017 再実行条件（N03 ZIP 差し替え時）の SRS 記載 vs HLD 委任を判断</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>FR-017 §実行タイミング（行276）は「初回のみ。出力ファイル群が未生成の場合に起動する」と定義しているが、N03 ZIP を新年版に差し替えた場合の再実行手順が未定義。「出力ファイルを削除してから再実行する」という操作手順を SRS 段階で明記するか、HLD に完全委任するかを決める必要がある。</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E146" s="5" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J146" s="2" t="inlineStr"/>
+      <c r="K146" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L146" s="2" t="inlineStr"/>
+      <c r="M146" s="2" t="inlineStr">
+        <is>
+          <t>SRS に「出力ファイルを手動削除することで再実行できる（詳細は HLD 参照）」程度の一文を追加する方向を推奨する。完全 HLD 委任とする場合は FR-017 §実行タイミングに『再実行はHLD参照』の一文を追記する。</t>
+        </is>
+      </c>
+      <c r="N146" s="2" t="inlineStr"/>
+      <c r="O146" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P146" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="40" customHeight="1">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-147</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>ADR-URD-005 Consequences が旧方式（FR-003 NODATA 扱い）のまま残存し ADR-SRS-018 と矛盾</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>ADR-URD-005 の §Consequences（行96–107）は「北方領土タイルは FR-001 で引き続き取得し FR-003 で NODATA 扱い」という旧方式の記述が残存している。しかし ADR-SRS-018（2026-06-07 採用）では FR-001 が HTTP リクエストを発行しない新方式に変更されており、ADR-URD-005 Decision 本文（行40–54）もこの新方式を記述している。Consequences のみが旧方式のまま放置されており、ADR 内で矛盾が生じている。</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr"/>
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I147" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J147" s="2" t="inlineStr"/>
+      <c r="K147" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L147" s="2" t="inlineStr"/>
+      <c r="M147" s="2" t="inlineStr">
+        <is>
+          <t>ADR-URD-005 §Consequences から FR-003 への言及（行101）と「北方領土タイルは FR-001 で引き続き取得される」記述（行102–104）を削除し、「FR-001 が HTTP リクエストを発行しないことで除外が完結する」旨に書き換える。</t>
+        </is>
+      </c>
+      <c r="N147" s="2" t="inlineStr"/>
+      <c r="O147" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P147" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="40" customHeight="1">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-148</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>FR-001 で DEM10b（Z14）取得時の北方領土除外方法が仕様に未記述</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>北方領土除外タイルリストは Z15 形式（x y 整数ペア、§7.2.2.1）と FR-001 行329 に明記されているが、DEM10b は Z14 で配信される（§6.2.10）。Z14 タイルを Z15 リストからどう除外するか（floor(x/2), floor(y/2) による変換で Z14 タイルを除外するか、別途 Z14 リストを生成するか、そもそも北方領土に DEM10b タイルが存在しないかなど）が FR-001 にも §7.2.2.1 にも記述なく、実装時にバグを招く可能性がある。ADR-URD-005 の Decision（行50）も「ズームレベル 15 の x/y 整数ペア」のみ言及し Z14 への言及がない。</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E148" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>prefetch</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr"/>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J148" s="2" t="inlineStr"/>
+      <c r="K148" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L148" s="2" t="inlineStr"/>
+      <c r="M148" s="2" t="inlineStr">
+        <is>
+          <t>ADR-URD-005 あるいは新規 ADR-SRS-XXX で Z14 タイル除外方法を設計決定し、FR-001 説明および §7.2.2.1 に明記する。設計の選択肢: (a) Z15 リストを floor(x/2),floor(y/2) で変換して Z14 タイルも除外 / (b) FR-017 が Z14 リストを別途生成 / (c) 地理院は北方領土の DEM10b タイルを提供しないため取得時に HTTP 404 になるだけで除外不要（実データ確認が先決）。</t>
+        </is>
+      </c>
+      <c r="N148" s="2" t="inlineStr"/>
+      <c r="O148" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P148" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="40" customHeight="1">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-149</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>FR-001 リトライ（HTTP 429/503）上限超過後の挙動が SRS 未定義</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>FR-001 説明 行333 に「HTTP 429/503 が返された場合は再試行する（リトライ戦略の詳細は HLD 参照）」とあるが、リトライ上限超過後の挙動（エラー終了して全体を止めるか、当該タイルをスキップして継続するか）が SRS レベルの方針として未定義。他の異常系（北方領土リスト未存在→エラー終了、HTTP 404→キャッシュ削除）は SRS で明確化されているが、リトライ超過のみ HLD 丸投げとなっている。</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E149" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>prefetch</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr"/>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J149" s="2" t="inlineStr"/>
+      <c r="K149" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L149" s="2" t="inlineStr"/>
+      <c r="M149" s="2" t="inlineStr">
+        <is>
+          <t>SRS の FR-001 説明にリトライ上限超過後の基本方針（エラー終了 or スキップ継続）を明記し、上限回数・バックオフアルゴリズム等の詳細は引き続き HLD に委任する。ユーザーへの影響（全タイル取得失敗か部分取得かで後段解析品質が大きく変わる）を考慮して設計方針を決定すること。</t>
+        </is>
+      </c>
+      <c r="N149" s="2" t="inlineStr"/>
+      <c r="O149" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P149" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="40" customHeight="1">
+      <c r="A150" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-150</t>
+        </is>
+      </c>
+      <c r="B150" s="6" t="inlineStr">
+        <is>
+          <t>FR-022 異常系: key_col_resolved カラム不在時の動作が未定義</t>
+        </is>
+      </c>
+      <c r="C150" s="6" t="inlineStr">
+        <is>
+          <t>spec-panel レビュー（2026-06-28）で検出。FR-022 の異常系には「ファイル不存在」「読み取りエラー」「空CSV」の3ケースを定義しているが、CSVが存在し読み取れても key_col_resolved カラムが欠落（スキーマ不整合）している場合の動作が規定されていない。実装者が判断を委ねられるリスクがある。</t>
+        </is>
+      </c>
+      <c r="D150" s="6" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E150" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F150" s="6" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G150" s="6" t="inlineStr"/>
+      <c r="H150" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I150" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J150" s="6" t="inlineStr"/>
+      <c r="K150" s="6" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L150" s="6" t="inlineStr"/>
+      <c r="M150" s="6" t="inlineStr">
+        <is>
+          <t>「読み取りエラー」の定義を「CSVスキーマ不整合（key_col_resolved カラム不在等）を含む」に拡張してエラー終了とする案、または別ケースとして追記する案を比較し、SRS FR-022 異常系に確定記述を追加する。対象: docs/20_SRS.md line 844–846</t>
+        </is>
+      </c>
+      <c r="N150" s="6" t="inlineStr"/>
+      <c r="O150" s="6" t="inlineStr"/>
+      <c r="P150" s="6" t="inlineStr"/>
+    </row>
+    <row r="151" ht="40" customHeight="1">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-151</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>FR-019: matchedのdelete_zoneビューア表示可否の設計決定</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>FR-009フィーチャ構成テーブル（line 962）でmatchedにPolygon（delete判定ゾーン）を追記したが、FR-019 line 1152が「delete判定ゾーンポリゴン（new / dominant）を独立したトグルレイヤーとして追加」のままで、matchedのdelete_zoneをビューアで表示するか否かが未定義。FR-019の表示ロジック（AZとの重なり除外・デフォルトON等）がmatchedにも適用されるかどうかも不明確。</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr"/>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I151" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J151" s="2" t="inlineStr"/>
+      <c r="K151" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L151" s="2" t="inlineStr"/>
+      <c r="M151" s="2" t="inlineStr">
+        <is>
+          <t>① matchedのdelete_zoneをビューアのトグルレイヤーで表示するか否かを設計決定する。② 表示する場合はFR-019 line 1152の「new / dominant」制限を削除してSRS修正。③ 表示しない場合は「matched を除く」旨を明示し、SRS FR-009 line 1028の「new / dominant のみ」と整合させる。いずれの場合もFR-009 line 1028・FR-019 line 1152の両方を同時修正する。</t>
+        </is>
+      </c>
+      <c r="N151" s="2" t="inlineStr"/>
+      <c r="O151" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P151" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="40" customHeight="1">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-152</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>SRS: 海面確定規則（層1）でのcol_lat/col_lon=0.0 sentinel 定義を明記する</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>FR-019 line 1185「陸地最高峰・島嶼部最高峰はcol_lat/col_lon=0.0 sentinelのためkey_col feature が除外」と記述しているが、FR-006 line 651（海面確定規則）はその場合のcol_lat/col_lonの値を明記していない。per-mesh CSVカラム定義（line 689）はkey_col_resolved=falseの場合のみ0.0と定義しており、key_col_resolved=trueかつKey Col=海面0m（陸地最高峰リスト・海面確定規則）の場合のcol_lat/col_lonが未定義。またFR-018 line 815が「陸地最高峰は0.0のため除外」のみで島嶼部最高峰（海面確定規則）への言及がなく、FR-019 line 1185と不整合。</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E152" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr"/>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J152" s="2" t="inlineStr"/>
+      <c r="K152" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L152" s="2" t="inlineStr"/>
+      <c r="M152" s="2" t="inlineStr">
+        <is>
+          <t>FR-006 line 651（海面確定規則）に「col_lat/col_lon=0.0 sentinelを設定する」旨を追記。per-mesh CSV カラム定義（line 689）をkey_col_resolved=falseの場合に加えて「海面確定（key_col_resolved=true + Key Col=0m）の場合もcol_lat=col_lon=0.0」と拡張。FR-018 line 815を「陸地最高峰・島嶼部最高峰（海面確定規則）は」に拡張。ADR-SRS-019の層1説明にもcol座標値を追記する。</t>
+        </is>
+      </c>
+      <c r="N152" s="2" t="inlineStr"/>
+      <c r="O152" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P152" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="40" customHeight="1">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-153</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>FR-019: popup表示文言「未定義（陸地最高峰）」の見直し</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>FR-019 line 1185でkey_col featureがない場合の表示文言を「未定義（陸地最高峰）」としているが、「陸地最高峰と島嶼部最高峰はビューア上で区別しない」という方針と齟齬がある。宮之浦岳（屋久島最高峰・SOTA申請対象）など地理的に陸地最高峰でない山にも「陸地最高峰」と表示される。前セッションで「UI上は陸地最高峰に統一」と決定したが、その理由がSRS本文に明記されておらず、担当者が混乱する可能性がある。</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E153" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr"/>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I153" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J153" s="2" t="inlineStr"/>
+      <c r="K153" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L153" s="2" t="inlineStr"/>
+      <c r="M153" s="2" t="inlineStr">
+        <is>
+          <t>① 表示文言を「未定義（Keyコルなし）」等の地理的事実に中立な文言に変更する、または ② 現文言「未定義（陸地最高峰）」を維持し「陸地最高峰・島嶼部最高峰を区別せず統一ラベルとして使用」旨を括弧書きで明記する。どちらを選ぶかをユーザーと合意してSRS line 1185を更新する。</t>
+        </is>
+      </c>
+      <c r="N153" s="2" t="inlineStr"/>
+      <c r="O153" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P153" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="40" customHeight="1">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-154</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>SRS FR-009: matchedピークが他サミットの主ピークになるシナリオを明示する</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>FR-016が全ピーク（match_status問わず）にdelete_zoneを生成し、FR-009の主ピーク特定（line 905-910）も全ピークのdelete_zoneを対象にする。matchedピークのdelete_zone内にAZ外のSOTAサミット（delete候補）が入った場合、matchedピークが主ピークになり得るが、この場合のpeak.match_status（matchedのまま？）・フィーチャ構成（matchedにdeleteサミットのPointを追加するか）が未定義。line 962のmatchedフィーチャ構成には削除候補サミットの複数Point/LineStringについての記述がない。</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E154" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr"/>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J154" s="2" t="inlineStr"/>
+      <c r="K154" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L154" s="2" t="inlineStr"/>
+      <c r="M154" s="2" t="inlineStr">
+        <is>
+          <t>以下のいずれかを決定してFR-009 line 905-910・line 962に反映する。① matchedピークは主ピーク候補から除外する（「AZ内にSOTAサミットがいるピーク（matched）はdelete_zone内に別のサミットがいても主ピークにならない」制約を追加）。② matchedかつ主ピークになるケースを許容し、フィーチャ構成にdeleteサミットPoint・LineStringを追加する記述を加える。</t>
+        </is>
+      </c>
+      <c r="N154" s="2" t="inlineStr"/>
+      <c r="O154" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="P154" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="40" customHeight="1">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-155</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>ADR-042 シナリオD で削除申請データ取りこぼし問題の再決定（ADR-043 + SRS 反映）</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>ADR-SRS-042（matched ピークを delete サミット主ピーク候補から除外）はシナリオD（AZ内1サミット＋delete_zone内1サミットが同一ピークに存在）で削除申請データを取りこぼす。九州・四国解析で実際に1件発生済み。matched ピークも主ピーク候補に含め、dominant_peak_code に matched ピークの既存 SOTA コードを付与して削除申請を自動生成する軽量修正に方針変更する。</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E155" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="I155" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J155" s="2" t="inlineStr"/>
+      <c r="K155" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L155" s="2" t="inlineStr"/>
+      <c r="M155" s="2" t="inlineStr">
+        <is>
+          <t>新規 ADR-SRS-043 で ADR-042 を supersede。FR-009 主ピーク特定ロジックの matched 除外を撤回し、matched フィーチャ構成に従属 delete サミット Point/LineString を追加定義する。</t>
+        </is>
+      </c>
+      <c r="N155" s="2" t="inlineStr"/>
+      <c r="O155" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="P155" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="40" customHeight="1">
+      <c r="A156" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-156</t>
+        </is>
+      </c>
+      <c r="B156" s="6" t="inlineStr">
+        <is>
+          <t>申請カテゴリをプロパティ化し FR-009 フィーチャ構成表をサミット中心5分類へ再編</t>
+        </is>
+      </c>
+      <c r="C156" s="6" t="inlineStr">
+        <is>
+          <t>FR-009 の merged_summit.geojson フィーチャ構成表が peak.match_status 軸で書かれており、サミット中心の申請カテゴリ（追加/変更あり/変更なし/削除/要確認）が直読できない。category プロパティを GeoJSON・XLSX・ZIP 全成果物に統一して持たせ、消費側の実行時導出を廃止する。ADR-SRS-035 を supersede する ADR-SRS-044 を新規作成し、FR-009/011/012/013/019/020/021・GLOSSARY を改訂する。</t>
+        </is>
+      </c>
+      <c r="D156" s="6" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E156" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F156" s="6" t="inlineStr"/>
+      <c r="G156" s="6" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H156" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="I156" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J156" s="6" t="inlineStr"/>
+      <c r="K156" s="6" t="inlineStr">
         <is>
           <t>対応完了</t>
         </is>
       </c>
-      <c r="L140" s="6" t="inlineStr"/>
-      <c r="M140" s="6" t="inlineStr">
-        <is>
-          <t>カラムを確定し（最低限 peak_lat, peak_lon。追加列があれば明示）、FR-022 出力テーブル備考欄か §7.2.2 に定義セクションを追加する。FR-014 入力備考欄も整合させる。</t>
-        </is>
-      </c>
-      <c r="N140" s="6" t="inlineStr"/>
-      <c r="O140" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="P140" s="6" t="inlineStr"/>
-    </row>
-    <row r="141" ht="40" customHeight="1">
-      <c r="A141" s="7" t="inlineStr">
-        <is>
-          <t>ISSUE-141</t>
-        </is>
-      </c>
-      <c r="B141" s="7" t="inlineStr">
-        <is>
-          <t>FR-022 異常系定義の追加（入力 CSV 不存在・空ピーク時の挙動）</t>
-        </is>
-      </c>
-      <c r="C141" s="7" t="inlineStr">
-        <is>
-          <t>FR-022 に異常系定義がない。FR-014・FR-004 等は「異常系」セクションを持つが FR-022 には存在しない。「merged_peak.csv が存在しない場合」「CSV が空（0件ピーク）の場合」の挙動が未定義。空ピークの場合は「ゼロ件 = 全充足」として正常終了してフェーズ4へ進んでよいかの設計判断も必要。</t>
-        </is>
-      </c>
-      <c r="D141" s="7" t="inlineStr">
+      <c r="L156" s="6" t="inlineStr"/>
+      <c r="M156" s="6" t="inlineStr"/>
+      <c r="N156" s="6" t="inlineStr"/>
+      <c r="O156" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="P156" s="6" t="inlineStr"/>
+    </row>
+    <row r="157" ht="40" customHeight="1">
+      <c r="A157" s="7" t="inlineStr">
+        <is>
+          <t>ISSUE-157</t>
+        </is>
+      </c>
+      <c r="B157" s="7" t="inlineStr">
+        <is>
+          <t>FR-009: コル（key_col）プロパティ定義に municipality を追加</t>
+        </is>
+      </c>
+      <c r="C157" s="7" t="inlineStr">
+        <is>
+          <t>merged_summit.geojson の Point フィーチャのうち、ピーク・サミットには municipality が付与されるが、コル（key_col）の properties 定義から漏れている。コル自身の座標で point-in-polygon 判定して municipality を付与する仕様に改訂する。</t>
+        </is>
+      </c>
+      <c r="D157" s="7" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E157" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F157" s="7" t="inlineStr">
+        <is>
+          <t>GeoJSON出力</t>
+        </is>
+      </c>
+      <c r="G157" s="7" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H157" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="I157" s="7" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J157" s="7" t="inlineStr"/>
+      <c r="K157" s="7" t="inlineStr">
+        <is>
+          <t>対応完了</t>
+        </is>
+      </c>
+      <c r="L157" s="7" t="inlineStr"/>
+      <c r="M157" s="7" t="inlineStr"/>
+      <c r="N157" s="7" t="inlineStr"/>
+      <c r="O157" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="P157" s="7" t="inlineStr"/>
+    </row>
+    <row r="158" ht="40" customHeight="1">
+      <c r="A158" s="6" t="inlineStr">
+        <is>
+          <t>ISSUE-158</t>
+        </is>
+      </c>
+      <c r="B158" s="6" t="inlineStr">
+        <is>
+          <t>FR-009/FR-012 サミット一覧 XLSX の行集約生成モデルが SRS 未定義</t>
+        </is>
+      </c>
+      <c r="C158" s="6" t="inlineStr">
+        <is>
+          <t>merged_summit.geojson は複数フィーチャ（ピーク Point／コル Point／AZ Polygon／既存サミット Point／LineString）を持つ。FR-009 の merged_summit.xlsx（サミット一覧（突合後））と FR-012 の merged_summit_revised.xlsx（申請内容反映版）はこれらを 1 行（＝1 ピーククラスタ想定）に集約してカラム化するが、(a) 行の単位（集約単位か Point 毎か）、(b) 結合キー（summit_code 等）、(c) 各カラムの取得元フィーチャ（peak_*/col_*/sota_* ＝各 Point geometry、area_complete ＝ AZ Polygon properties、dominant の sota_* ＝ dominant_peak_code 経由）が SRS 未定義。FR-012 概要は「Point フィーチャのみが行に変換される」（SRS 1298行）としか書かず集約モデルが欠落している。FR-012 は「FR-009 と同じ作り方＋ユーザー編集反映」なので、FR-009 側の行集約モデルが決まれば FR-012 は従属的に決まる。</t>
+        </is>
+      </c>
+      <c r="D158" s="6" t="inlineStr">
         <is>
           <t>設計</t>
         </is>
       </c>
-      <c r="E141" s="4" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="F141" s="7" t="inlineStr">
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F158" s="6" t="inlineStr">
         <is>
           <t>その他</t>
         </is>
       </c>
-      <c r="G141" s="7" t="inlineStr"/>
-      <c r="H141" s="7" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="I141" s="7" t="inlineStr">
-        <is>
-          <t>SRS</t>
-        </is>
-      </c>
-      <c r="J141" s="7" t="inlineStr"/>
-      <c r="K141" s="7" t="inlineStr">
-        <is>
-          <t>対応完了</t>
-        </is>
-      </c>
-      <c r="L141" s="7" t="inlineStr"/>
-      <c r="M141" s="7" t="inlineStr">
-        <is>
-          <t>FR-022 説明に「異常系」セクションを追加。「入力 CSV が存在しない場合はエラー終了（FR-023 に伝播）」「ピーク0件（空 CSV）の場合は「ゼロ」を返し正常終了（フェーズ4へ進む）」の方針を確定して記述する。</t>
-        </is>
-      </c>
-      <c r="N141" s="7" t="inlineStr"/>
-      <c r="O141" s="7" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="P141" s="7" t="inlineStr"/>
-    </row>
-    <row r="142" ht="40" customHeight="1">
-      <c r="A142" s="6" t="inlineStr">
-        <is>
-          <t>ISSUE-142</t>
-        </is>
-      </c>
-      <c r="B142" s="6" t="inlineStr">
-        <is>
-          <t>FR-023 の下位 FR エラー時のエラー伝播方針を SRS に明記</t>
-        </is>
-      </c>
-      <c r="C142" s="6" t="inlineStr">
-        <is>
-          <t>FR-023 の説明に、下位 FR（FR-004・FR-014・FR-008・FR-018・FR-022 等）が異常終了した場合の挙動が記述されていない。シェルスクリプトとして即時終了（エラー伝播）するかどうかの方針が不明。スキップして継続する設計も考えられるが、フェイルファースト原則（lessons.md 参照）に照らせば即時終了が適切と推定される。</t>
-        </is>
-      </c>
-      <c r="D142" s="6" t="inlineStr">
-        <is>
-          <t>設計</t>
-        </is>
-      </c>
-      <c r="E142" s="4" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="F142" s="6" t="inlineStr">
-        <is>
-          <t>その他</t>
-        </is>
-      </c>
-      <c r="G142" s="6" t="inlineStr"/>
-      <c r="H142" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="I142" s="6" t="inlineStr">
-        <is>
-          <t>SRS</t>
-        </is>
-      </c>
-      <c r="J142" s="6" t="inlineStr"/>
-      <c r="K142" s="6" t="inlineStr">
-        <is>
-          <t>対応完了</t>
-        </is>
-      </c>
-      <c r="L142" s="6" t="inlineStr"/>
-      <c r="M142" s="6" t="inlineStr">
-        <is>
-          <t>方針を確定し（推奨: 即時終了・エラー伝播）、FR-023 説明のループ終了条件周辺に「呼び出した FR がエラー終了した場合は FR-023 も即時終了する」旨を追記する。</t>
-        </is>
-      </c>
-      <c r="N142" s="6" t="inlineStr"/>
-      <c r="O142" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="P142" s="6" t="inlineStr"/>
-    </row>
-    <row r="143" ht="40" customHeight="1">
-      <c r="A143" s="7" t="inlineStr">
-        <is>
-          <t>ISSUE-143</t>
-        </is>
-      </c>
-      <c r="B143" s="7" t="inlineStr">
-        <is>
-          <t>FR-020: NFR-010（描画応答性）スコープに公開用 HTML を含めるか確認・RTM 更新</t>
-        </is>
-      </c>
-      <c r="C143" s="7" t="inlineStr">
-        <is>
-          <t>spec-panel FR-020 レビュー指摘③。NFR-010（描画応答性・連続操作の滑らかさ）は「本 NFR は HTML ビューア（FR-013）のマーカー描画に適用する」と FR-013 のみに限定されている。公開用 HTML（FR-020）も同規模（最大1万件）のマーカーを表示するビューアであり、60fps の描画応答性要件が同様に適用されるべきかどうかを確認する必要がある。RTM でも FR-020 → UR-014 のマッピングが欠落している。</t>
-        </is>
-      </c>
-      <c r="D143" s="7" t="inlineStr">
-        <is>
-          <t>設計</t>
-        </is>
-      </c>
-      <c r="E143" s="4" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="F143" s="7" t="inlineStr">
-        <is>
-          <t>その他</t>
-        </is>
-      </c>
-      <c r="G143" s="7" t="inlineStr">
-        <is>
-          <t>Sonnet</t>
-        </is>
-      </c>
-      <c r="H143" s="7" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="I143" s="7" t="inlineStr">
-        <is>
-          <t>SRS</t>
-        </is>
-      </c>
-      <c r="J143" s="7" t="inlineStr"/>
-      <c r="K143" s="7" t="inlineStr">
-        <is>
-          <t>対応完了</t>
-        </is>
-      </c>
-      <c r="L143" s="7" t="inlineStr"/>
-      <c r="M143" s="7" t="inlineStr">
-        <is>
-          <t>NFR-010 のスコープを FR-020 にも明示的に拡張する（「HTML ビューア（FR-013・FR-020）のマーカー描画に適用する」）か、FR-013 と同等の要件が FR-020 に引き継がれることを NFR-010 本文または ADR に明記するかを選択し、RTM の FR-020 行 UR-014 列に ✅ を追記する。</t>
-        </is>
-      </c>
-      <c r="N143" s="7" t="inlineStr"/>
-      <c r="O143" s="7" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="P143" s="7" t="inlineStr"/>
-    </row>
-    <row r="144" ht="40" customHeight="1">
-      <c r="A144" s="6" t="inlineStr">
-        <is>
-          <t>ISSUE-144</t>
-        </is>
-      </c>
-      <c r="B144" s="6" t="inlineStr">
-        <is>
-          <t>FR-017 生成1（60地域GeoJSON）への北方領土ポリゴン含有の扱いを明示</t>
-        </is>
-      </c>
-      <c r="C144" s="6" t="inlineStr">
-        <is>
-          <t>FR-017 §生成1（60地域GeoJSON）を作成する際、北方領土6村（N03_007: 01695〜01700）のポリゴンを dissolve 対象に含めるか除外するかが未定義。生成3（北方領土除外タイルリスト）は同コードを抽出して別途処理するが、生成1の dissolve 処理で除外するか残すかが記述されていない。含めたままにすると FR-009 でのエリアコード付与対象に北方領土のポリゴン範囲が残るが、北方領土のピーク候補は FR-001 タイル取得スキップにより解析結果に流れ込まない設計のため実害はない。ただし設計意図が読み取れない状態であり、実装者が迷う可能性がある。</t>
-        </is>
-      </c>
-      <c r="D144" s="6" t="inlineStr">
-        <is>
-          <t>設計</t>
-        </is>
-      </c>
-      <c r="E144" s="4" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="F144" s="6" t="inlineStr">
-        <is>
-          <t>その他</t>
-        </is>
-      </c>
-      <c r="G144" s="6" t="inlineStr">
-        <is>
-          <t>Sonnet</t>
-        </is>
-      </c>
-      <c r="H144" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="I144" s="6" t="inlineStr">
-        <is>
-          <t>SRS</t>
-        </is>
-      </c>
-      <c r="J144" s="6" t="inlineStr"/>
-      <c r="K144" s="6" t="inlineStr">
-        <is>
-          <t>対応完了</t>
-        </is>
-      </c>
-      <c r="L144" s="6" t="inlineStr"/>
-      <c r="M144" s="6" t="inlineStr">
-        <is>
-          <t>「生成1では北方領土ポリゴンを dissolve 対象に含める（除外は生成3＋FR-001 で完結しているため重複除外は不要）」または「生成3と同一条件で生成1から除外する」どちらかを決定し、FR-017 §生成1 の説明文に明記する。</t>
-        </is>
-      </c>
-      <c r="N144" s="6" t="inlineStr"/>
-      <c r="O144" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="P144" s="6" t="inlineStr"/>
-    </row>
-    <row r="145" ht="40" customHeight="1">
-      <c r="A145" s="7" t="inlineStr">
-        <is>
-          <t>ISSUE-145</t>
-        </is>
-      </c>
-      <c r="B145" s="7" t="inlineStr">
-        <is>
-          <t>FR-017 生成1 dissolve の出力形状（MultiPolygon 可否）を明示</t>
-        </is>
-      </c>
-      <c r="C145" s="7" t="inlineStr">
-        <is>
-          <t>FR-017 §生成1（行282）に「1地域1ポリゴンに集約」と記述されているが、沖縄・鹿児島等の離島は本島と隣接しないため dissolve の自然な結果は MultiPolygon になる。「1ポリゴン」が MultiPolygon 許容なのか厳密に単一 Polygon なのかが未定義。FR-009 での point-in-polygon 処理の実装時（GeoJSON ライブラリの扱い）に影響する。</t>
-        </is>
-      </c>
-      <c r="D145" s="7" t="inlineStr">
-        <is>
-          <t>設計</t>
-        </is>
-      </c>
-      <c r="E145" s="4" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="F145" s="7" t="inlineStr">
-        <is>
-          <t>その他</t>
-        </is>
-      </c>
-      <c r="G145" s="7" t="inlineStr">
-        <is>
-          <t>Sonnet</t>
-        </is>
-      </c>
-      <c r="H145" s="7" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="I145" s="7" t="inlineStr">
-        <is>
-          <t>SRS</t>
-        </is>
-      </c>
-      <c r="J145" s="7" t="inlineStr"/>
-      <c r="K145" s="7" t="inlineStr">
-        <is>
-          <t>対応完了</t>
-        </is>
-      </c>
-      <c r="L145" s="7" t="inlineStr"/>
-      <c r="M145" s="7" t="inlineStr">
-        <is>
-          <t>「1フィーチャ（MultiPolygon 許容）に集約」として SRS の記述「1地域1ポリゴン」を「1地域1フィーチャ（MultiPolygon 許容）」に更新することを推奨する。離島を含む都府県は必然的に MultiPolygon になるため単一 Polygon への厳密化は現実的でない。</t>
-        </is>
-      </c>
-      <c r="N145" s="7" t="inlineStr"/>
-      <c r="O145" s="7" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="P145" s="7" t="inlineStr"/>
-    </row>
-    <row r="146" ht="40" customHeight="1">
-      <c r="A146" s="6" t="inlineStr">
-        <is>
-          <t>ISSUE-146</t>
-        </is>
-      </c>
-      <c r="B146" s="6" t="inlineStr">
-        <is>
-          <t>FR-017 再実行条件（N03 ZIP 差し替え時）の SRS 記載 vs HLD 委任を判断</t>
-        </is>
-      </c>
-      <c r="C146" s="6" t="inlineStr">
-        <is>
-          <t>FR-017 §実行タイミング（行276）は「初回のみ。出力ファイル群が未生成の場合に起動する」と定義しているが、N03 ZIP を新年版に差し替えた場合の再実行手順が未定義。「出力ファイルを削除してから再実行する」という操作手順を SRS 段階で明記するか、HLD に完全委任するかを決める必要がある。</t>
-        </is>
-      </c>
-      <c r="D146" s="6" t="inlineStr">
-        <is>
-          <t>設計</t>
-        </is>
-      </c>
-      <c r="E146" s="5" t="inlineStr">
-        <is>
-          <t>低</t>
-        </is>
-      </c>
-      <c r="F146" s="6" t="inlineStr">
-        <is>
-          <t>その他</t>
-        </is>
-      </c>
-      <c r="G146" s="6" t="inlineStr">
-        <is>
-          <t>Sonnet</t>
-        </is>
-      </c>
-      <c r="H146" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="I146" s="6" t="inlineStr">
-        <is>
-          <t>SRS</t>
-        </is>
-      </c>
-      <c r="J146" s="6" t="inlineStr"/>
-      <c r="K146" s="6" t="inlineStr">
-        <is>
-          <t>対応完了</t>
-        </is>
-      </c>
-      <c r="L146" s="6" t="inlineStr"/>
-      <c r="M146" s="6" t="inlineStr">
-        <is>
-          <t>SRS に「出力ファイルを手動削除することで再実行できる（詳細は HLD 参照）」程度の一文を追加する方向を推奨する。完全 HLD 委任とする場合は FR-017 §実行タイミングに『再実行はHLD参照』の一文を追記する。</t>
-        </is>
-      </c>
-      <c r="N146" s="6" t="inlineStr"/>
-      <c r="O146" s="6" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="P146" s="6" t="inlineStr"/>
+      <c r="G158" s="6" t="inlineStr"/>
+      <c r="H158" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="I158" s="6" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J158" s="6" t="inlineStr"/>
+      <c r="K158" s="6" t="inlineStr">
+        <is>
+          <t>未対応</t>
+        </is>
+      </c>
+      <c r="L158" s="6" t="inlineStr"/>
+      <c r="M158" s="6" t="inlineStr">
+        <is>
+          <t>FR-009 を行集約モデルの正本として XLSX 行生成モデルを定義し、FR-012 はそれを参照する形で記述する。必要なら ADR 化（ADR-SRS-041「geojson スキーマ拡張で全カラム生成可能」の前提を補完）。</t>
+        </is>
+      </c>
+      <c r="N158" s="6" t="inlineStr"/>
+      <c r="O158" s="6" t="inlineStr"/>
+      <c r="P158" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K158" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E158" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D158" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I158" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J158" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10899,7 +11695,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>145</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3">
@@ -10909,7 +11705,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
@@ -10919,7 +11715,7 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>102</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5">
@@ -10930,7 +11726,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>70.3%</t>
+          <t>74.5%</t>
         </is>
       </c>
     </row>
@@ -10949,7 +11745,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -10969,7 +11765,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -10979,7 +11775,7 @@
         </is>
       </c>
       <c r="B11" s="11" t="n">
-        <v>102</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12">
@@ -11017,7 +11813,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
@@ -11027,7 +11823,7 @@
         </is>
       </c>
       <c r="B17" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -11045,7 +11841,7 @@
         </is>
       </c>
       <c r="B20" s="11" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21">
@@ -11065,7 +11861,7 @@
         </is>
       </c>
       <c r="B22" s="11" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24">
@@ -11103,7 +11899,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
@@ -11113,7 +11909,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
@@ -11131,7 +11927,7 @@
         </is>
       </c>
       <c r="B31" s="11" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="32">
@@ -11165,7 +11961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12195,13 +12991,29 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C64" t="n">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="D64" t="n">
         <v>119</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>157</v>
+      </c>
+      <c r="C65" t="n">
+        <v>136</v>
+      </c>
+      <c r="D65" t="n">
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: §6 spec-panel 対応完了（ISSUE-162/163 解決済・todo③④完了・findings 記録）
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mgmt/tracker/reports/issues_export.xlsx
+++ b/mgmt/tracker/reports/issues_export.xlsx
@@ -744,7 +744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P158"/>
+  <dimension ref="A1:P163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11468,22 +11468,22 @@
       </c>
     </row>
     <row r="156" ht="40" customHeight="1">
-      <c r="A156" s="6" t="inlineStr">
+      <c r="A156" s="2" t="inlineStr">
         <is>
           <t>ISSUE-156</t>
         </is>
       </c>
-      <c r="B156" s="6" t="inlineStr">
+      <c r="B156" s="2" t="inlineStr">
         <is>
           <t>申請カテゴリをプロパティ化し FR-009 フィーチャ構成表をサミット中心5分類へ再編</t>
         </is>
       </c>
-      <c r="C156" s="6" t="inlineStr">
+      <c r="C156" s="2" t="inlineStr">
         <is>
           <t>FR-009 の merged_summit.geojson フィーチャ構成表が peak.match_status 軸で書かれており、サミット中心の申請カテゴリ（追加/変更あり/変更なし/削除/要確認）が直読できない。category プロパティを GeoJSON・XLSX・ZIP 全成果物に統一して持たせ、消費側の実行時導出を廃止する。ADR-SRS-035 を supersede する ADR-SRS-044 を新規作成し、FR-009/011/012/013/019/020/021・GLOSSARY を改訂する。</t>
         </is>
       </c>
-      <c r="D156" s="6" t="inlineStr">
+      <c r="D156" s="2" t="inlineStr">
         <is>
           <t>設計</t>
         </is>
@@ -11493,55 +11493,59 @@
           <t>中</t>
         </is>
       </c>
-      <c r="F156" s="6" t="inlineStr"/>
-      <c r="G156" s="6" t="inlineStr">
+      <c r="F156" s="2" t="inlineStr"/>
+      <c r="G156" s="2" t="inlineStr">
         <is>
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="H156" s="6" t="inlineStr">
+      <c r="H156" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="I156" s="6" t="inlineStr">
-        <is>
-          <t>SRS</t>
-        </is>
-      </c>
-      <c r="J156" s="6" t="inlineStr"/>
-      <c r="K156" s="6" t="inlineStr">
-        <is>
-          <t>対応完了</t>
-        </is>
-      </c>
-      <c r="L156" s="6" t="inlineStr"/>
-      <c r="M156" s="6" t="inlineStr"/>
-      <c r="N156" s="6" t="inlineStr"/>
-      <c r="O156" s="6" t="inlineStr">
+      <c r="I156" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J156" s="2" t="inlineStr"/>
+      <c r="K156" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L156" s="2" t="inlineStr"/>
+      <c r="M156" s="2" t="inlineStr"/>
+      <c r="N156" s="2" t="inlineStr"/>
+      <c r="O156" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="P156" s="6" t="inlineStr"/>
+      <c r="P156" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
     </row>
     <row r="157" ht="40" customHeight="1">
-      <c r="A157" s="7" t="inlineStr">
+      <c r="A157" s="2" t="inlineStr">
         <is>
           <t>ISSUE-157</t>
         </is>
       </c>
-      <c r="B157" s="7" t="inlineStr">
+      <c r="B157" s="2" t="inlineStr">
         <is>
           <t>FR-009: コル（key_col）プロパティ定義に municipality を追加</t>
         </is>
       </c>
-      <c r="C157" s="7" t="inlineStr">
+      <c r="C157" s="2" t="inlineStr">
         <is>
           <t>merged_summit.geojson の Point フィーチャのうち、ピーク・サミットには municipality が付与されるが、コル（key_col）の properties 定義から漏れている。コル自身の座標で point-in-polygon 判定して municipality を付与する仕様に改訂する。</t>
         </is>
       </c>
-      <c r="D157" s="7" t="inlineStr">
+      <c r="D157" s="2" t="inlineStr">
         <is>
           <t>改善</t>
         </is>
@@ -11551,59 +11555,63 @@
           <t>中</t>
         </is>
       </c>
-      <c r="F157" s="7" t="inlineStr">
+      <c r="F157" s="2" t="inlineStr">
         <is>
           <t>GeoJSON出力</t>
         </is>
       </c>
-      <c r="G157" s="7" t="inlineStr">
+      <c r="G157" s="2" t="inlineStr">
         <is>
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="H157" s="7" t="inlineStr">
+      <c r="H157" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="I157" s="7" t="inlineStr">
-        <is>
-          <t>SRS</t>
-        </is>
-      </c>
-      <c r="J157" s="7" t="inlineStr"/>
-      <c r="K157" s="7" t="inlineStr">
-        <is>
-          <t>対応完了</t>
-        </is>
-      </c>
-      <c r="L157" s="7" t="inlineStr"/>
-      <c r="M157" s="7" t="inlineStr"/>
-      <c r="N157" s="7" t="inlineStr"/>
-      <c r="O157" s="7" t="inlineStr">
+      <c r="I157" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J157" s="2" t="inlineStr"/>
+      <c r="K157" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L157" s="2" t="inlineStr"/>
+      <c r="M157" s="2" t="inlineStr"/>
+      <c r="N157" s="2" t="inlineStr"/>
+      <c r="O157" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="P157" s="7" t="inlineStr"/>
+      <c r="P157" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
     </row>
     <row r="158" ht="40" customHeight="1">
-      <c r="A158" s="6" t="inlineStr">
+      <c r="A158" s="2" t="inlineStr">
         <is>
           <t>ISSUE-158</t>
         </is>
       </c>
-      <c r="B158" s="6" t="inlineStr">
+      <c r="B158" s="2" t="inlineStr">
         <is>
           <t>FR-009/FR-012 サミット一覧 XLSX の行集約生成モデルが SRS 未定義</t>
         </is>
       </c>
-      <c r="C158" s="6" t="inlineStr">
+      <c r="C158" s="2" t="inlineStr">
         <is>
           <t>merged_summit.geojson は複数フィーチャ（ピーク Point／コル Point／AZ Polygon／既存サミット Point／LineString）を持つ。FR-009 の merged_summit.xlsx（サミット一覧（突合後））と FR-012 の merged_summit_revised.xlsx（申請内容反映版）はこれらを 1 行（＝1 ピーククラスタ想定）に集約してカラム化するが、(a) 行の単位（集約単位か Point 毎か）、(b) 結合キー（summit_code 等）、(c) 各カラムの取得元フィーチャ（peak_*/col_*/sota_* ＝各 Point geometry、area_complete ＝ AZ Polygon properties、dominant の sota_* ＝ dominant_peak_code 経由）が SRS 未定義。FR-012 概要は「Point フィーチャのみが行に変換される」（SRS 1298行）としか書かず集約モデルが欠落している。FR-012 は「FR-009 と同じ作り方＋ユーザー編集反映」なので、FR-009 側の行集約モデルが決まれば FR-012 は従属的に決まる。</t>
         </is>
       </c>
-      <c r="D158" s="6" t="inlineStr">
+      <c r="D158" s="2" t="inlineStr">
         <is>
           <t>設計</t>
         </is>
@@ -11613,53 +11621,399 @@
           <t>高</t>
         </is>
       </c>
-      <c r="F158" s="6" t="inlineStr">
+      <c r="F158" s="2" t="inlineStr">
         <is>
           <t>その他</t>
         </is>
       </c>
-      <c r="G158" s="6" t="inlineStr"/>
-      <c r="H158" s="6" t="inlineStr">
+      <c r="G158" s="2" t="inlineStr"/>
+      <c r="H158" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="I158" s="6" t="inlineStr">
-        <is>
-          <t>SRS</t>
-        </is>
-      </c>
-      <c r="J158" s="6" t="inlineStr"/>
-      <c r="K158" s="6" t="inlineStr">
-        <is>
-          <t>未対応</t>
-        </is>
-      </c>
-      <c r="L158" s="6" t="inlineStr"/>
-      <c r="M158" s="6" t="inlineStr">
+      <c r="I158" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J158" s="2" t="inlineStr"/>
+      <c r="K158" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L158" s="2" t="inlineStr"/>
+      <c r="M158" s="2" t="inlineStr">
         <is>
           <t>FR-009 を行集約モデルの正本として XLSX 行生成モデルを定義し、FR-012 はそれを参照する形で記述する。必要なら ADR 化（ADR-SRS-041「geojson スキーマ拡張で全カラム生成可能」の前提を補完）。</t>
         </is>
       </c>
-      <c r="N158" s="6" t="inlineStr"/>
-      <c r="O158" s="6" t="inlineStr"/>
-      <c r="P158" s="6" t="inlineStr"/>
+      <c r="N158" s="2" t="inlineStr"/>
+      <c r="O158" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="P158" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="40" customHeight="1">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-159</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>FR-009 ZIP 分割(§6.2.9)の category 体系追従と review カテゴリ欠落</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>FR-009 が category(add/band_change/no_change/delete/review の5分類・ADR-SRS-044)を正本付与する一方、§6.2.9 ZIP 分割は旧 match_status 命名(new/dominant/changed/unchanged)のまま。GLOSSARY L162「ZIP分割に category 使用」と矛盾し、review 用 geojson も欠落。category 参照元↔定義元の不完全性。ZIP命名のcategory追従要否・review同梱可否を協議し、§6.2.9/FR-021 と FR-009 を同期する。</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E159" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F159" s="2" t="inlineStr"/>
+      <c r="G159" s="2" t="inlineStr">
+        <is>
+          <t>Opus</t>
+        </is>
+      </c>
+      <c r="H159" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="I159" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J159" s="2" t="inlineStr"/>
+      <c r="K159" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L159" s="2" t="inlineStr"/>
+      <c r="M159" s="2" t="inlineStr"/>
+      <c r="N159" s="2" t="inlineStr">
+        <is>
+          <t>協議完了・SRS反映は次セッション。ADR-SRS-044 で既決（ZIP は add/band_change/no_change/delete/review の5ファイル・delete独立・review同梱。状態=採用未実装）の §6.2.9 追従漏れと判明。ファイル名は category 値に厳密準拠で合意（band_change/no_change を使う。ADR表記の changed/unchanged は旧名残存）。次セッション作業: ①§6.2.9 同梱ファイル一覧を5ファイルに修正 ②ADR-SRS-043 の『delete を dominant.geojson に同梱』記述も ADR-SRS-044（delete独立）に追従 ③FR-021本文のZIP分割記述の追従確認 ④旧ファイル名 new/dominant/changed/unchanged.geojson の全残存を grep 確認。</t>
+        </is>
+      </c>
+      <c r="O159" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="P159" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="40" customHeight="1">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-160</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>FR-009 仮サミットコード採番の prominence=null ソート挙動が未定義</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>採番順序(SRS L894)の2次キーがプロミネンス降順だが、key_col_resolved=false のピークは prominence=null(L1008)。採番は不備ゲート(全判定後・L940)より前に全件実行されるため、null を含むソートの決定論性(NFR-003)が未定義。null ピークのソート位置(末尾固定等)を明示するか、採番対象から除外する旨を規定する。</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E160" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr"/>
+      <c r="G160" s="2" t="inlineStr">
+        <is>
+          <t>Opus</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="I160" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J160" s="2" t="inlineStr"/>
+      <c r="K160" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L160" s="2" t="inlineStr"/>
+      <c r="M160" s="2" t="inlineStr"/>
+      <c r="N160" s="2" t="inlineStr">
+        <is>
+          <t>FR-009 spec-panel レビュー指摘⑤（2026-06-29）。</t>
+        </is>
+      </c>
+      <c r="O160" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="P160" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="40" customHeight="1">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-161</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>FR-009 1サミットが複数ピークのAZに同時包含される場合の帰属規則が未定義</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>AZ内のSOTAサミット一意性(1AZに複数サミット無し・L877)は保証されるが、逆方向(1サミットが複数ピークのAZに同時包含)の帰属規則が未定義。どのピークが band_change 判定基準になるか曖昧(L880/L883-884)。AZ同士は数学的に重ならない根拠を明記するか、複数包含時の帰属タイブレークを規定する。</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>設計</t>
+        </is>
+      </c>
+      <c r="E161" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F161" s="2" t="inlineStr"/>
+      <c r="G161" s="2" t="inlineStr">
+        <is>
+          <t>Opus</t>
+        </is>
+      </c>
+      <c r="H161" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="I161" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J161" s="2" t="inlineStr"/>
+      <c r="K161" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L161" s="2" t="inlineStr"/>
+      <c r="M161" s="2" t="inlineStr"/>
+      <c r="N161" s="2" t="inlineStr">
+        <is>
+          <t>FR-009 spec-panel レビュー指摘⑥（2026-06-29）。</t>
+        </is>
+      </c>
+      <c r="O161" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="P161" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="40" customHeight="1">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-162</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>§6.2.11 SOTA サミットリスト CSV の使用カラムに ValidTo が欠落・FR-009 に廃止済みサミット除外仕様がない</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>§6.2.11 の使用カラム（SummitCode, SummitName, AltM, Latitude, Longitude）に ValidTo が含まれておらず、廃止済み JA サミットの除外仕様が定義されていない。FR-009 の説明にも「JA プレフィックスサミットと突合する」とだけ書かれており ValidTo チェックの記述がない。実際に JA プレフィックスの廃止済みサミット（ValidTo ≠ 31/12/2099）が 147 件存在する。フィルタなしで突合対象に含めると ①delete 判定ゾーン内の廃止サミット → match_status=delete → 申請書に誤った削除行が自動出力 ②判定ゾーン外 → unmatched 件数増加 → 不備ゲート誤発動のリスクがある（lessons.md: 廃止データを母集団に含めない）。</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E162" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H162" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="I162" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J162" s="2" t="inlineStr"/>
+      <c r="K162" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L162" s="2" t="inlineStr"/>
+      <c r="M162" s="2" t="inlineStr">
+        <is>
+          <t>§6.2.11 の使用カラムに ValidTo を追記し、FR-009 の突合前処理として「ValidTo が実行日以降のサミットのみを突合対象とする」旨を明示する。除外条件の表現（実行日比較 vs 31/12/2099 固定判定）を仕様化する。</t>
+        </is>
+      </c>
+      <c r="N162" s="2" t="inlineStr"/>
+      <c r="O162" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="P162" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="40" customHeight="1">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>ISSUE-163</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>§6.1 No.10「使用/生成 FR」欄と FR 入出力テーブルの不整合（FR-004/FR-014 と地理院標高タイルの分類）</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>§6.1 No.10（地理院標高タイル）の「使用/生成 FR」欄に FR-001/FR-004/FR-014/FR-019 と記載されているが、FR-004/FR-014 の入力テーブルでは「標高タイル（ローカルキャッシュ）」を「内部データ」として記載しており、外部I/F としての地理院標高タイルは列挙していない。ADR-SRS-016「ローカルキャッシュは内部データ」に基づくと FR-004/FR-014 が参照するのは内部データであり、§6.1 の「使用 FR」欄と FR 入出力テーブルが矛盾する。ADR-SRS-038「入出力テーブルが外部I/Fの単一の俯瞰点になる」という目的からも不整合が生じる。</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>改善</t>
+        </is>
+      </c>
+      <c r="E163" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="I163" s="2" t="inlineStr">
+        <is>
+          <t>SRS</t>
+        </is>
+      </c>
+      <c r="J163" s="2" t="inlineStr"/>
+      <c r="K163" s="2" t="inlineStr">
+        <is>
+          <t>解決済</t>
+        </is>
+      </c>
+      <c r="L163" s="2" t="inlineStr"/>
+      <c r="M163" s="2" t="inlineStr">
+        <is>
+          <t>以下どちらかを選択して SRS を修正する。①§6.1 No.10 の「使用/生成 FR」を FR-001/FR-019 のみに修正（FR-004/FR-014 は外部I/F を直接使わず ADR-SRS-016 に従い内部データ経由とみなす）。②FR-004/FR-014 の入力テーブルに「地理院標高タイル（外部I/F・キャッシュ再利用）」を追加する（ADR-SRS-038 の「キャッシュ再利用を問わず列挙」を優先）。ADR-SRS-016 と ADR-SRS-038 のどちらを上位原則とするかを決めてから修正する。</t>
+        </is>
+      </c>
+      <c r="N163" s="2" t="inlineStr"/>
+      <c r="O163" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="P163" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="K2:K158" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K163" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未対応,対応中,対応完了,解決済,却下"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E158" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E163" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D158" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D163" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"改善,調査,設計"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I158" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I163" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J158" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J163" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"URD,SRS,HLD,LLD,COD,UT,IT,ST,OPS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -11695,7 +12049,7 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3">
@@ -11705,7 +12059,7 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -11715,7 +12069,7 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5">
@@ -11726,7 +12080,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>74.5%</t>
+          <t>77.2%</t>
         </is>
       </c>
     </row>
@@ -11745,7 +12099,7 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -11765,7 +12119,7 @@
         </is>
       </c>
       <c r="B10" s="11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -11775,7 +12129,7 @@
         </is>
       </c>
       <c r="B11" s="11" t="n">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12">
@@ -11803,7 +12157,7 @@
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
@@ -11813,7 +12167,7 @@
         </is>
       </c>
       <c r="B16" s="11" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
@@ -11841,7 +12195,7 @@
         </is>
       </c>
       <c r="B20" s="11" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21">
@@ -11861,7 +12215,7 @@
         </is>
       </c>
       <c r="B22" s="11" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
@@ -11899,7 +12253,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
@@ -11909,7 +12263,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -11927,7 +12281,7 @@
         </is>
       </c>
       <c r="B31" s="11" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="32">
@@ -13007,13 +13361,13 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="C65" t="n">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="D65" t="n">
-        <v>134</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>